<commit_message>
Update at 22:26 on 07/27/2020
</commit_message>
<xml_diff>
--- a/site_libs/records/fall 2020.xlsx
+++ b/site_libs/records/fall 2020.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Portfolio\site_libs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Portfolio\site_libs\records\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19DB343C-07C6-4022-B398-3CAE05446461}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7098D1C2-84E8-4B42-941C-5EFFFB6396C1}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="231" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="233" uniqueCount="126">
   <si>
     <t>Monday</t>
   </si>
@@ -95,12 +95,6 @@
     <t>Burton</t>
   </si>
   <si>
-    <t>MATH 488
-Consulting
-Hathaway
-Rks 229</t>
-  </si>
-  <si>
     <t>MATH</t>
   </si>
   <si>
@@ -117,9 +111,6 @@
   </si>
   <si>
     <t>Saunders</t>
-  </si>
-  <si>
-    <t>Consulting</t>
   </si>
   <si>
     <t>Rks</t>
@@ -428,19 +419,41 @@
     <t>Barney</t>
   </si>
   <si>
-    <t>CSE 121b JavaScript Barney Remote</t>
-  </si>
-  <si>
     <t>TA 
 ECEN 361
 Grimmett</t>
+  </si>
+  <si>
+    <t>CSE 121b 
+JavaScript 
+Barney 
+Remote</t>
+  </si>
+  <si>
+    <t>TA 
+ECEN 340 
+Jack</t>
+  </si>
+  <si>
+    <t>TA 
+ECEN 160L 
+Jack</t>
+  </si>
+  <si>
+    <t>Data Consulting</t>
+  </si>
+  <si>
+    <t>MATH 488
+Data Consulting
+Hathaway
+Rks 229</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="14" x14ac:knownFonts="1">
+  <fonts count="16" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -516,6 +529,18 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF0000FF"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -549,7 +574,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -612,33 +637,46 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -858,17 +896,20 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:U36"/>
+  <dimension ref="A1:U37"/>
   <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="11.7109375" customWidth="1"/>
-    <col min="2" max="2" width="14.42578125" customWidth="1"/>
-    <col min="3" max="3" width="8.7109375" customWidth="1"/>
+    <col min="2" max="2" width="11.28515625" customWidth="1"/>
+    <col min="3" max="3" width="9.42578125" customWidth="1"/>
     <col min="4" max="4" width="10.42578125" customWidth="1"/>
     <col min="5" max="5" width="8.7109375" customWidth="1"/>
-    <col min="7" max="7" width="9.85546875" customWidth="1"/>
+    <col min="6" max="6" width="11.28515625" customWidth="1"/>
+    <col min="7" max="7" width="9.42578125" customWidth="1"/>
     <col min="8" max="8" width="10.140625" customWidth="1"/>
     <col min="9" max="9" width="9.85546875" customWidth="1"/>
+    <col min="10" max="10" width="11.28515625" customWidth="1"/>
+    <col min="11" max="11" width="9.42578125" customWidth="1"/>
     <col min="12" max="12" width="6" customWidth="1"/>
     <col min="13" max="13" width="10.85546875" customWidth="1"/>
     <col min="14" max="14" width="5.5703125" customWidth="1"/>
@@ -880,27 +921,27 @@
     <col min="21" max="21" width="5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="B1" s="26" t="s">
+    <row r="1" spans="1:21" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B1" s="28" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="31"/>
-      <c r="D1" s="26" t="s">
+      <c r="C1" s="29"/>
+      <c r="D1" s="28" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="31"/>
-      <c r="F1" s="26" t="s">
+      <c r="E1" s="29"/>
+      <c r="F1" s="28" t="s">
         <v>2</v>
       </c>
-      <c r="G1" s="31"/>
-      <c r="H1" s="26" t="s">
+      <c r="G1" s="29"/>
+      <c r="H1" s="28" t="s">
         <v>3</v>
       </c>
-      <c r="I1" s="31"/>
-      <c r="J1" s="26" t="s">
+      <c r="I1" s="29"/>
+      <c r="J1" s="28" t="s">
         <v>4</v>
       </c>
-      <c r="K1" s="31"/>
+      <c r="K1" s="29"/>
       <c r="L1" s="1"/>
       <c r="M1" s="2" t="s">
         <v>5</v>
@@ -949,38 +990,38 @@
         <v>14</v>
       </c>
       <c r="N2" s="13" t="s">
+        <v>116</v>
+      </c>
+      <c r="O2" s="13" t="s">
+        <v>117</v>
+      </c>
+      <c r="P2" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q2" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="R2" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="S2" s="13" t="s">
         <v>118</v>
       </c>
-      <c r="O2" s="13" t="s">
+      <c r="T2" s="13" t="s">
         <v>119</v>
-      </c>
-      <c r="P2" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="Q2" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="R2" s="13" t="s">
-        <v>29</v>
-      </c>
-      <c r="S2" s="13" t="s">
-        <v>120</v>
-      </c>
-      <c r="T2" s="13" t="s">
-        <v>121</v>
       </c>
       <c r="U2" s="13">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:21" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A3" s="8">
         <v>0.33333333333333331</v>
       </c>
       <c r="B3" s="4"/>
       <c r="C3" s="25"/>
-      <c r="D3" s="30" t="s">
-        <v>20</v>
+      <c r="D3" s="40" t="s">
+        <v>125</v>
       </c>
       <c r="E3" s="6"/>
       <c r="F3" s="6"/>
@@ -988,7 +1029,7 @@
       <c r="H3" s="30" t="str">
         <f>D3</f>
         <v>MATH 488
-Consulting
+Data Consulting
 Hathaway
 Rks 229</v>
       </c>
@@ -1030,81 +1071,81 @@
       </c>
       <c r="B4" s="4"/>
       <c r="C4" s="25"/>
-      <c r="D4" s="27"/>
+      <c r="D4" s="31"/>
       <c r="E4" s="6"/>
       <c r="F4" s="6"/>
       <c r="G4" s="6"/>
-      <c r="H4" s="27"/>
+      <c r="H4" s="31"/>
       <c r="I4" s="4"/>
       <c r="J4" s="4"/>
       <c r="K4" s="4"/>
       <c r="L4" s="4"/>
       <c r="M4" s="7" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="N4" s="7">
         <v>325</v>
       </c>
       <c r="O4" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="P4" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="P4" s="7" t="s">
+      <c r="Q4" s="7" t="s">
         <v>23</v>
-      </c>
-      <c r="Q4" s="7" t="s">
-        <v>24</v>
       </c>
       <c r="R4" s="7" t="s">
         <v>17</v>
       </c>
       <c r="S4" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="T4" s="7" t="s">
         <v>25</v>
-      </c>
-      <c r="T4" s="7" t="s">
-        <v>26</v>
       </c>
       <c r="U4" s="7">
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:21" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A5" s="8">
         <v>0.35416666666666669</v>
       </c>
       <c r="B5" s="4"/>
       <c r="C5" s="25"/>
-      <c r="D5" s="27"/>
+      <c r="D5" s="31"/>
       <c r="E5" s="6"/>
       <c r="F5" s="6"/>
       <c r="G5" s="6"/>
-      <c r="H5" s="27"/>
+      <c r="H5" s="31"/>
       <c r="I5" s="4"/>
       <c r="J5" s="4"/>
       <c r="K5" s="4"/>
       <c r="L5" s="4"/>
       <c r="M5" s="7" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="N5" s="7">
         <v>488</v>
       </c>
-      <c r="O5" s="7" t="s">
-        <v>27</v>
+      <c r="O5" s="39" t="s">
+        <v>124</v>
       </c>
       <c r="P5" s="7" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="Q5" s="7">
         <v>229</v>
       </c>
       <c r="R5" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="S5" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="T5" s="7" t="s">
         <v>29</v>
-      </c>
-      <c r="S5" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="T5" s="7" t="s">
-        <v>31</v>
       </c>
       <c r="U5" s="7">
         <v>3</v>
@@ -1116,11 +1157,11 @@
       </c>
       <c r="B6" s="4"/>
       <c r="C6" s="25"/>
-      <c r="D6" s="27"/>
+      <c r="D6" s="31"/>
       <c r="E6" s="6"/>
       <c r="F6" s="6"/>
       <c r="G6" s="6"/>
-      <c r="H6" s="27"/>
+      <c r="H6" s="31"/>
       <c r="I6" s="4"/>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
@@ -1136,11 +1177,11 @@
       </c>
       <c r="B7" s="4"/>
       <c r="C7" s="25"/>
-      <c r="D7" s="27"/>
+      <c r="D7" s="31"/>
       <c r="E7" s="6"/>
       <c r="F7" s="6"/>
       <c r="G7" s="6"/>
-      <c r="H7" s="27"/>
+      <c r="H7" s="31"/>
       <c r="I7" s="4"/>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
@@ -1152,11 +1193,11 @@
       </c>
       <c r="B8" s="4"/>
       <c r="C8" s="25"/>
-      <c r="D8" s="27"/>
+      <c r="D8" s="31"/>
       <c r="E8" s="6"/>
       <c r="F8" s="6"/>
       <c r="G8" s="6"/>
-      <c r="H8" s="27"/>
+      <c r="H8" s="31"/>
       <c r="I8" s="4"/>
       <c r="J8" s="4"/>
       <c r="K8" s="4"/>
@@ -1177,9 +1218,7 @@
       <c r="J9" s="4"/>
       <c r="K9" s="4"/>
       <c r="L9" s="4"/>
-      <c r="M9" s="9" t="s">
-        <v>32</v>
-      </c>
+      <c r="M9" s="9"/>
     </row>
     <row r="10" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A10" s="8">
@@ -1197,7 +1236,7 @@
       <c r="K10" s="4"/>
       <c r="L10" s="4"/>
       <c r="M10" s="10" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="11" spans="1:21" x14ac:dyDescent="0.2">
@@ -1221,68 +1260,74 @@
         <v>0.42708333333333331</v>
       </c>
       <c r="B12" s="4"/>
-      <c r="C12" s="29" t="s">
-        <v>34</v>
-      </c>
-      <c r="D12" s="28" t="s">
-        <v>122</v>
+      <c r="C12" s="32" t="s">
+        <v>32</v>
+      </c>
+      <c r="D12" s="33" t="s">
+        <v>121</v>
       </c>
       <c r="E12" s="4"/>
       <c r="F12" s="4"/>
-      <c r="G12" s="29" t="s">
-        <v>35</v>
-      </c>
-      <c r="H12" s="28" t="s">
-        <v>122</v>
+      <c r="G12" s="32" t="s">
+        <v>33</v>
+      </c>
+      <c r="H12" s="33" t="str">
+        <f>D12</f>
+        <v>CSE 121b 
+JavaScript 
+Barney 
+Remote</v>
       </c>
       <c r="I12" s="4"/>
       <c r="J12" s="4"/>
-      <c r="K12" s="25"/>
+      <c r="K12" s="38" t="s">
+        <v>123</v>
+      </c>
     </row>
     <row r="13" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A13" s="8">
         <v>0.4375</v>
       </c>
       <c r="B13" s="4"/>
-      <c r="C13" s="27"/>
-      <c r="D13" s="28"/>
+      <c r="C13" s="31"/>
+      <c r="D13" s="33"/>
       <c r="E13" s="4"/>
       <c r="F13" s="4"/>
-      <c r="G13" s="27"/>
-      <c r="H13" s="28"/>
+      <c r="G13" s="31"/>
+      <c r="H13" s="33"/>
       <c r="I13" s="4"/>
       <c r="J13" s="4"/>
-      <c r="K13" s="25"/>
+      <c r="K13" s="38"/>
     </row>
     <row r="14" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A14" s="8">
         <v>0.44791666666666669</v>
       </c>
       <c r="B14" s="4"/>
-      <c r="C14" s="27"/>
-      <c r="D14" s="28"/>
+      <c r="C14" s="31"/>
+      <c r="D14" s="33"/>
       <c r="E14" s="4"/>
       <c r="F14" s="4"/>
-      <c r="G14" s="27"/>
-      <c r="H14" s="28"/>
+      <c r="G14" s="31"/>
+      <c r="H14" s="33"/>
       <c r="I14" s="4"/>
       <c r="J14" s="4"/>
-      <c r="K14" s="25"/>
+      <c r="K14" s="38"/>
     </row>
     <row r="15" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A15" s="8">
         <v>0.45833333333333331</v>
       </c>
       <c r="B15" s="4"/>
-      <c r="C15" s="27"/>
-      <c r="D15" s="28"/>
+      <c r="C15" s="31"/>
+      <c r="D15" s="33"/>
       <c r="E15" s="4"/>
       <c r="F15" s="4"/>
-      <c r="G15" s="27"/>
-      <c r="H15" s="28"/>
+      <c r="G15" s="31"/>
+      <c r="H15" s="33"/>
       <c r="I15" s="4"/>
       <c r="J15" s="4"/>
-      <c r="K15" s="25"/>
+      <c r="K15" s="38"/>
     </row>
     <row r="16" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A16" s="8">
@@ -1297,14 +1342,14 @@
       <c r="H16" s="4"/>
       <c r="I16" s="4"/>
       <c r="J16" s="4"/>
-      <c r="K16" s="25"/>
+      <c r="K16" s="37"/>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A17" s="8">
         <v>0.47916666666666669</v>
       </c>
       <c r="B17" s="30" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C17" s="25"/>
       <c r="D17" s="12"/>
@@ -1332,45 +1377,45 @@
       <c r="A18" s="8">
         <v>0.48958333333333331</v>
       </c>
-      <c r="B18" s="27"/>
+      <c r="B18" s="31"/>
       <c r="C18" s="25"/>
       <c r="D18" s="12"/>
       <c r="E18" s="12"/>
-      <c r="F18" s="27"/>
+      <c r="F18" s="31"/>
       <c r="G18" s="12"/>
       <c r="H18" s="12"/>
       <c r="I18" s="12"/>
-      <c r="J18" s="27"/>
+      <c r="J18" s="31"/>
       <c r="K18" s="25"/>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A19" s="8">
         <v>0.5</v>
       </c>
-      <c r="B19" s="27"/>
+      <c r="B19" s="31"/>
       <c r="C19" s="25"/>
       <c r="D19" s="12"/>
       <c r="E19" s="12"/>
-      <c r="F19" s="27"/>
+      <c r="F19" s="31"/>
       <c r="G19" s="12"/>
       <c r="H19" s="12"/>
       <c r="I19" s="12"/>
-      <c r="J19" s="27"/>
+      <c r="J19" s="31"/>
       <c r="K19" s="25"/>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A20" s="8">
         <v>0.51041666666666663</v>
       </c>
-      <c r="B20" s="27"/>
+      <c r="B20" s="31"/>
       <c r="C20" s="25"/>
       <c r="D20" s="4"/>
       <c r="E20" s="4"/>
-      <c r="F20" s="27"/>
+      <c r="F20" s="31"/>
       <c r="G20" s="4"/>
       <c r="H20" s="4"/>
       <c r="I20" s="4"/>
-      <c r="J20" s="27"/>
+      <c r="J20" s="31"/>
       <c r="K20" s="25"/>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.2">
@@ -1392,65 +1437,67 @@
       <c r="A22" s="8">
         <v>0.53125</v>
       </c>
-      <c r="C22" s="29" t="s">
+      <c r="C22" s="32" t="s">
+        <v>120</v>
+      </c>
+      <c r="D22" s="4"/>
+      <c r="E22" s="32" t="s">
+        <v>32</v>
+      </c>
+      <c r="F22" s="4"/>
+      <c r="G22" s="32" t="s">
+        <v>120</v>
+      </c>
+      <c r="H22" s="4"/>
+      <c r="I22" s="32" t="s">
+        <v>33</v>
+      </c>
+      <c r="J22" s="4"/>
+      <c r="K22" s="38" t="s">
         <v>123</v>
       </c>
-      <c r="D22" s="4"/>
-      <c r="E22" s="29" t="s">
-        <v>34</v>
-      </c>
-      <c r="F22" s="4"/>
-      <c r="G22" s="29" t="s">
-        <v>123</v>
-      </c>
-      <c r="H22" s="4"/>
-      <c r="I22" s="29" t="s">
-        <v>35</v>
-      </c>
-      <c r="J22" s="4"/>
-      <c r="K22" s="25"/>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A23" s="8">
         <v>0.54166666666666663</v>
       </c>
-      <c r="C23" s="27"/>
+      <c r="C23" s="31"/>
       <c r="D23" s="4"/>
-      <c r="E23" s="27"/>
+      <c r="E23" s="31"/>
       <c r="F23" s="4"/>
-      <c r="G23" s="27"/>
+      <c r="G23" s="31"/>
       <c r="H23" s="4"/>
-      <c r="I23" s="27"/>
+      <c r="I23" s="31"/>
       <c r="J23" s="4"/>
-      <c r="K23" s="25"/>
+      <c r="K23" s="38"/>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A24" s="8">
         <v>0.55208333333333337</v>
       </c>
-      <c r="C24" s="27"/>
+      <c r="C24" s="31"/>
       <c r="D24" s="4"/>
-      <c r="E24" s="27"/>
+      <c r="E24" s="31"/>
       <c r="F24" s="4"/>
-      <c r="G24" s="27"/>
+      <c r="G24" s="31"/>
       <c r="H24" s="4"/>
-      <c r="I24" s="27"/>
+      <c r="I24" s="31"/>
       <c r="J24" s="4"/>
-      <c r="K24" s="25"/>
+      <c r="K24" s="38"/>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A25" s="8">
         <v>0.5625</v>
       </c>
-      <c r="C25" s="27"/>
+      <c r="C25" s="31"/>
       <c r="D25" s="4"/>
-      <c r="E25" s="27"/>
+      <c r="E25" s="31"/>
       <c r="F25" s="4"/>
-      <c r="G25" s="27"/>
+      <c r="G25" s="31"/>
       <c r="H25" s="4"/>
-      <c r="I25" s="27"/>
+      <c r="I25" s="31"/>
       <c r="J25" s="4"/>
-      <c r="K25" s="25"/>
+      <c r="K25" s="38"/>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A26" s="8">
@@ -1471,15 +1518,15 @@
       <c r="A27" s="8">
         <v>0.58333333333333337</v>
       </c>
-      <c r="B27" s="26" t="s">
-        <v>37</v>
+      <c r="B27" s="28" t="s">
+        <v>35</v>
       </c>
       <c r="C27" s="25"/>
       <c r="D27" s="4"/>
-      <c r="E27" s="29" t="s">
-        <v>38</v>
-      </c>
-      <c r="F27" s="26" t="str">
+      <c r="E27" s="32" t="s">
+        <v>36</v>
+      </c>
+      <c r="F27" s="28" t="str">
         <f>B27</f>
         <v>MATH 325
 Intermediate Stats 
@@ -1488,10 +1535,10 @@
       </c>
       <c r="G27" s="25"/>
       <c r="H27" s="4"/>
-      <c r="I27" s="29" t="s">
-        <v>38</v>
-      </c>
-      <c r="J27" s="26" t="str">
+      <c r="I27" s="32" t="s">
+        <v>36</v>
+      </c>
+      <c r="J27" s="28" t="str">
         <f>F27</f>
         <v>MATH 325
 Intermediate Stats 
@@ -1504,45 +1551,45 @@
       <c r="A28" s="8">
         <v>0.59375</v>
       </c>
-      <c r="B28" s="27"/>
+      <c r="B28" s="31"/>
       <c r="C28" s="25"/>
       <c r="D28" s="4"/>
-      <c r="E28" s="27"/>
-      <c r="F28" s="27"/>
+      <c r="E28" s="31"/>
+      <c r="F28" s="31"/>
       <c r="G28" s="25"/>
       <c r="H28" s="4"/>
-      <c r="I28" s="27"/>
-      <c r="J28" s="27"/>
+      <c r="I28" s="31"/>
+      <c r="J28" s="31"/>
       <c r="K28" s="25"/>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A29" s="8">
         <v>0.60416666666666663</v>
       </c>
-      <c r="B29" s="27"/>
+      <c r="B29" s="31"/>
       <c r="C29" s="25"/>
       <c r="D29" s="4"/>
-      <c r="E29" s="27"/>
-      <c r="F29" s="27"/>
+      <c r="E29" s="31"/>
+      <c r="F29" s="31"/>
       <c r="G29" s="25"/>
       <c r="H29" s="4"/>
-      <c r="I29" s="27"/>
-      <c r="J29" s="27"/>
+      <c r="I29" s="31"/>
+      <c r="J29" s="31"/>
       <c r="K29" s="25"/>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A30" s="8">
         <v>0.61458333333333337</v>
       </c>
-      <c r="B30" s="27"/>
+      <c r="B30" s="31"/>
       <c r="C30" s="25"/>
       <c r="D30" s="4"/>
-      <c r="E30" s="27"/>
-      <c r="F30" s="27"/>
+      <c r="E30" s="31"/>
+      <c r="F30" s="31"/>
       <c r="G30" s="25"/>
       <c r="H30" s="4"/>
-      <c r="I30" s="27"/>
-      <c r="J30" s="27"/>
+      <c r="I30" s="31"/>
+      <c r="J30" s="31"/>
       <c r="K30" s="25"/>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.2">
@@ -1554,7 +1601,7 @@
       <c r="D31" s="4"/>
       <c r="E31" s="4"/>
       <c r="F31" s="4" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="G31" s="25"/>
       <c r="H31" s="4"/>
@@ -1567,11 +1614,15 @@
         <v>0.63541666666666663</v>
       </c>
       <c r="B32" s="6"/>
-      <c r="C32" s="6"/>
+      <c r="C32" s="38" t="s">
+        <v>122</v>
+      </c>
       <c r="D32" s="6"/>
       <c r="E32" s="6"/>
       <c r="F32" s="6"/>
-      <c r="G32" s="6"/>
+      <c r="G32" s="38" t="s">
+        <v>122</v>
+      </c>
       <c r="H32" s="6"/>
       <c r="I32" s="6"/>
       <c r="J32" s="6"/>
@@ -1582,11 +1633,11 @@
         <v>0.64583333333333337</v>
       </c>
       <c r="B33" s="6"/>
-      <c r="C33" s="6"/>
+      <c r="C33" s="32"/>
       <c r="D33" s="6"/>
       <c r="E33" s="6"/>
       <c r="F33" s="6"/>
-      <c r="G33" s="6"/>
+      <c r="G33" s="32"/>
       <c r="H33" s="6"/>
       <c r="I33" s="6"/>
       <c r="J33" s="6"/>
@@ -1597,11 +1648,11 @@
         <v>0.65625</v>
       </c>
       <c r="B34" s="6"/>
-      <c r="C34" s="6"/>
+      <c r="C34" s="32"/>
       <c r="D34" s="6"/>
       <c r="E34" s="6"/>
       <c r="F34" s="6"/>
-      <c r="G34" s="6"/>
+      <c r="G34" s="32"/>
       <c r="H34" s="6"/>
       <c r="I34" s="6"/>
       <c r="J34" s="6"/>
@@ -1612,11 +1663,11 @@
         <v>0.66666666666666663</v>
       </c>
       <c r="B35" s="6"/>
-      <c r="C35" s="6"/>
+      <c r="C35" s="32"/>
       <c r="D35" s="6"/>
       <c r="E35" s="6"/>
       <c r="F35" s="6"/>
-      <c r="G35" s="6"/>
+      <c r="G35" s="32"/>
       <c r="H35" s="6"/>
       <c r="I35" s="6"/>
       <c r="J35" s="6"/>
@@ -1627,30 +1678,27 @@
         <v>0.67708333333333337</v>
       </c>
       <c r="B36" s="4"/>
-      <c r="C36" s="4"/>
+      <c r="C36" s="32"/>
       <c r="D36" s="4"/>
       <c r="E36" s="4"/>
       <c r="F36" s="4"/>
-      <c r="G36" s="4"/>
+      <c r="G36" s="32"/>
       <c r="H36" s="4"/>
       <c r="I36" s="4"/>
       <c r="J36" s="4"/>
       <c r="K36" s="25"/>
     </row>
+    <row r="37" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A37" s="8">
+        <v>0.6875</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="23">
-    <mergeCell ref="B1:C1"/>
-    <mergeCell ref="D1:E1"/>
-    <mergeCell ref="F1:G1"/>
-    <mergeCell ref="H1:I1"/>
-    <mergeCell ref="J1:K1"/>
-    <mergeCell ref="D3:D8"/>
-    <mergeCell ref="H3:H8"/>
-    <mergeCell ref="E22:E25"/>
-    <mergeCell ref="E27:E30"/>
-    <mergeCell ref="I22:I25"/>
-    <mergeCell ref="I27:I30"/>
-    <mergeCell ref="G22:G25"/>
+  <mergeCells count="27">
+    <mergeCell ref="C32:C36"/>
+    <mergeCell ref="G32:G36"/>
+    <mergeCell ref="K12:K15"/>
+    <mergeCell ref="K22:K25"/>
     <mergeCell ref="B27:B30"/>
     <mergeCell ref="F27:F30"/>
     <mergeCell ref="J27:J30"/>
@@ -1662,6 +1710,18 @@
     <mergeCell ref="F17:F20"/>
     <mergeCell ref="J17:J20"/>
     <mergeCell ref="C22:C25"/>
+    <mergeCell ref="D3:D8"/>
+    <mergeCell ref="H3:H8"/>
+    <mergeCell ref="E22:E25"/>
+    <mergeCell ref="E27:E30"/>
+    <mergeCell ref="I22:I25"/>
+    <mergeCell ref="I27:I30"/>
+    <mergeCell ref="G22:G25"/>
+    <mergeCell ref="B1:C1"/>
+    <mergeCell ref="D1:E1"/>
+    <mergeCell ref="F1:G1"/>
+    <mergeCell ref="H1:I1"/>
+    <mergeCell ref="J1:K1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1695,26 +1755,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="B1" s="26" t="s">
+      <c r="B1" s="28" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="31"/>
-      <c r="D1" s="26" t="s">
+      <c r="C1" s="29"/>
+      <c r="D1" s="28" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="31"/>
-      <c r="F1" s="26" t="s">
+      <c r="E1" s="29"/>
+      <c r="F1" s="28" t="s">
         <v>2</v>
       </c>
-      <c r="G1" s="31"/>
-      <c r="H1" s="26" t="s">
+      <c r="G1" s="29"/>
+      <c r="H1" s="28" t="s">
         <v>3</v>
       </c>
-      <c r="I1" s="31"/>
-      <c r="J1" s="26" t="s">
+      <c r="I1" s="29"/>
+      <c r="J1" s="28" t="s">
         <v>4</v>
       </c>
-      <c r="K1" s="31"/>
+      <c r="K1" s="29"/>
       <c r="L1" s="1"/>
       <c r="M1" s="2" t="s">
         <v>5</v>
@@ -1749,13 +1809,13 @@
         <v>0.33333333333333331</v>
       </c>
       <c r="B2" s="4"/>
-      <c r="D2" s="32" t="s">
-        <v>40</v>
+      <c r="D2" s="35" t="s">
+        <v>38</v>
       </c>
       <c r="E2" s="4"/>
       <c r="F2" s="4"/>
       <c r="G2" s="4"/>
-      <c r="H2" s="32" t="str">
+      <c r="H2" s="35" t="str">
         <f>D2</f>
         <v>CSE 341
 Web Backend 2
@@ -1799,38 +1859,38 @@
         <v>0.34375</v>
       </c>
       <c r="B3" s="4"/>
-      <c r="D3" s="31"/>
+      <c r="D3" s="29"/>
       <c r="E3" s="4"/>
       <c r="F3" s="4"/>
       <c r="G3" s="4"/>
-      <c r="H3" s="31"/>
+      <c r="H3" s="29"/>
       <c r="I3" s="4"/>
       <c r="J3" s="4"/>
       <c r="K3" s="4"/>
       <c r="L3" s="4"/>
       <c r="M3" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="N3" s="2">
         <v>325</v>
       </c>
       <c r="O3" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="P3" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="P3" s="2" t="s">
+      <c r="Q3" s="2" t="s">
         <v>23</v>
-      </c>
-      <c r="Q3" s="2" t="s">
-        <v>24</v>
       </c>
       <c r="R3" s="2" t="s">
         <v>17</v>
       </c>
       <c r="S3" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="T3" s="2" t="s">
         <v>25</v>
-      </c>
-      <c r="T3" s="2" t="s">
-        <v>26</v>
       </c>
       <c r="U3" s="2">
         <v>3</v>
@@ -1841,23 +1901,23 @@
         <v>0.35416666666666669</v>
       </c>
       <c r="B4" s="4"/>
-      <c r="D4" s="31"/>
+      <c r="D4" s="29"/>
       <c r="E4" s="4"/>
       <c r="F4" s="4"/>
       <c r="G4" s="4"/>
-      <c r="H4" s="31"/>
+      <c r="H4" s="29"/>
       <c r="I4" s="4"/>
       <c r="J4" s="4"/>
       <c r="K4" s="4"/>
       <c r="L4" s="4"/>
       <c r="M4" s="2" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="N4" s="2">
         <v>330</v>
       </c>
       <c r="O4" s="2" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="P4" s="2" t="s">
         <v>16</v>
@@ -1866,13 +1926,13 @@
         <v>347</v>
       </c>
       <c r="R4" s="2" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="S4" s="2" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="T4" s="13" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="U4" s="2">
         <v>3</v>
@@ -1883,11 +1943,11 @@
         <v>0.36458333333333331</v>
       </c>
       <c r="B5" s="4"/>
-      <c r="D5" s="31"/>
+      <c r="D5" s="29"/>
       <c r="E5" s="4"/>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
-      <c r="H5" s="31"/>
+      <c r="H5" s="29"/>
       <c r="I5" s="4"/>
       <c r="J5" s="4"/>
       <c r="K5" s="4"/>
@@ -1899,22 +1959,22 @@
         <v>341</v>
       </c>
       <c r="O5" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="P5" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q5" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="R5" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="S5" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="T5" s="13" t="s">
         <v>45</v>
-      </c>
-      <c r="P5" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="Q5" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="R5" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="S5" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="T5" s="13" t="s">
-        <v>47</v>
       </c>
       <c r="U5" s="2">
         <v>3</v>
@@ -1925,11 +1985,11 @@
         <v>0.375</v>
       </c>
       <c r="B6" s="4"/>
-      <c r="D6" s="31"/>
+      <c r="D6" s="29"/>
       <c r="E6" s="4"/>
       <c r="F6" s="4"/>
       <c r="G6" s="4"/>
-      <c r="H6" s="31"/>
+      <c r="H6" s="29"/>
       <c r="I6" s="4"/>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
@@ -1940,17 +2000,17 @@
         <v>0.38541666666666669</v>
       </c>
       <c r="B7" s="4"/>
-      <c r="D7" s="31"/>
+      <c r="D7" s="29"/>
       <c r="E7" s="4"/>
       <c r="F7" s="4"/>
       <c r="G7" s="4"/>
-      <c r="H7" s="31"/>
+      <c r="H7" s="29"/>
       <c r="I7" s="4"/>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
       <c r="L7" s="4"/>
       <c r="M7" s="9" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="8" spans="1:21" x14ac:dyDescent="0.2">
@@ -1968,7 +2028,7 @@
       <c r="K8" s="4"/>
       <c r="L8" s="4"/>
       <c r="M8" s="10" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="9" spans="1:21" x14ac:dyDescent="0.2">
@@ -1976,14 +2036,14 @@
         <v>0.40625</v>
       </c>
       <c r="B9" s="4"/>
-      <c r="D9" s="32" t="s">
-        <v>48</v>
+      <c r="D9" s="35" t="s">
+        <v>46</v>
       </c>
       <c r="E9" s="4"/>
       <c r="F9" s="4"/>
       <c r="G9" s="4"/>
-      <c r="H9" s="32" t="s">
-        <v>48</v>
+      <c r="H9" s="35" t="s">
+        <v>46</v>
       </c>
       <c r="I9" s="4"/>
       <c r="J9" s="4"/>
@@ -1995,11 +2055,11 @@
         <v>0.41666666666666669</v>
       </c>
       <c r="B10" s="4"/>
-      <c r="D10" s="31"/>
+      <c r="D10" s="29"/>
       <c r="E10" s="4"/>
       <c r="F10" s="4"/>
       <c r="G10" s="4"/>
-      <c r="H10" s="31"/>
+      <c r="H10" s="29"/>
       <c r="I10" s="4"/>
       <c r="J10" s="4"/>
       <c r="K10" s="4"/>
@@ -2010,19 +2070,19 @@
         <v>0.42708333333333331</v>
       </c>
       <c r="B11" s="1"/>
-      <c r="C11" s="33" t="s">
-        <v>34</v>
-      </c>
-      <c r="D11" s="31"/>
+      <c r="C11" s="34" t="s">
+        <v>32</v>
+      </c>
+      <c r="D11" s="29"/>
       <c r="E11" s="4"/>
       <c r="F11" s="1">
         <f>B11</f>
         <v>0</v>
       </c>
-      <c r="G11" s="33" t="s">
-        <v>35</v>
-      </c>
-      <c r="H11" s="31"/>
+      <c r="G11" s="34" t="s">
+        <v>33</v>
+      </c>
+      <c r="H11" s="29"/>
       <c r="I11" s="4"/>
       <c r="J11" s="1"/>
     </row>
@@ -2031,12 +2091,12 @@
         <v>0.4375</v>
       </c>
       <c r="B12" s="1"/>
-      <c r="C12" s="31"/>
-      <c r="D12" s="31"/>
+      <c r="C12" s="29"/>
+      <c r="D12" s="29"/>
       <c r="E12" s="4"/>
       <c r="F12" s="1"/>
-      <c r="G12" s="31"/>
-      <c r="H12" s="31"/>
+      <c r="G12" s="29"/>
+      <c r="H12" s="29"/>
       <c r="I12" s="4"/>
       <c r="J12" s="1"/>
     </row>
@@ -2045,12 +2105,12 @@
         <v>0.44791666666666669</v>
       </c>
       <c r="B13" s="1"/>
-      <c r="C13" s="31"/>
-      <c r="D13" s="31"/>
+      <c r="C13" s="29"/>
+      <c r="D13" s="29"/>
       <c r="E13" s="4"/>
       <c r="F13" s="1"/>
-      <c r="G13" s="31"/>
-      <c r="H13" s="31"/>
+      <c r="G13" s="29"/>
+      <c r="H13" s="29"/>
       <c r="I13" s="4"/>
       <c r="J13" s="1"/>
     </row>
@@ -2059,12 +2119,12 @@
         <v>0.45833333333333331</v>
       </c>
       <c r="B14" s="1"/>
-      <c r="C14" s="31"/>
-      <c r="D14" s="31"/>
+      <c r="C14" s="29"/>
+      <c r="D14" s="29"/>
       <c r="E14" s="4"/>
       <c r="F14" s="1"/>
-      <c r="G14" s="31"/>
-      <c r="H14" s="31"/>
+      <c r="G14" s="29"/>
+      <c r="H14" s="29"/>
       <c r="I14" s="4"/>
       <c r="J14" s="1"/>
     </row>
@@ -2086,7 +2146,7 @@
         <v>0.47916666666666669</v>
       </c>
       <c r="B16" s="30" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="D16" s="12"/>
       <c r="E16" s="12"/>
@@ -2112,40 +2172,40 @@
       <c r="A17" s="8">
         <v>0.48958333333333331</v>
       </c>
-      <c r="B17" s="31"/>
+      <c r="B17" s="29"/>
       <c r="D17" s="12"/>
       <c r="E17" s="12"/>
-      <c r="F17" s="31"/>
+      <c r="F17" s="29"/>
       <c r="G17" s="12"/>
       <c r="H17" s="12"/>
       <c r="I17" s="12"/>
-      <c r="J17" s="31"/>
+      <c r="J17" s="29"/>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A18" s="8">
         <v>0.5</v>
       </c>
-      <c r="B18" s="31"/>
+      <c r="B18" s="29"/>
       <c r="D18" s="12"/>
       <c r="E18" s="12"/>
-      <c r="F18" s="31"/>
+      <c r="F18" s="29"/>
       <c r="G18" s="12"/>
       <c r="H18" s="12"/>
       <c r="I18" s="12"/>
-      <c r="J18" s="31"/>
+      <c r="J18" s="29"/>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A19" s="8">
         <v>0.51041666666666663</v>
       </c>
-      <c r="B19" s="31"/>
+      <c r="B19" s="29"/>
       <c r="D19" s="4"/>
       <c r="E19" s="4"/>
-      <c r="F19" s="31"/>
+      <c r="F19" s="29"/>
       <c r="G19" s="4"/>
       <c r="H19" s="4"/>
       <c r="I19" s="4"/>
-      <c r="J19" s="31"/>
+      <c r="J19" s="29"/>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A20" s="8">
@@ -2166,14 +2226,14 @@
       </c>
       <c r="B21" s="4"/>
       <c r="D21" s="4"/>
-      <c r="E21" s="33" t="s">
-        <v>34</v>
+      <c r="E21" s="34" t="s">
+        <v>32</v>
       </c>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
       <c r="H21" s="4"/>
-      <c r="I21" s="33" t="s">
-        <v>35</v>
+      <c r="I21" s="34" t="s">
+        <v>33</v>
       </c>
       <c r="J21" s="4"/>
     </row>
@@ -2183,11 +2243,11 @@
       </c>
       <c r="B22" s="4"/>
       <c r="D22" s="4"/>
-      <c r="E22" s="31"/>
+      <c r="E22" s="29"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
-      <c r="I22" s="31"/>
+      <c r="I22" s="29"/>
       <c r="J22" s="4"/>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.2">
@@ -2196,11 +2256,11 @@
       </c>
       <c r="B23" s="4"/>
       <c r="D23" s="4"/>
-      <c r="E23" s="31"/>
+      <c r="E23" s="29"/>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
-      <c r="I23" s="31"/>
+      <c r="I23" s="29"/>
       <c r="J23" s="4"/>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.2">
@@ -2209,11 +2269,11 @@
       </c>
       <c r="B24" s="4"/>
       <c r="D24" s="4"/>
-      <c r="E24" s="31"/>
+      <c r="E24" s="29"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
-      <c r="I24" s="31"/>
+      <c r="I24" s="29"/>
       <c r="J24" s="4"/>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.2">
@@ -2225,14 +2285,14 @@
       <c r="A26" s="8">
         <v>0.58333333333333337</v>
       </c>
-      <c r="B26" s="26" t="s">
-        <v>37</v>
+      <c r="B26" s="28" t="s">
+        <v>35</v>
       </c>
       <c r="D26" s="1"/>
-      <c r="E26" s="29" t="s">
-        <v>38</v>
-      </c>
-      <c r="F26" s="26" t="str">
+      <c r="E26" s="32" t="s">
+        <v>36</v>
+      </c>
+      <c r="F26" s="28" t="str">
         <f>B26</f>
         <v>MATH 325
 Intermediate Stats 
@@ -2240,10 +2300,10 @@
 Remote</v>
       </c>
       <c r="H26" s="1"/>
-      <c r="I26" s="29" t="s">
-        <v>38</v>
-      </c>
-      <c r="J26" s="26" t="str">
+      <c r="I26" s="32" t="s">
+        <v>36</v>
+      </c>
+      <c r="J26" s="28" t="str">
         <f>F26</f>
         <v>MATH 325
 Intermediate Stats 
@@ -2255,37 +2315,37 @@
       <c r="A27" s="8">
         <v>0.59375</v>
       </c>
-      <c r="B27" s="31"/>
+      <c r="B27" s="29"/>
       <c r="D27" s="1"/>
-      <c r="E27" s="31"/>
-      <c r="F27" s="31"/>
+      <c r="E27" s="29"/>
+      <c r="F27" s="29"/>
       <c r="H27" s="1"/>
-      <c r="I27" s="31"/>
-      <c r="J27" s="31"/>
+      <c r="I27" s="29"/>
+      <c r="J27" s="29"/>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A28" s="8">
         <v>0.60416666666666663</v>
       </c>
-      <c r="B28" s="31"/>
+      <c r="B28" s="29"/>
       <c r="D28" s="1"/>
-      <c r="E28" s="31"/>
-      <c r="F28" s="31"/>
+      <c r="E28" s="29"/>
+      <c r="F28" s="29"/>
       <c r="H28" s="1"/>
-      <c r="I28" s="31"/>
-      <c r="J28" s="31"/>
+      <c r="I28" s="29"/>
+      <c r="J28" s="29"/>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A29" s="8">
         <v>0.61458333333333337</v>
       </c>
-      <c r="B29" s="31"/>
+      <c r="B29" s="29"/>
       <c r="D29" s="1"/>
-      <c r="E29" s="31"/>
-      <c r="F29" s="31"/>
+      <c r="E29" s="29"/>
+      <c r="F29" s="29"/>
       <c r="H29" s="1"/>
-      <c r="I29" s="31"/>
-      <c r="J29" s="31"/>
+      <c r="I29" s="29"/>
+      <c r="J29" s="29"/>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A30" s="8">
@@ -2295,7 +2355,7 @@
       <c r="D30" s="4"/>
       <c r="E30" s="4"/>
       <c r="F30" s="1" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="H30" s="4"/>
       <c r="I30" s="4"/>
@@ -2373,11 +2433,12 @@
     </row>
   </sheetData>
   <mergeCells count="21">
-    <mergeCell ref="B1:C1"/>
-    <mergeCell ref="D1:E1"/>
-    <mergeCell ref="F1:G1"/>
-    <mergeCell ref="H1:I1"/>
-    <mergeCell ref="C11:C14"/>
+    <mergeCell ref="B16:B19"/>
+    <mergeCell ref="F16:F19"/>
+    <mergeCell ref="J16:J19"/>
+    <mergeCell ref="B26:B29"/>
+    <mergeCell ref="F26:F29"/>
+    <mergeCell ref="J26:J29"/>
     <mergeCell ref="J1:K1"/>
     <mergeCell ref="D2:D7"/>
     <mergeCell ref="D9:D14"/>
@@ -2388,12 +2449,11 @@
     <mergeCell ref="G11:G14"/>
     <mergeCell ref="H2:H7"/>
     <mergeCell ref="H9:H14"/>
-    <mergeCell ref="B16:B19"/>
-    <mergeCell ref="F16:F19"/>
-    <mergeCell ref="J16:J19"/>
-    <mergeCell ref="B26:B29"/>
-    <mergeCell ref="F26:F29"/>
-    <mergeCell ref="J26:J29"/>
+    <mergeCell ref="B1:C1"/>
+    <mergeCell ref="D1:E1"/>
+    <mergeCell ref="F1:G1"/>
+    <mergeCell ref="H1:I1"/>
+    <mergeCell ref="C11:C14"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2415,431 +2475,432 @@
   <sheetData>
     <row r="1" spans="1:6" ht="15" x14ac:dyDescent="0.2">
       <c r="A1" s="14" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B1" s="15" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C1" s="15">
         <v>1</v>
       </c>
       <c r="D1" s="15" t="s">
+        <v>49</v>
+      </c>
+      <c r="E1" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="F1" s="15" t="s">
         <v>51</v>
-      </c>
-      <c r="E1" s="16" t="s">
-        <v>52</v>
-      </c>
-      <c r="F1" s="15" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="15" x14ac:dyDescent="0.2">
       <c r="A2" s="14" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B2" s="17" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C2" s="17">
         <v>1</v>
       </c>
       <c r="D2" s="17" t="s">
+        <v>49</v>
+      </c>
+      <c r="E2" s="18" t="s">
+        <v>53</v>
+      </c>
+      <c r="F2" s="17" t="s">
         <v>51</v>
       </c>
-      <c r="E2" s="18" t="s">
-        <v>55</v>
-      </c>
-      <c r="F2" s="17" t="s">
-        <v>53</v>
-      </c>
     </row>
     <row r="3" spans="1:6" ht="15" x14ac:dyDescent="0.2">
-      <c r="A3" s="14" t="s">
-        <v>56</v>
-      </c>
-      <c r="B3" s="15" t="s">
-        <v>57</v>
-      </c>
-      <c r="C3" s="15">
+      <c r="A3" s="19" t="s">
+        <v>59</v>
+      </c>
+      <c r="B3" s="18" t="s">
+        <v>60</v>
+      </c>
+      <c r="C3" s="17">
         <v>1</v>
       </c>
-      <c r="D3" s="15" t="s">
-        <v>51</v>
-      </c>
-      <c r="E3" s="16" t="s">
-        <v>58</v>
-      </c>
-      <c r="F3" s="15" t="s">
-        <v>53</v>
+      <c r="D3" s="17" t="s">
+        <v>61</v>
+      </c>
+      <c r="E3" s="18" t="s">
+        <v>62</v>
+      </c>
+      <c r="F3" s="18" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="15" x14ac:dyDescent="0.2">
-      <c r="A4" s="14" t="s">
-        <v>59</v>
+      <c r="A4" s="19" t="s">
+        <v>64</v>
       </c>
       <c r="B4" s="17" t="s">
-        <v>57</v>
+        <v>65</v>
       </c>
       <c r="C4" s="17">
         <v>1</v>
       </c>
       <c r="D4" s="17" t="s">
+        <v>61</v>
+      </c>
+      <c r="E4" s="18" t="s">
+        <v>66</v>
+      </c>
+      <c r="F4" s="18" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="15" x14ac:dyDescent="0.2">
+      <c r="A5" s="14" t="s">
+        <v>54</v>
+      </c>
+      <c r="B5" s="15" t="s">
+        <v>55</v>
+      </c>
+      <c r="C5" s="15">
+        <v>1</v>
+      </c>
+      <c r="D5" s="15" t="s">
+        <v>49</v>
+      </c>
+      <c r="E5" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="F5" s="15" t="s">
         <v>51</v>
       </c>
-      <c r="E4" s="18" t="s">
-        <v>60</v>
-      </c>
-      <c r="F4" s="17" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" ht="15" x14ac:dyDescent="0.2">
-      <c r="A5" s="19" t="s">
-        <v>61</v>
-      </c>
-      <c r="B5" s="18" t="s">
-        <v>62</v>
-      </c>
-      <c r="C5" s="17">
-        <v>1</v>
-      </c>
-      <c r="D5" s="17" t="s">
-        <v>63</v>
-      </c>
-      <c r="E5" s="18" t="s">
-        <v>64</v>
-      </c>
-      <c r="F5" s="18" t="s">
-        <v>65</v>
-      </c>
     </row>
     <row r="6" spans="1:6" ht="15" x14ac:dyDescent="0.2">
-      <c r="A6" s="19" t="s">
-        <v>66</v>
+      <c r="A6" s="14" t="s">
+        <v>57</v>
       </c>
       <c r="B6" s="17" t="s">
-        <v>67</v>
+        <v>55</v>
       </c>
       <c r="C6" s="17">
         <v>1</v>
       </c>
       <c r="D6" s="17" t="s">
-        <v>63</v>
+        <v>49</v>
       </c>
       <c r="E6" s="18" t="s">
+        <v>58</v>
+      </c>
+      <c r="F6" s="17" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="26" t="s">
+        <v>90</v>
+      </c>
+      <c r="B7" s="36" t="s">
+        <v>91</v>
+      </c>
+      <c r="C7" s="36">
+        <v>1</v>
+      </c>
+      <c r="D7" s="36" t="s">
+        <v>86</v>
+      </c>
+      <c r="E7" s="36" t="s">
+        <v>92</v>
+      </c>
+      <c r="F7" s="36" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="26" t="s">
+        <v>94</v>
+      </c>
+      <c r="B8" s="27" t="s">
+        <v>91</v>
+      </c>
+      <c r="C8" s="27">
+        <v>1</v>
+      </c>
+      <c r="D8" s="27" t="s">
+        <v>86</v>
+      </c>
+      <c r="E8" s="27" t="s">
+        <v>95</v>
+      </c>
+      <c r="F8" s="27" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="26" t="s">
+        <v>96</v>
+      </c>
+      <c r="B9" s="36" t="s">
+        <v>97</v>
+      </c>
+      <c r="C9" s="36">
+        <v>3</v>
+      </c>
+      <c r="D9" s="36" t="s">
+        <v>86</v>
+      </c>
+      <c r="E9" s="36" t="s">
+        <v>98</v>
+      </c>
+      <c r="F9" s="27" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="15" x14ac:dyDescent="0.2">
+      <c r="A10" s="26" t="s">
+        <v>101</v>
+      </c>
+      <c r="B10" s="27" t="s">
+        <v>102</v>
+      </c>
+      <c r="C10" s="27">
+        <v>3</v>
+      </c>
+      <c r="D10" s="27" t="s">
+        <v>49</v>
+      </c>
+      <c r="E10" s="27" t="s">
+        <v>103</v>
+      </c>
+      <c r="F10" s="27" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="12.75" x14ac:dyDescent="0.2"/>
+    <row r="12" spans="1:6" ht="12.75" x14ac:dyDescent="0.2"/>
+    <row r="13" spans="1:6" ht="12.75" x14ac:dyDescent="0.2"/>
+    <row r="14" spans="1:6" ht="12.75" x14ac:dyDescent="0.2"/>
+    <row r="15" spans="1:6" ht="12.75" x14ac:dyDescent="0.2"/>
+    <row r="16" spans="1:6" ht="12.75" x14ac:dyDescent="0.2"/>
+    <row r="17" spans="1:6" ht="12.75" x14ac:dyDescent="0.2"/>
+    <row r="18" spans="1:6" ht="12.75" x14ac:dyDescent="0.2"/>
+    <row r="19" spans="1:6" ht="12.75" x14ac:dyDescent="0.2"/>
+    <row r="20" spans="1:6" ht="12.75" x14ac:dyDescent="0.2"/>
+    <row r="21" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A21" s="20" t="s">
         <v>68</v>
       </c>
-      <c r="F6" s="18" t="s">
+      <c r="B21" s="21" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="34" t="s">
-        <v>103</v>
-      </c>
-      <c r="B7" s="35" t="s">
-        <v>104</v>
-      </c>
-      <c r="C7" s="35">
+      <c r="C21" s="21">
+        <v>2</v>
+      </c>
+      <c r="D21" s="21" t="s">
+        <v>70</v>
+      </c>
+      <c r="E21" s="22" t="s">
+        <v>71</v>
+      </c>
+      <c r="F21" s="21" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A22" s="20" t="s">
+        <v>72</v>
+      </c>
+      <c r="B22" s="23" t="s">
+        <v>69</v>
+      </c>
+      <c r="C22" s="23">
+        <v>2</v>
+      </c>
+      <c r="D22" s="23" t="s">
+        <v>73</v>
+      </c>
+      <c r="E22" s="24" t="s">
+        <v>74</v>
+      </c>
+      <c r="F22" s="23" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A23" s="20" t="s">
+        <v>75</v>
+      </c>
+      <c r="B23" s="21" t="s">
+        <v>69</v>
+      </c>
+      <c r="C23" s="21">
+        <v>2</v>
+      </c>
+      <c r="D23" s="21" t="s">
+        <v>49</v>
+      </c>
+      <c r="E23" s="22" t="s">
+        <v>76</v>
+      </c>
+      <c r="F23" s="22" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A24" s="20" t="s">
+        <v>78</v>
+      </c>
+      <c r="B24" s="23" t="s">
+        <v>69</v>
+      </c>
+      <c r="C24" s="23">
+        <v>2</v>
+      </c>
+      <c r="D24" s="23" t="s">
+        <v>79</v>
+      </c>
+      <c r="E24" s="24" t="s">
+        <v>80</v>
+      </c>
+      <c r="F24" s="23" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A25" s="20" t="s">
+        <v>81</v>
+      </c>
+      <c r="B25" s="21" t="s">
+        <v>69</v>
+      </c>
+      <c r="C25" s="21">
+        <v>2</v>
+      </c>
+      <c r="D25" s="21" t="s">
+        <v>82</v>
+      </c>
+      <c r="E25" s="22" t="s">
+        <v>83</v>
+      </c>
+      <c r="F25" s="21" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A26" s="20" t="s">
+        <v>84</v>
+      </c>
+      <c r="B26" s="21" t="s">
+        <v>85</v>
+      </c>
+      <c r="C26" s="21">
         <v>3</v>
       </c>
-      <c r="D7" s="35" t="s">
+      <c r="D26" s="21" t="s">
+        <v>86</v>
+      </c>
+      <c r="E26" s="22" t="s">
+        <v>87</v>
+      </c>
+      <c r="F26" s="22" t="s">
         <v>51</v>
       </c>
-      <c r="E7" s="35" t="s">
-        <v>105</v>
-      </c>
-      <c r="F7" s="35" t="s">
+    </row>
+    <row r="27" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A27" s="20" t="s">
+        <v>88</v>
+      </c>
+      <c r="B27" s="23" t="s">
+        <v>85</v>
+      </c>
+      <c r="C27" s="23">
+        <v>3</v>
+      </c>
+      <c r="D27" s="23" t="s">
         <v>79</v>
       </c>
-    </row>
-    <row r="10" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A10" s="20" t="s">
-        <v>70</v>
-      </c>
-      <c r="B10" s="21" t="s">
-        <v>71</v>
-      </c>
-      <c r="C10" s="21">
-        <v>2</v>
-      </c>
-      <c r="D10" s="21" t="s">
-        <v>72</v>
-      </c>
-      <c r="E10" s="22" t="s">
-        <v>73</v>
-      </c>
-      <c r="F10" s="21" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A11" s="20" t="s">
-        <v>74</v>
-      </c>
-      <c r="B11" s="23" t="s">
-        <v>71</v>
-      </c>
-      <c r="C11" s="23">
-        <v>2</v>
-      </c>
-      <c r="D11" s="23" t="s">
-        <v>75</v>
-      </c>
-      <c r="E11" s="24" t="s">
-        <v>76</v>
-      </c>
-      <c r="F11" s="23" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A12" s="20" t="s">
-        <v>77</v>
-      </c>
-      <c r="B12" s="21" t="s">
-        <v>71</v>
-      </c>
-      <c r="C12" s="21">
-        <v>2</v>
-      </c>
-      <c r="D12" s="21" t="s">
+      <c r="E27" s="24" t="s">
+        <v>89</v>
+      </c>
+      <c r="F27" s="22" t="s">
         <v>51</v>
       </c>
-      <c r="E12" s="22" t="s">
-        <v>78</v>
-      </c>
-      <c r="F12" s="22" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A13" s="20" t="s">
-        <v>80</v>
-      </c>
-      <c r="B13" s="23" t="s">
-        <v>71</v>
-      </c>
-      <c r="C13" s="23">
-        <v>2</v>
-      </c>
-      <c r="D13" s="23" t="s">
-        <v>81</v>
-      </c>
-      <c r="E13" s="24" t="s">
-        <v>82</v>
-      </c>
-      <c r="F13" s="23" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A14" s="20" t="s">
-        <v>83</v>
-      </c>
-      <c r="B14" s="21" t="s">
-        <v>71</v>
-      </c>
-      <c r="C14" s="21">
-        <v>2</v>
-      </c>
-      <c r="D14" s="21" t="s">
-        <v>84</v>
-      </c>
-      <c r="E14" s="22" t="s">
-        <v>85</v>
-      </c>
-      <c r="F14" s="21" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A15" s="20" t="s">
+    </row>
+    <row r="28" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A28" s="20" t="s">
+        <v>100</v>
+      </c>
+      <c r="B28" s="21" t="s">
+        <v>97</v>
+      </c>
+      <c r="C28" s="21">
+        <v>3</v>
+      </c>
+      <c r="D28" s="21" t="s">
         <v>86</v>
       </c>
-      <c r="B15" s="21" t="s">
-        <v>87</v>
-      </c>
-      <c r="C15" s="21">
-        <v>3</v>
-      </c>
-      <c r="D15" s="21" t="s">
-        <v>88</v>
-      </c>
-      <c r="E15" s="22" t="s">
+      <c r="E28" s="22" t="s">
         <v>89</v>
       </c>
-      <c r="F15" s="22" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A16" s="20" t="s">
-        <v>90</v>
-      </c>
-      <c r="B16" s="23" t="s">
-        <v>87</v>
-      </c>
-      <c r="C16" s="23">
-        <v>3</v>
-      </c>
-      <c r="D16" s="23" t="s">
-        <v>81</v>
-      </c>
-      <c r="E16" s="24" t="s">
-        <v>91</v>
-      </c>
-      <c r="F16" s="22" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A17" s="20" t="s">
-        <v>92</v>
-      </c>
-      <c r="B17" s="23" t="s">
-        <v>93</v>
-      </c>
-      <c r="C17" s="23">
-        <v>1</v>
-      </c>
-      <c r="D17" s="23" t="s">
-        <v>88</v>
-      </c>
-      <c r="E17" s="24" t="s">
-        <v>94</v>
-      </c>
-      <c r="F17" s="23" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A18" s="20" t="s">
-        <v>96</v>
-      </c>
-      <c r="B18" s="21" t="s">
-        <v>93</v>
-      </c>
-      <c r="C18" s="21">
-        <v>1</v>
-      </c>
-      <c r="D18" s="21" t="s">
-        <v>88</v>
-      </c>
-      <c r="E18" s="22" t="s">
-        <v>97</v>
-      </c>
-      <c r="F18" s="21" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A19" s="20" t="s">
-        <v>98</v>
-      </c>
-      <c r="B19" s="23" t="s">
+      <c r="F28" s="22" t="s">
         <v>99</v>
       </c>
-      <c r="C19" s="23">
-        <v>3</v>
-      </c>
-      <c r="D19" s="23" t="s">
-        <v>88</v>
-      </c>
-      <c r="E19" s="24" t="s">
-        <v>100</v>
-      </c>
-      <c r="F19" s="22" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A20" s="20" t="s">
-        <v>102</v>
-      </c>
-      <c r="B20" s="21" t="s">
-        <v>99</v>
-      </c>
-      <c r="C20" s="21">
-        <v>3</v>
-      </c>
-      <c r="D20" s="21" t="s">
-        <v>88</v>
-      </c>
-      <c r="E20" s="22" t="s">
-        <v>91</v>
-      </c>
-      <c r="F20" s="22" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6" ht="12.75" x14ac:dyDescent="0.2"/>
-    <row r="22" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A22" s="20"/>
-      <c r="B22" s="23"/>
-      <c r="C22" s="23"/>
-      <c r="D22" s="23"/>
-      <c r="E22" s="23"/>
-      <c r="F22" s="23"/>
     </row>
     <row r="29" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="20" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="B29" s="23" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C29" s="23">
         <v>3</v>
       </c>
       <c r="D29" s="23" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="E29" s="24" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="F29" s="23" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
     </row>
     <row r="30" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="20" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="B30" s="21" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C30" s="21">
         <v>3</v>
       </c>
       <c r="D30" s="21" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="E30" s="22" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="F30" s="21" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
     </row>
     <row r="31" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="20" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="B31" s="23" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C31" s="23">
         <v>3</v>
       </c>
       <c r="D31" s="23" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="E31" s="24" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="F31" s="23" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
     </row>
   </sheetData>
@@ -2930,47 +2991,47 @@
       <c r="A7" s="8">
         <v>0.42708333333333331</v>
       </c>
-      <c r="B7" s="26" t="s">
-        <v>115</v>
+      <c r="B7" s="28" t="s">
+        <v>113</v>
       </c>
       <c r="C7" s="4"/>
-      <c r="D7" s="26" t="s">
-        <v>115</v>
+      <c r="D7" s="28" t="s">
+        <v>113</v>
       </c>
       <c r="E7" s="4"/>
-      <c r="F7" s="26" t="s">
-        <v>115</v>
+      <c r="F7" s="28" t="s">
+        <v>113</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" s="8">
         <v>0.4375</v>
       </c>
-      <c r="B8" s="31"/>
+      <c r="B8" s="29"/>
       <c r="C8" s="4"/>
-      <c r="D8" s="31"/>
+      <c r="D8" s="29"/>
       <c r="E8" s="4"/>
-      <c r="F8" s="31"/>
+      <c r="F8" s="29"/>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" s="8">
         <v>0.44791666666666669</v>
       </c>
-      <c r="B9" s="31"/>
+      <c r="B9" s="29"/>
       <c r="C9" s="4"/>
-      <c r="D9" s="31"/>
+      <c r="D9" s="29"/>
       <c r="E9" s="4"/>
-      <c r="F9" s="31"/>
+      <c r="F9" s="29"/>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" s="8">
         <v>0.45833333333333331</v>
       </c>
-      <c r="B10" s="31"/>
+      <c r="B10" s="29"/>
       <c r="C10" s="4"/>
-      <c r="D10" s="31"/>
+      <c r="D10" s="29"/>
       <c r="E10" s="4"/>
-      <c r="F10" s="31"/>
+      <c r="F10" s="29"/>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" s="8">
@@ -3086,47 +3147,47 @@
       <c r="A22" s="8">
         <v>0.58333333333333337</v>
       </c>
-      <c r="B22" s="26" t="s">
-        <v>116</v>
+      <c r="B22" s="28" t="s">
+        <v>114</v>
       </c>
       <c r="C22" s="4"/>
-      <c r="D22" s="26" t="s">
-        <v>116</v>
+      <c r="D22" s="28" t="s">
+        <v>114</v>
       </c>
       <c r="E22" s="4"/>
-      <c r="F22" s="26" t="s">
-        <v>116</v>
+      <c r="F22" s="28" t="s">
+        <v>114</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A23" s="8">
         <v>0.59375</v>
       </c>
-      <c r="B23" s="31"/>
+      <c r="B23" s="29"/>
       <c r="C23" s="4"/>
-      <c r="D23" s="31"/>
+      <c r="D23" s="29"/>
       <c r="E23" s="4"/>
-      <c r="F23" s="31"/>
+      <c r="F23" s="29"/>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A24" s="8">
         <v>0.60416666666666663</v>
       </c>
-      <c r="B24" s="31"/>
+      <c r="B24" s="29"/>
       <c r="C24" s="4"/>
-      <c r="D24" s="31"/>
+      <c r="D24" s="29"/>
       <c r="E24" s="4"/>
-      <c r="F24" s="31"/>
+      <c r="F24" s="29"/>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A25" s="8">
         <v>0.61458333333333337</v>
       </c>
-      <c r="B25" s="31"/>
+      <c r="B25" s="29"/>
       <c r="C25" s="4"/>
-      <c r="D25" s="31"/>
+      <c r="D25" s="29"/>
       <c r="E25" s="4"/>
-      <c r="F25" s="31"/>
+      <c r="F25" s="29"/>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A26" s="8">
@@ -3135,7 +3196,7 @@
       <c r="B26" s="4"/>
       <c r="C26" s="4"/>
       <c r="D26" s="1" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="E26" s="4"/>
       <c r="F26" s="4"/>
@@ -3145,46 +3206,46 @@
         <v>0.63541666666666663</v>
       </c>
       <c r="B27" s="30" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="C27" s="6"/>
       <c r="D27" s="30" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="E27" s="6"/>
       <c r="F27" s="30" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A28" s="8">
         <v>0.64583333333333337</v>
       </c>
-      <c r="B28" s="31"/>
+      <c r="B28" s="29"/>
       <c r="C28" s="6"/>
-      <c r="D28" s="31"/>
+      <c r="D28" s="29"/>
       <c r="E28" s="6"/>
-      <c r="F28" s="31"/>
+      <c r="F28" s="29"/>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A29" s="8">
         <v>0.65625</v>
       </c>
-      <c r="B29" s="31"/>
+      <c r="B29" s="29"/>
       <c r="C29" s="6"/>
-      <c r="D29" s="31"/>
+      <c r="D29" s="29"/>
       <c r="E29" s="6"/>
-      <c r="F29" s="31"/>
+      <c r="F29" s="29"/>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A30" s="8">
         <v>0.66666666666666663</v>
       </c>
-      <c r="B30" s="31"/>
+      <c r="B30" s="29"/>
       <c r="C30" s="6"/>
-      <c r="D30" s="31"/>
+      <c r="D30" s="29"/>
       <c r="E30" s="6"/>
-      <c r="F30" s="31"/>
+      <c r="F30" s="29"/>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A31" s="8">

</xml_diff>

<commit_message>
Update at 22:16 on 08/14/2020
</commit_message>
<xml_diff>
--- a/site_libs/records/fall 2020.xlsx
+++ b/site_libs/records/fall 2020.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="23001"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="23029"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Portfolio\site_libs\records\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7098D1C2-84E8-4B42-941C-5EFFFB6396C1}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{868691F6-4BEA-4A3E-94CC-84CB82B4BB95}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="30" yWindow="0" windowWidth="20460" windowHeight="10920" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Schedule" sheetId="1" r:id="rId1"/>
@@ -643,40 +643,40 @@
     <xf numFmtId="0" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="13" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -922,26 +922,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:21" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B1" s="28" t="s">
+      <c r="B1" s="33" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="29"/>
-      <c r="D1" s="28" t="s">
+      <c r="C1" s="38"/>
+      <c r="D1" s="33" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="29"/>
-      <c r="F1" s="28" t="s">
+      <c r="E1" s="38"/>
+      <c r="F1" s="33" t="s">
         <v>2</v>
       </c>
-      <c r="G1" s="29"/>
-      <c r="H1" s="28" t="s">
+      <c r="G1" s="38"/>
+      <c r="H1" s="33" t="s">
         <v>3</v>
       </c>
-      <c r="I1" s="29"/>
-      <c r="J1" s="28" t="s">
+      <c r="I1" s="38"/>
+      <c r="J1" s="33" t="s">
         <v>4</v>
       </c>
-      <c r="K1" s="29"/>
+      <c r="K1" s="38"/>
       <c r="L1" s="1"/>
       <c r="M1" s="2" t="s">
         <v>5</v>
@@ -971,7 +971,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:21" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A2" s="3">
         <v>0.32291666666666669</v>
       </c>
@@ -1020,13 +1020,13 @@
       </c>
       <c r="B3" s="4"/>
       <c r="C3" s="25"/>
-      <c r="D3" s="40" t="s">
+      <c r="D3" s="37" t="s">
         <v>125</v>
       </c>
       <c r="E3" s="6"/>
       <c r="F3" s="6"/>
       <c r="G3" s="6"/>
-      <c r="H3" s="30" t="str">
+      <c r="H3" s="36" t="str">
         <f>D3</f>
         <v>MATH 488
 Data Consulting
@@ -1065,17 +1065,17 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:21" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A4" s="8">
         <v>0.34375</v>
       </c>
       <c r="B4" s="4"/>
       <c r="C4" s="25"/>
-      <c r="D4" s="31"/>
+      <c r="D4" s="34"/>
       <c r="E4" s="6"/>
       <c r="F4" s="6"/>
       <c r="G4" s="6"/>
-      <c r="H4" s="31"/>
+      <c r="H4" s="34"/>
       <c r="I4" s="4"/>
       <c r="J4" s="4"/>
       <c r="K4" s="4"/>
@@ -1114,11 +1114,11 @@
       </c>
       <c r="B5" s="4"/>
       <c r="C5" s="25"/>
-      <c r="D5" s="31"/>
+      <c r="D5" s="34"/>
       <c r="E5" s="6"/>
       <c r="F5" s="6"/>
       <c r="G5" s="6"/>
-      <c r="H5" s="31"/>
+      <c r="H5" s="34"/>
       <c r="I5" s="4"/>
       <c r="J5" s="4"/>
       <c r="K5" s="4"/>
@@ -1129,7 +1129,7 @@
       <c r="N5" s="7">
         <v>488</v>
       </c>
-      <c r="O5" s="39" t="s">
+      <c r="O5" s="30" t="s">
         <v>124</v>
       </c>
       <c r="P5" s="7" t="s">
@@ -1151,17 +1151,17 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:21" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A6" s="8">
         <v>0.36458333333333331</v>
       </c>
       <c r="B6" s="4"/>
       <c r="C6" s="25"/>
-      <c r="D6" s="31"/>
+      <c r="D6" s="34"/>
       <c r="E6" s="6"/>
       <c r="F6" s="6"/>
       <c r="G6" s="6"/>
-      <c r="H6" s="31"/>
+      <c r="H6" s="34"/>
       <c r="I6" s="4"/>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
@@ -1171,39 +1171,39 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:21" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A7" s="8">
         <v>0.375</v>
       </c>
       <c r="B7" s="4"/>
       <c r="C7" s="25"/>
-      <c r="D7" s="31"/>
+      <c r="D7" s="34"/>
       <c r="E7" s="6"/>
       <c r="F7" s="6"/>
       <c r="G7" s="6"/>
-      <c r="H7" s="31"/>
+      <c r="H7" s="34"/>
       <c r="I7" s="4"/>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
       <c r="L7" s="4"/>
     </row>
-    <row r="8" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:21" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A8" s="8">
         <v>0.38541666666666669</v>
       </c>
       <c r="B8" s="4"/>
       <c r="C8" s="25"/>
-      <c r="D8" s="31"/>
+      <c r="D8" s="34"/>
       <c r="E8" s="6"/>
       <c r="F8" s="6"/>
       <c r="G8" s="6"/>
-      <c r="H8" s="31"/>
+      <c r="H8" s="34"/>
       <c r="I8" s="4"/>
       <c r="J8" s="4"/>
       <c r="K8" s="4"/>
       <c r="L8" s="4"/>
     </row>
-    <row r="9" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:21" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A9" s="8">
         <v>0.39583333333333331</v>
       </c>
@@ -1220,7 +1220,7 @@
       <c r="L9" s="4"/>
       <c r="M9" s="9"/>
     </row>
-    <row r="10" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:21" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A10" s="8">
         <v>0.40625</v>
       </c>
@@ -1239,7 +1239,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="11" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:21" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A11" s="8">
         <v>0.41666666666666669</v>
       </c>
@@ -1255,7 +1255,7 @@
       <c r="K11" s="4"/>
       <c r="L11" s="4"/>
     </row>
-    <row r="12" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:21" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A12" s="8">
         <v>0.42708333333333331</v>
       </c>
@@ -1263,7 +1263,7 @@
       <c r="C12" s="32" t="s">
         <v>32</v>
       </c>
-      <c r="D12" s="33" t="s">
+      <c r="D12" s="35" t="s">
         <v>121</v>
       </c>
       <c r="E12" s="4"/>
@@ -1271,7 +1271,7 @@
       <c r="G12" s="32" t="s">
         <v>33</v>
       </c>
-      <c r="H12" s="33" t="str">
+      <c r="H12" s="35" t="str">
         <f>D12</f>
         <v>CSE 121b 
 JavaScript 
@@ -1280,56 +1280,56 @@
       </c>
       <c r="I12" s="4"/>
       <c r="J12" s="4"/>
-      <c r="K12" s="38" t="s">
+      <c r="K12" s="31" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="13" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:21" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A13" s="8">
         <v>0.4375</v>
       </c>
       <c r="B13" s="4"/>
-      <c r="C13" s="31"/>
-      <c r="D13" s="33"/>
+      <c r="C13" s="34"/>
+      <c r="D13" s="35"/>
       <c r="E13" s="4"/>
       <c r="F13" s="4"/>
-      <c r="G13" s="31"/>
-      <c r="H13" s="33"/>
+      <c r="G13" s="34"/>
+      <c r="H13" s="35"/>
       <c r="I13" s="4"/>
       <c r="J13" s="4"/>
-      <c r="K13" s="38"/>
-    </row>
-    <row r="14" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="K13" s="31"/>
+    </row>
+    <row r="14" spans="1:21" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A14" s="8">
         <v>0.44791666666666669</v>
       </c>
       <c r="B14" s="4"/>
-      <c r="C14" s="31"/>
-      <c r="D14" s="33"/>
+      <c r="C14" s="34"/>
+      <c r="D14" s="35"/>
       <c r="E14" s="4"/>
       <c r="F14" s="4"/>
-      <c r="G14" s="31"/>
-      <c r="H14" s="33"/>
+      <c r="G14" s="34"/>
+      <c r="H14" s="35"/>
       <c r="I14" s="4"/>
       <c r="J14" s="4"/>
-      <c r="K14" s="38"/>
-    </row>
-    <row r="15" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="K14" s="31"/>
+    </row>
+    <row r="15" spans="1:21" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A15" s="8">
         <v>0.45833333333333331</v>
       </c>
       <c r="B15" s="4"/>
-      <c r="C15" s="31"/>
-      <c r="D15" s="33"/>
+      <c r="C15" s="34"/>
+      <c r="D15" s="35"/>
       <c r="E15" s="4"/>
       <c r="F15" s="4"/>
-      <c r="G15" s="31"/>
-      <c r="H15" s="33"/>
+      <c r="G15" s="34"/>
+      <c r="H15" s="35"/>
       <c r="I15" s="4"/>
       <c r="J15" s="4"/>
-      <c r="K15" s="38"/>
-    </row>
-    <row r="16" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="K15" s="31"/>
+    </row>
+    <row r="16" spans="1:21" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A16" s="8">
         <v>0.46875</v>
       </c>
@@ -1342,19 +1342,19 @@
       <c r="H16" s="4"/>
       <c r="I16" s="4"/>
       <c r="J16" s="4"/>
-      <c r="K16" s="37"/>
-    </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="K16" s="29"/>
+    </row>
+    <row r="17" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A17" s="8">
         <v>0.47916666666666669</v>
       </c>
-      <c r="B17" s="30" t="s">
+      <c r="B17" s="36" t="s">
         <v>34</v>
       </c>
       <c r="C17" s="25"/>
       <c r="D17" s="12"/>
       <c r="E17" s="12"/>
-      <c r="F17" s="30" t="str">
+      <c r="F17" s="36" t="str">
         <f>B17</f>
         <v>CSE 450
 Machine Learning
@@ -1364,7 +1364,7 @@
       <c r="G17" s="12"/>
       <c r="H17" s="12"/>
       <c r="I17" s="12"/>
-      <c r="J17" s="30" t="str">
+      <c r="J17" s="36" t="str">
         <f>F17</f>
         <v>CSE 450
 Machine Learning
@@ -1373,52 +1373,52 @@
       </c>
       <c r="K17" s="25"/>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A18" s="8">
         <v>0.48958333333333331</v>
       </c>
-      <c r="B18" s="31"/>
+      <c r="B18" s="34"/>
       <c r="C18" s="25"/>
       <c r="D18" s="12"/>
       <c r="E18" s="12"/>
-      <c r="F18" s="31"/>
+      <c r="F18" s="34"/>
       <c r="G18" s="12"/>
       <c r="H18" s="12"/>
       <c r="I18" s="12"/>
-      <c r="J18" s="31"/>
+      <c r="J18" s="34"/>
       <c r="K18" s="25"/>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A19" s="8">
         <v>0.5</v>
       </c>
-      <c r="B19" s="31"/>
+      <c r="B19" s="34"/>
       <c r="C19" s="25"/>
       <c r="D19" s="12"/>
       <c r="E19" s="12"/>
-      <c r="F19" s="31"/>
+      <c r="F19" s="34"/>
       <c r="G19" s="12"/>
       <c r="H19" s="12"/>
       <c r="I19" s="12"/>
-      <c r="J19" s="31"/>
+      <c r="J19" s="34"/>
       <c r="K19" s="25"/>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A20" s="8">
         <v>0.51041666666666663</v>
       </c>
-      <c r="B20" s="31"/>
+      <c r="B20" s="34"/>
       <c r="C20" s="25"/>
       <c r="D20" s="4"/>
       <c r="E20" s="4"/>
-      <c r="F20" s="31"/>
+      <c r="F20" s="34"/>
       <c r="G20" s="4"/>
       <c r="H20" s="4"/>
       <c r="I20" s="4"/>
-      <c r="J20" s="31"/>
+      <c r="J20" s="34"/>
       <c r="K20" s="25"/>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A21" s="8">
         <v>0.52083333333333337</v>
       </c>
@@ -1433,7 +1433,7 @@
       <c r="J21" s="4"/>
       <c r="K21" s="25"/>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A22" s="8">
         <v>0.53125</v>
       </c>
@@ -1453,53 +1453,53 @@
         <v>33</v>
       </c>
       <c r="J22" s="4"/>
-      <c r="K22" s="38" t="s">
+      <c r="K22" s="31" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A23" s="8">
         <v>0.54166666666666663</v>
       </c>
-      <c r="C23" s="31"/>
+      <c r="C23" s="34"/>
       <c r="D23" s="4"/>
-      <c r="E23" s="31"/>
+      <c r="E23" s="34"/>
       <c r="F23" s="4"/>
-      <c r="G23" s="31"/>
+      <c r="G23" s="34"/>
       <c r="H23" s="4"/>
-      <c r="I23" s="31"/>
+      <c r="I23" s="34"/>
       <c r="J23" s="4"/>
-      <c r="K23" s="38"/>
-    </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="K23" s="31"/>
+    </row>
+    <row r="24" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A24" s="8">
         <v>0.55208333333333337</v>
       </c>
-      <c r="C24" s="31"/>
+      <c r="C24" s="34"/>
       <c r="D24" s="4"/>
-      <c r="E24" s="31"/>
+      <c r="E24" s="34"/>
       <c r="F24" s="4"/>
-      <c r="G24" s="31"/>
+      <c r="G24" s="34"/>
       <c r="H24" s="4"/>
-      <c r="I24" s="31"/>
+      <c r="I24" s="34"/>
       <c r="J24" s="4"/>
-      <c r="K24" s="38"/>
-    </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="K24" s="31"/>
+    </row>
+    <row r="25" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A25" s="8">
         <v>0.5625</v>
       </c>
-      <c r="C25" s="31"/>
+      <c r="C25" s="34"/>
       <c r="D25" s="4"/>
-      <c r="E25" s="31"/>
+      <c r="E25" s="34"/>
       <c r="F25" s="4"/>
-      <c r="G25" s="31"/>
+      <c r="G25" s="34"/>
       <c r="H25" s="4"/>
-      <c r="I25" s="31"/>
+      <c r="I25" s="34"/>
       <c r="J25" s="4"/>
-      <c r="K25" s="38"/>
-    </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="K25" s="31"/>
+    </row>
+    <row r="26" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A26" s="8">
         <v>0.57291666666666663</v>
       </c>
@@ -1514,11 +1514,11 @@
       <c r="J26" s="25"/>
       <c r="K26" s="25"/>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A27" s="8">
         <v>0.58333333333333337</v>
       </c>
-      <c r="B27" s="28" t="s">
+      <c r="B27" s="33" t="s">
         <v>35</v>
       </c>
       <c r="C27" s="25"/>
@@ -1526,7 +1526,7 @@
       <c r="E27" s="32" t="s">
         <v>36</v>
       </c>
-      <c r="F27" s="28" t="str">
+      <c r="F27" s="33" t="str">
         <f>B27</f>
         <v>MATH 325
 Intermediate Stats 
@@ -1538,7 +1538,7 @@
       <c r="I27" s="32" t="s">
         <v>36</v>
       </c>
-      <c r="J27" s="28" t="str">
+      <c r="J27" s="33" t="str">
         <f>F27</f>
         <v>MATH 325
 Intermediate Stats 
@@ -1547,52 +1547,52 @@
       </c>
       <c r="K27" s="25"/>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A28" s="8">
         <v>0.59375</v>
       </c>
-      <c r="B28" s="31"/>
+      <c r="B28" s="34"/>
       <c r="C28" s="25"/>
       <c r="D28" s="4"/>
-      <c r="E28" s="31"/>
-      <c r="F28" s="31"/>
+      <c r="E28" s="34"/>
+      <c r="F28" s="34"/>
       <c r="G28" s="25"/>
       <c r="H28" s="4"/>
-      <c r="I28" s="31"/>
-      <c r="J28" s="31"/>
+      <c r="I28" s="34"/>
+      <c r="J28" s="34"/>
       <c r="K28" s="25"/>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A29" s="8">
         <v>0.60416666666666663</v>
       </c>
-      <c r="B29" s="31"/>
+      <c r="B29" s="34"/>
       <c r="C29" s="25"/>
       <c r="D29" s="4"/>
-      <c r="E29" s="31"/>
-      <c r="F29" s="31"/>
+      <c r="E29" s="34"/>
+      <c r="F29" s="34"/>
       <c r="G29" s="25"/>
       <c r="H29" s="4"/>
-      <c r="I29" s="31"/>
-      <c r="J29" s="31"/>
+      <c r="I29" s="34"/>
+      <c r="J29" s="34"/>
       <c r="K29" s="25"/>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A30" s="8">
         <v>0.61458333333333337</v>
       </c>
-      <c r="B30" s="31"/>
+      <c r="B30" s="34"/>
       <c r="C30" s="25"/>
       <c r="D30" s="4"/>
-      <c r="E30" s="31"/>
-      <c r="F30" s="31"/>
+      <c r="E30" s="34"/>
+      <c r="F30" s="34"/>
       <c r="G30" s="25"/>
       <c r="H30" s="4"/>
-      <c r="I30" s="31"/>
-      <c r="J30" s="31"/>
+      <c r="I30" s="34"/>
+      <c r="J30" s="34"/>
       <c r="K30" s="25"/>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A31" s="8">
         <v>0.625</v>
       </c>
@@ -1609,18 +1609,18 @@
       <c r="J31" s="4"/>
       <c r="K31" s="25"/>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A32" s="8">
         <v>0.63541666666666663</v>
       </c>
       <c r="B32" s="6"/>
-      <c r="C32" s="38" t="s">
+      <c r="C32" s="31" t="s">
         <v>122</v>
       </c>
       <c r="D32" s="6"/>
       <c r="E32" s="6"/>
       <c r="F32" s="6"/>
-      <c r="G32" s="38" t="s">
+      <c r="G32" s="31" t="s">
         <v>122</v>
       </c>
       <c r="H32" s="6"/>
@@ -1628,7 +1628,7 @@
       <c r="J32" s="6"/>
       <c r="K32" s="25"/>
     </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A33" s="8">
         <v>0.64583333333333337</v>
       </c>
@@ -1643,7 +1643,7 @@
       <c r="J33" s="6"/>
       <c r="K33" s="25"/>
     </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A34" s="8">
         <v>0.65625</v>
       </c>
@@ -1658,7 +1658,7 @@
       <c r="J34" s="6"/>
       <c r="K34" s="25"/>
     </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A35" s="8">
         <v>0.66666666666666663</v>
       </c>
@@ -1673,7 +1673,7 @@
       <c r="J35" s="6"/>
       <c r="K35" s="25"/>
     </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A36" s="8">
         <v>0.67708333333333337</v>
       </c>
@@ -1695,6 +1695,18 @@
     </row>
   </sheetData>
   <mergeCells count="27">
+    <mergeCell ref="B1:C1"/>
+    <mergeCell ref="D1:E1"/>
+    <mergeCell ref="F1:G1"/>
+    <mergeCell ref="H1:I1"/>
+    <mergeCell ref="J1:K1"/>
+    <mergeCell ref="D3:D8"/>
+    <mergeCell ref="H3:H8"/>
+    <mergeCell ref="E22:E25"/>
+    <mergeCell ref="E27:E30"/>
+    <mergeCell ref="I22:I25"/>
+    <mergeCell ref="I27:I30"/>
+    <mergeCell ref="G22:G25"/>
     <mergeCell ref="C32:C36"/>
     <mergeCell ref="G32:G36"/>
     <mergeCell ref="K12:K15"/>
@@ -1710,18 +1722,6 @@
     <mergeCell ref="F17:F20"/>
     <mergeCell ref="J17:J20"/>
     <mergeCell ref="C22:C25"/>
-    <mergeCell ref="D3:D8"/>
-    <mergeCell ref="H3:H8"/>
-    <mergeCell ref="E22:E25"/>
-    <mergeCell ref="E27:E30"/>
-    <mergeCell ref="I22:I25"/>
-    <mergeCell ref="I27:I30"/>
-    <mergeCell ref="G22:G25"/>
-    <mergeCell ref="B1:C1"/>
-    <mergeCell ref="D1:E1"/>
-    <mergeCell ref="F1:G1"/>
-    <mergeCell ref="H1:I1"/>
-    <mergeCell ref="J1:K1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1755,26 +1755,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="B1" s="28" t="s">
+      <c r="B1" s="33" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="29"/>
-      <c r="D1" s="28" t="s">
+      <c r="C1" s="38"/>
+      <c r="D1" s="33" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="29"/>
-      <c r="F1" s="28" t="s">
+      <c r="E1" s="38"/>
+      <c r="F1" s="33" t="s">
         <v>2</v>
       </c>
-      <c r="G1" s="29"/>
-      <c r="H1" s="28" t="s">
+      <c r="G1" s="38"/>
+      <c r="H1" s="33" t="s">
         <v>3</v>
       </c>
-      <c r="I1" s="29"/>
-      <c r="J1" s="28" t="s">
+      <c r="I1" s="38"/>
+      <c r="J1" s="33" t="s">
         <v>4</v>
       </c>
-      <c r="K1" s="29"/>
+      <c r="K1" s="38"/>
       <c r="L1" s="1"/>
       <c r="M1" s="2" t="s">
         <v>5</v>
@@ -1809,13 +1809,13 @@
         <v>0.33333333333333331</v>
       </c>
       <c r="B2" s="4"/>
-      <c r="D2" s="35" t="s">
+      <c r="D2" s="39" t="s">
         <v>38</v>
       </c>
       <c r="E2" s="4"/>
       <c r="F2" s="4"/>
       <c r="G2" s="4"/>
-      <c r="H2" s="35" t="str">
+      <c r="H2" s="39" t="str">
         <f>D2</f>
         <v>CSE 341
 Web Backend 2
@@ -1859,11 +1859,11 @@
         <v>0.34375</v>
       </c>
       <c r="B3" s="4"/>
-      <c r="D3" s="29"/>
+      <c r="D3" s="38"/>
       <c r="E3" s="4"/>
       <c r="F3" s="4"/>
       <c r="G3" s="4"/>
-      <c r="H3" s="29"/>
+      <c r="H3" s="38"/>
       <c r="I3" s="4"/>
       <c r="J3" s="4"/>
       <c r="K3" s="4"/>
@@ -1901,11 +1901,11 @@
         <v>0.35416666666666669</v>
       </c>
       <c r="B4" s="4"/>
-      <c r="D4" s="29"/>
+      <c r="D4" s="38"/>
       <c r="E4" s="4"/>
       <c r="F4" s="4"/>
       <c r="G4" s="4"/>
-      <c r="H4" s="29"/>
+      <c r="H4" s="38"/>
       <c r="I4" s="4"/>
       <c r="J4" s="4"/>
       <c r="K4" s="4"/>
@@ -1943,11 +1943,11 @@
         <v>0.36458333333333331</v>
       </c>
       <c r="B5" s="4"/>
-      <c r="D5" s="29"/>
+      <c r="D5" s="38"/>
       <c r="E5" s="4"/>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
-      <c r="H5" s="29"/>
+      <c r="H5" s="38"/>
       <c r="I5" s="4"/>
       <c r="J5" s="4"/>
       <c r="K5" s="4"/>
@@ -1985,11 +1985,11 @@
         <v>0.375</v>
       </c>
       <c r="B6" s="4"/>
-      <c r="D6" s="29"/>
+      <c r="D6" s="38"/>
       <c r="E6" s="4"/>
       <c r="F6" s="4"/>
       <c r="G6" s="4"/>
-      <c r="H6" s="29"/>
+      <c r="H6" s="38"/>
       <c r="I6" s="4"/>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
@@ -2000,11 +2000,11 @@
         <v>0.38541666666666669</v>
       </c>
       <c r="B7" s="4"/>
-      <c r="D7" s="29"/>
+      <c r="D7" s="38"/>
       <c r="E7" s="4"/>
       <c r="F7" s="4"/>
       <c r="G7" s="4"/>
-      <c r="H7" s="29"/>
+      <c r="H7" s="38"/>
       <c r="I7" s="4"/>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
@@ -2036,13 +2036,13 @@
         <v>0.40625</v>
       </c>
       <c r="B9" s="4"/>
-      <c r="D9" s="35" t="s">
+      <c r="D9" s="39" t="s">
         <v>46</v>
       </c>
       <c r="E9" s="4"/>
       <c r="F9" s="4"/>
       <c r="G9" s="4"/>
-      <c r="H9" s="35" t="s">
+      <c r="H9" s="39" t="s">
         <v>46</v>
       </c>
       <c r="I9" s="4"/>
@@ -2055,11 +2055,11 @@
         <v>0.41666666666666669</v>
       </c>
       <c r="B10" s="4"/>
-      <c r="D10" s="29"/>
+      <c r="D10" s="38"/>
       <c r="E10" s="4"/>
       <c r="F10" s="4"/>
       <c r="G10" s="4"/>
-      <c r="H10" s="29"/>
+      <c r="H10" s="38"/>
       <c r="I10" s="4"/>
       <c r="J10" s="4"/>
       <c r="K10" s="4"/>
@@ -2070,19 +2070,19 @@
         <v>0.42708333333333331</v>
       </c>
       <c r="B11" s="1"/>
-      <c r="C11" s="34" t="s">
+      <c r="C11" s="40" t="s">
         <v>32</v>
       </c>
-      <c r="D11" s="29"/>
+      <c r="D11" s="38"/>
       <c r="E11" s="4"/>
       <c r="F11" s="1">
         <f>B11</f>
         <v>0</v>
       </c>
-      <c r="G11" s="34" t="s">
+      <c r="G11" s="40" t="s">
         <v>33</v>
       </c>
-      <c r="H11" s="29"/>
+      <c r="H11" s="38"/>
       <c r="I11" s="4"/>
       <c r="J11" s="1"/>
     </row>
@@ -2091,12 +2091,12 @@
         <v>0.4375</v>
       </c>
       <c r="B12" s="1"/>
-      <c r="C12" s="29"/>
-      <c r="D12" s="29"/>
+      <c r="C12" s="38"/>
+      <c r="D12" s="38"/>
       <c r="E12" s="4"/>
       <c r="F12" s="1"/>
-      <c r="G12" s="29"/>
-      <c r="H12" s="29"/>
+      <c r="G12" s="38"/>
+      <c r="H12" s="38"/>
       <c r="I12" s="4"/>
       <c r="J12" s="1"/>
     </row>
@@ -2105,12 +2105,12 @@
         <v>0.44791666666666669</v>
       </c>
       <c r="B13" s="1"/>
-      <c r="C13" s="29"/>
-      <c r="D13" s="29"/>
+      <c r="C13" s="38"/>
+      <c r="D13" s="38"/>
       <c r="E13" s="4"/>
       <c r="F13" s="1"/>
-      <c r="G13" s="29"/>
-      <c r="H13" s="29"/>
+      <c r="G13" s="38"/>
+      <c r="H13" s="38"/>
       <c r="I13" s="4"/>
       <c r="J13" s="1"/>
     </row>
@@ -2119,12 +2119,12 @@
         <v>0.45833333333333331</v>
       </c>
       <c r="B14" s="1"/>
-      <c r="C14" s="29"/>
-      <c r="D14" s="29"/>
+      <c r="C14" s="38"/>
+      <c r="D14" s="38"/>
       <c r="E14" s="4"/>
       <c r="F14" s="1"/>
-      <c r="G14" s="29"/>
-      <c r="H14" s="29"/>
+      <c r="G14" s="38"/>
+      <c r="H14" s="38"/>
       <c r="I14" s="4"/>
       <c r="J14" s="1"/>
     </row>
@@ -2145,12 +2145,12 @@
       <c r="A16" s="8">
         <v>0.47916666666666669</v>
       </c>
-      <c r="B16" s="30" t="s">
+      <c r="B16" s="36" t="s">
         <v>34</v>
       </c>
       <c r="D16" s="12"/>
       <c r="E16" s="12"/>
-      <c r="F16" s="30" t="str">
+      <c r="F16" s="36" t="str">
         <f>B16</f>
         <v>CSE 450
 Machine Learning
@@ -2160,7 +2160,7 @@
       <c r="G16" s="12"/>
       <c r="H16" s="12"/>
       <c r="I16" s="12"/>
-      <c r="J16" s="30" t="str">
+      <c r="J16" s="36" t="str">
         <f>F16</f>
         <v>CSE 450
 Machine Learning
@@ -2172,40 +2172,40 @@
       <c r="A17" s="8">
         <v>0.48958333333333331</v>
       </c>
-      <c r="B17" s="29"/>
+      <c r="B17" s="38"/>
       <c r="D17" s="12"/>
       <c r="E17" s="12"/>
-      <c r="F17" s="29"/>
+      <c r="F17" s="38"/>
       <c r="G17" s="12"/>
       <c r="H17" s="12"/>
       <c r="I17" s="12"/>
-      <c r="J17" s="29"/>
+      <c r="J17" s="38"/>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A18" s="8">
         <v>0.5</v>
       </c>
-      <c r="B18" s="29"/>
+      <c r="B18" s="38"/>
       <c r="D18" s="12"/>
       <c r="E18" s="12"/>
-      <c r="F18" s="29"/>
+      <c r="F18" s="38"/>
       <c r="G18" s="12"/>
       <c r="H18" s="12"/>
       <c r="I18" s="12"/>
-      <c r="J18" s="29"/>
+      <c r="J18" s="38"/>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A19" s="8">
         <v>0.51041666666666663</v>
       </c>
-      <c r="B19" s="29"/>
+      <c r="B19" s="38"/>
       <c r="D19" s="4"/>
       <c r="E19" s="4"/>
-      <c r="F19" s="29"/>
+      <c r="F19" s="38"/>
       <c r="G19" s="4"/>
       <c r="H19" s="4"/>
       <c r="I19" s="4"/>
-      <c r="J19" s="29"/>
+      <c r="J19" s="38"/>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A20" s="8">
@@ -2226,13 +2226,13 @@
       </c>
       <c r="B21" s="4"/>
       <c r="D21" s="4"/>
-      <c r="E21" s="34" t="s">
+      <c r="E21" s="40" t="s">
         <v>32</v>
       </c>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
       <c r="H21" s="4"/>
-      <c r="I21" s="34" t="s">
+      <c r="I21" s="40" t="s">
         <v>33</v>
       </c>
       <c r="J21" s="4"/>
@@ -2243,11 +2243,11 @@
       </c>
       <c r="B22" s="4"/>
       <c r="D22" s="4"/>
-      <c r="E22" s="29"/>
+      <c r="E22" s="38"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
-      <c r="I22" s="29"/>
+      <c r="I22" s="38"/>
       <c r="J22" s="4"/>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.2">
@@ -2256,11 +2256,11 @@
       </c>
       <c r="B23" s="4"/>
       <c r="D23" s="4"/>
-      <c r="E23" s="29"/>
+      <c r="E23" s="38"/>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
-      <c r="I23" s="29"/>
+      <c r="I23" s="38"/>
       <c r="J23" s="4"/>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.2">
@@ -2269,11 +2269,11 @@
       </c>
       <c r="B24" s="4"/>
       <c r="D24" s="4"/>
-      <c r="E24" s="29"/>
+      <c r="E24" s="38"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
-      <c r="I24" s="29"/>
+      <c r="I24" s="38"/>
       <c r="J24" s="4"/>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.2">
@@ -2285,14 +2285,14 @@
       <c r="A26" s="8">
         <v>0.58333333333333337</v>
       </c>
-      <c r="B26" s="28" t="s">
+      <c r="B26" s="33" t="s">
         <v>35</v>
       </c>
       <c r="D26" s="1"/>
       <c r="E26" s="32" t="s">
         <v>36</v>
       </c>
-      <c r="F26" s="28" t="str">
+      <c r="F26" s="33" t="str">
         <f>B26</f>
         <v>MATH 325
 Intermediate Stats 
@@ -2303,7 +2303,7 @@
       <c r="I26" s="32" t="s">
         <v>36</v>
       </c>
-      <c r="J26" s="28" t="str">
+      <c r="J26" s="33" t="str">
         <f>F26</f>
         <v>MATH 325
 Intermediate Stats 
@@ -2315,37 +2315,37 @@
       <c r="A27" s="8">
         <v>0.59375</v>
       </c>
-      <c r="B27" s="29"/>
+      <c r="B27" s="38"/>
       <c r="D27" s="1"/>
-      <c r="E27" s="29"/>
-      <c r="F27" s="29"/>
+      <c r="E27" s="38"/>
+      <c r="F27" s="38"/>
       <c r="H27" s="1"/>
-      <c r="I27" s="29"/>
-      <c r="J27" s="29"/>
+      <c r="I27" s="38"/>
+      <c r="J27" s="38"/>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A28" s="8">
         <v>0.60416666666666663</v>
       </c>
-      <c r="B28" s="29"/>
+      <c r="B28" s="38"/>
       <c r="D28" s="1"/>
-      <c r="E28" s="29"/>
-      <c r="F28" s="29"/>
+      <c r="E28" s="38"/>
+      <c r="F28" s="38"/>
       <c r="H28" s="1"/>
-      <c r="I28" s="29"/>
-      <c r="J28" s="29"/>
+      <c r="I28" s="38"/>
+      <c r="J28" s="38"/>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A29" s="8">
         <v>0.61458333333333337</v>
       </c>
-      <c r="B29" s="29"/>
+      <c r="B29" s="38"/>
       <c r="D29" s="1"/>
-      <c r="E29" s="29"/>
-      <c r="F29" s="29"/>
+      <c r="E29" s="38"/>
+      <c r="F29" s="38"/>
       <c r="H29" s="1"/>
-      <c r="I29" s="29"/>
-      <c r="J29" s="29"/>
+      <c r="I29" s="38"/>
+      <c r="J29" s="38"/>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A30" s="8">
@@ -2433,12 +2433,11 @@
     </row>
   </sheetData>
   <mergeCells count="21">
-    <mergeCell ref="B16:B19"/>
-    <mergeCell ref="F16:F19"/>
-    <mergeCell ref="J16:J19"/>
-    <mergeCell ref="B26:B29"/>
-    <mergeCell ref="F26:F29"/>
-    <mergeCell ref="J26:J29"/>
+    <mergeCell ref="B1:C1"/>
+    <mergeCell ref="D1:E1"/>
+    <mergeCell ref="F1:G1"/>
+    <mergeCell ref="H1:I1"/>
+    <mergeCell ref="C11:C14"/>
     <mergeCell ref="J1:K1"/>
     <mergeCell ref="D2:D7"/>
     <mergeCell ref="D9:D14"/>
@@ -2449,11 +2448,12 @@
     <mergeCell ref="G11:G14"/>
     <mergeCell ref="H2:H7"/>
     <mergeCell ref="H9:H14"/>
-    <mergeCell ref="B1:C1"/>
-    <mergeCell ref="D1:E1"/>
-    <mergeCell ref="F1:G1"/>
-    <mergeCell ref="H1:I1"/>
-    <mergeCell ref="C11:C14"/>
+    <mergeCell ref="B16:B19"/>
+    <mergeCell ref="F16:F19"/>
+    <mergeCell ref="J16:J19"/>
+    <mergeCell ref="B26:B29"/>
+    <mergeCell ref="F26:F29"/>
+    <mergeCell ref="J26:J29"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2597,19 +2597,19 @@
       <c r="A7" s="26" t="s">
         <v>90</v>
       </c>
-      <c r="B7" s="36" t="s">
+      <c r="B7" s="28" t="s">
         <v>91</v>
       </c>
-      <c r="C7" s="36">
+      <c r="C7" s="28">
         <v>1</v>
       </c>
-      <c r="D7" s="36" t="s">
+      <c r="D7" s="28" t="s">
         <v>86</v>
       </c>
-      <c r="E7" s="36" t="s">
+      <c r="E7" s="28" t="s">
         <v>92</v>
       </c>
-      <c r="F7" s="36" t="s">
+      <c r="F7" s="28" t="s">
         <v>93</v>
       </c>
     </row>
@@ -2637,16 +2637,16 @@
       <c r="A9" s="26" t="s">
         <v>96</v>
       </c>
-      <c r="B9" s="36" t="s">
+      <c r="B9" s="28" t="s">
         <v>97</v>
       </c>
-      <c r="C9" s="36">
+      <c r="C9" s="28">
         <v>3</v>
       </c>
-      <c r="D9" s="36" t="s">
+      <c r="D9" s="28" t="s">
         <v>86</v>
       </c>
-      <c r="E9" s="36" t="s">
+      <c r="E9" s="28" t="s">
         <v>98</v>
       </c>
       <c r="F9" s="27" t="s">
@@ -2991,15 +2991,15 @@
       <c r="A7" s="8">
         <v>0.42708333333333331</v>
       </c>
-      <c r="B7" s="28" t="s">
+      <c r="B7" s="33" t="s">
         <v>113</v>
       </c>
       <c r="C7" s="4"/>
-      <c r="D7" s="28" t="s">
+      <c r="D7" s="33" t="s">
         <v>113</v>
       </c>
       <c r="E7" s="4"/>
-      <c r="F7" s="28" t="s">
+      <c r="F7" s="33" t="s">
         <v>113</v>
       </c>
     </row>
@@ -3007,31 +3007,31 @@
       <c r="A8" s="8">
         <v>0.4375</v>
       </c>
-      <c r="B8" s="29"/>
+      <c r="B8" s="38"/>
       <c r="C8" s="4"/>
-      <c r="D8" s="29"/>
+      <c r="D8" s="38"/>
       <c r="E8" s="4"/>
-      <c r="F8" s="29"/>
+      <c r="F8" s="38"/>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" s="8">
         <v>0.44791666666666669</v>
       </c>
-      <c r="B9" s="29"/>
+      <c r="B9" s="38"/>
       <c r="C9" s="4"/>
-      <c r="D9" s="29"/>
+      <c r="D9" s="38"/>
       <c r="E9" s="4"/>
-      <c r="F9" s="29"/>
+      <c r="F9" s="38"/>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" s="8">
         <v>0.45833333333333331</v>
       </c>
-      <c r="B10" s="29"/>
+      <c r="B10" s="38"/>
       <c r="C10" s="4"/>
-      <c r="D10" s="29"/>
+      <c r="D10" s="38"/>
       <c r="E10" s="4"/>
-      <c r="F10" s="29"/>
+      <c r="F10" s="38"/>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" s="8">
@@ -3147,15 +3147,15 @@
       <c r="A22" s="8">
         <v>0.58333333333333337</v>
       </c>
-      <c r="B22" s="28" t="s">
+      <c r="B22" s="33" t="s">
         <v>114</v>
       </c>
       <c r="C22" s="4"/>
-      <c r="D22" s="28" t="s">
+      <c r="D22" s="33" t="s">
         <v>114</v>
       </c>
       <c r="E22" s="4"/>
-      <c r="F22" s="28" t="s">
+      <c r="F22" s="33" t="s">
         <v>114</v>
       </c>
     </row>
@@ -3163,31 +3163,31 @@
       <c r="A23" s="8">
         <v>0.59375</v>
       </c>
-      <c r="B23" s="29"/>
+      <c r="B23" s="38"/>
       <c r="C23" s="4"/>
-      <c r="D23" s="29"/>
+      <c r="D23" s="38"/>
       <c r="E23" s="4"/>
-      <c r="F23" s="29"/>
+      <c r="F23" s="38"/>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A24" s="8">
         <v>0.60416666666666663</v>
       </c>
-      <c r="B24" s="29"/>
+      <c r="B24" s="38"/>
       <c r="C24" s="4"/>
-      <c r="D24" s="29"/>
+      <c r="D24" s="38"/>
       <c r="E24" s="4"/>
-      <c r="F24" s="29"/>
+      <c r="F24" s="38"/>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A25" s="8">
         <v>0.61458333333333337</v>
       </c>
-      <c r="B25" s="29"/>
+      <c r="B25" s="38"/>
       <c r="C25" s="4"/>
-      <c r="D25" s="29"/>
+      <c r="D25" s="38"/>
       <c r="E25" s="4"/>
-      <c r="F25" s="29"/>
+      <c r="F25" s="38"/>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A26" s="8">
@@ -3205,15 +3205,15 @@
       <c r="A27" s="8">
         <v>0.63541666666666663</v>
       </c>
-      <c r="B27" s="30" t="s">
+      <c r="B27" s="36" t="s">
         <v>115</v>
       </c>
       <c r="C27" s="6"/>
-      <c r="D27" s="30" t="s">
+      <c r="D27" s="36" t="s">
         <v>115</v>
       </c>
       <c r="E27" s="6"/>
-      <c r="F27" s="30" t="s">
+      <c r="F27" s="36" t="s">
         <v>115</v>
       </c>
     </row>
@@ -3221,31 +3221,31 @@
       <c r="A28" s="8">
         <v>0.64583333333333337</v>
       </c>
-      <c r="B28" s="29"/>
+      <c r="B28" s="38"/>
       <c r="C28" s="6"/>
-      <c r="D28" s="29"/>
+      <c r="D28" s="38"/>
       <c r="E28" s="6"/>
-      <c r="F28" s="29"/>
+      <c r="F28" s="38"/>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A29" s="8">
         <v>0.65625</v>
       </c>
-      <c r="B29" s="29"/>
+      <c r="B29" s="38"/>
       <c r="C29" s="6"/>
-      <c r="D29" s="29"/>
+      <c r="D29" s="38"/>
       <c r="E29" s="6"/>
-      <c r="F29" s="29"/>
+      <c r="F29" s="38"/>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A30" s="8">
         <v>0.66666666666666663</v>
       </c>
-      <c r="B30" s="29"/>
+      <c r="B30" s="38"/>
       <c r="C30" s="6"/>
-      <c r="D30" s="29"/>
+      <c r="D30" s="38"/>
       <c r="E30" s="6"/>
-      <c r="F30" s="29"/>
+      <c r="F30" s="38"/>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A31" s="8">

</xml_diff>

<commit_message>
Update at 22:29 on 08/14/2020
</commit_message>
<xml_diff>
--- a/site_libs/records/fall 2020.xlsx
+++ b/site_libs/records/fall 2020.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Portfolio\site_libs\records\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{868691F6-4BEA-4A3E-94CC-84CB82B4BB95}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C00CCAC3-EEF5-41ED-92FC-78DCE6F15CC8}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="30" yWindow="0" windowWidth="20460" windowHeight="10920" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="233" uniqueCount="126">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="235" uniqueCount="124">
   <si>
     <t>Monday</t>
   </si>
@@ -113,16 +113,7 @@
     <t>Saunders</t>
   </si>
   <si>
-    <t>Rks</t>
-  </si>
-  <si>
     <t>TR</t>
-  </si>
-  <si>
-    <t>8:00-9:30</t>
-  </si>
-  <si>
-    <t>Hathaway</t>
   </si>
   <si>
     <t>Possible</t>
@@ -440,20 +431,20 @@
 Jack</t>
   </si>
   <si>
-    <t>Data Consulting</t>
-  </si>
-  <si>
-    <t>MATH 488
-Data Consulting
-Hathaway
-Rks 229</t>
+    <t>8:00-9:00</t>
+  </si>
+  <si>
+    <t>2:00-3:00</t>
+  </si>
+  <si>
+    <t>CSE 341 Web Backend 2 Birch Remote</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="16" x14ac:knownFonts="1">
+  <fonts count="17" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -540,6 +531,10 @@
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Arial"/>
     </font>
   </fonts>
   <fills count="4">
@@ -649,34 +644,36 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -900,7 +897,7 @@
   <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="11.7109375" customWidth="1"/>
-    <col min="2" max="2" width="11.28515625" customWidth="1"/>
+    <col min="2" max="2" width="11.140625" customWidth="1"/>
     <col min="3" max="3" width="9.42578125" customWidth="1"/>
     <col min="4" max="4" width="10.42578125" customWidth="1"/>
     <col min="5" max="5" width="8.7109375" customWidth="1"/>
@@ -908,10 +905,10 @@
     <col min="7" max="7" width="9.42578125" customWidth="1"/>
     <col min="8" max="8" width="10.140625" customWidth="1"/>
     <col min="9" max="9" width="9.85546875" customWidth="1"/>
-    <col min="10" max="10" width="11.28515625" customWidth="1"/>
-    <col min="11" max="11" width="9.42578125" customWidth="1"/>
-    <col min="12" max="12" width="6" customWidth="1"/>
-    <col min="13" max="13" width="10.85546875" customWidth="1"/>
+    <col min="10" max="10" width="11.7109375" customWidth="1"/>
+    <col min="11" max="11" width="6.140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="4" customWidth="1"/>
+    <col min="13" max="13" width="10.5703125" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="5.5703125" customWidth="1"/>
     <col min="15" max="15" width="16.140625" customWidth="1"/>
     <col min="16" max="17" width="7.7109375" customWidth="1"/>
@@ -922,26 +919,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:21" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B1" s="33" t="s">
+      <c r="B1" s="30" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="38"/>
-      <c r="D1" s="33" t="s">
+      <c r="C1" s="31"/>
+      <c r="D1" s="30" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="38"/>
-      <c r="F1" s="33" t="s">
+      <c r="E1" s="31"/>
+      <c r="F1" s="30" t="s">
         <v>2</v>
       </c>
-      <c r="G1" s="38"/>
-      <c r="H1" s="33" t="s">
+      <c r="G1" s="31"/>
+      <c r="H1" s="30" t="s">
         <v>3</v>
       </c>
-      <c r="I1" s="38"/>
-      <c r="J1" s="33" t="s">
+      <c r="I1" s="31"/>
+      <c r="J1" s="30" t="s">
         <v>4</v>
       </c>
-      <c r="K1" s="38"/>
+      <c r="K1" s="31"/>
       <c r="L1" s="1"/>
       <c r="M1" s="2" t="s">
         <v>5</v>
@@ -990,10 +987,10 @@
         <v>14</v>
       </c>
       <c r="N2" s="13" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="O2" s="13" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="P2" s="7" t="s">
         <v>22</v>
@@ -1002,13 +999,13 @@
         <v>23</v>
       </c>
       <c r="R2" s="13" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="S2" s="13" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="T2" s="13" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="U2" s="13">
         <v>1</v>
@@ -1020,48 +1017,44 @@
       </c>
       <c r="B3" s="4"/>
       <c r="C3" s="25"/>
-      <c r="D3" s="37" t="s">
-        <v>125</v>
-      </c>
-      <c r="E3" s="6"/>
-      <c r="F3" s="6"/>
-      <c r="G3" s="6"/>
-      <c r="H3" s="36" t="str">
-        <f>D3</f>
-        <v>MATH 488
-Data Consulting
-Hathaway
-Rks 229</v>
+      <c r="D3" s="32" t="s">
+        <v>123</v>
+      </c>
+      <c r="E3" s="40"/>
+      <c r="F3" s="40"/>
+      <c r="G3" s="40"/>
+      <c r="H3" s="32" t="s">
+        <v>123</v>
       </c>
       <c r="I3" s="4"/>
       <c r="J3" s="4"/>
       <c r="K3" s="4"/>
       <c r="L3" s="4"/>
-      <c r="M3" s="7" t="s">
+      <c r="M3" t="s">
         <v>14</v>
       </c>
-      <c r="N3" s="7">
-        <v>450</v>
-      </c>
-      <c r="O3" s="7" t="s">
-        <v>15</v>
+      <c r="N3">
+        <v>341</v>
+      </c>
+      <c r="O3" t="s">
+        <v>40</v>
       </c>
       <c r="P3" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="Q3" s="7">
-        <v>347</v>
-      </c>
-      <c r="R3" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="S3" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="T3" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="U3" s="7">
+        <v>22</v>
+      </c>
+      <c r="Q3" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="R3" s="13" t="s">
+        <v>26</v>
+      </c>
+      <c r="S3" s="13" t="s">
+        <v>121</v>
+      </c>
+      <c r="T3" s="13" t="s">
+        <v>42</v>
+      </c>
+      <c r="U3" s="13">
         <v>3</v>
       </c>
     </row>
@@ -1071,38 +1064,38 @@
       </c>
       <c r="B4" s="4"/>
       <c r="C4" s="25"/>
-      <c r="D4" s="34"/>
-      <c r="E4" s="6"/>
-      <c r="F4" s="6"/>
-      <c r="G4" s="6"/>
-      <c r="H4" s="34"/>
+      <c r="D4" s="32"/>
+      <c r="E4" s="40"/>
+      <c r="F4" s="40"/>
+      <c r="G4" s="40"/>
+      <c r="H4" s="32"/>
       <c r="I4" s="4"/>
       <c r="J4" s="4"/>
       <c r="K4" s="4"/>
       <c r="L4" s="4"/>
       <c r="M4" s="7" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="N4" s="7">
-        <v>325</v>
+        <v>450</v>
       </c>
       <c r="O4" s="7" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="P4" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="Q4" s="7" t="s">
-        <v>23</v>
+        <v>16</v>
+      </c>
+      <c r="Q4" s="7">
+        <v>347</v>
       </c>
       <c r="R4" s="7" t="s">
         <v>17</v>
       </c>
       <c r="S4" s="7" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="T4" s="7" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="U4" s="7">
         <v>3</v>
@@ -1114,11 +1107,11 @@
       </c>
       <c r="B5" s="4"/>
       <c r="C5" s="25"/>
-      <c r="D5" s="34"/>
-      <c r="E5" s="6"/>
-      <c r="F5" s="6"/>
-      <c r="G5" s="6"/>
-      <c r="H5" s="34"/>
+      <c r="D5" s="32"/>
+      <c r="E5" s="40"/>
+      <c r="F5" s="40"/>
+      <c r="G5" s="40"/>
+      <c r="H5" s="32"/>
       <c r="I5" s="4"/>
       <c r="J5" s="4"/>
       <c r="K5" s="4"/>
@@ -1127,25 +1120,25 @@
         <v>20</v>
       </c>
       <c r="N5" s="7">
-        <v>488</v>
-      </c>
-      <c r="O5" s="30" t="s">
-        <v>124</v>
+        <v>325</v>
+      </c>
+      <c r="O5" s="7" t="s">
+        <v>21</v>
       </c>
       <c r="P5" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="Q5" s="7">
-        <v>229</v>
+        <v>22</v>
+      </c>
+      <c r="Q5" s="7" t="s">
+        <v>23</v>
       </c>
       <c r="R5" s="7" t="s">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="S5" s="7" t="s">
-        <v>28</v>
+        <v>122</v>
       </c>
       <c r="T5" s="7" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="U5" s="7">
         <v>3</v>
@@ -1157,11 +1150,11 @@
       </c>
       <c r="B6" s="4"/>
       <c r="C6" s="25"/>
-      <c r="D6" s="34"/>
-      <c r="E6" s="6"/>
-      <c r="F6" s="6"/>
-      <c r="G6" s="6"/>
-      <c r="H6" s="34"/>
+      <c r="D6" s="32"/>
+      <c r="E6" s="40"/>
+      <c r="F6" s="40"/>
+      <c r="G6" s="40"/>
+      <c r="H6" s="32"/>
       <c r="I6" s="4"/>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
@@ -1177,11 +1170,11 @@
       </c>
       <c r="B7" s="4"/>
       <c r="C7" s="25"/>
-      <c r="D7" s="34"/>
-      <c r="E7" s="6"/>
-      <c r="F7" s="6"/>
-      <c r="G7" s="6"/>
-      <c r="H7" s="34"/>
+      <c r="D7" s="32"/>
+      <c r="E7" s="40"/>
+      <c r="F7" s="40"/>
+      <c r="G7" s="40"/>
+      <c r="H7" s="32"/>
       <c r="I7" s="4"/>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
@@ -1193,11 +1186,11 @@
       </c>
       <c r="B8" s="4"/>
       <c r="C8" s="25"/>
-      <c r="D8" s="34"/>
-      <c r="E8" s="6"/>
-      <c r="F8" s="6"/>
-      <c r="G8" s="6"/>
-      <c r="H8" s="34"/>
+      <c r="D8" s="32"/>
+      <c r="E8" s="40"/>
+      <c r="F8" s="40"/>
+      <c r="G8" s="40"/>
+      <c r="H8" s="32"/>
       <c r="I8" s="4"/>
       <c r="J8" s="4"/>
       <c r="K8" s="4"/>
@@ -1236,7 +1229,7 @@
       <c r="K10" s="4"/>
       <c r="L10" s="4"/>
       <c r="M10" s="10" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
     </row>
     <row r="11" spans="1:21" ht="12.75" x14ac:dyDescent="0.2">
@@ -1260,18 +1253,18 @@
         <v>0.42708333333333331</v>
       </c>
       <c r="B12" s="4"/>
-      <c r="C12" s="32" t="s">
-        <v>32</v>
-      </c>
-      <c r="D12" s="35" t="s">
-        <v>121</v>
+      <c r="C12" s="35" t="s">
+        <v>29</v>
+      </c>
+      <c r="D12" s="37" t="s">
+        <v>118</v>
       </c>
       <c r="E12" s="4"/>
       <c r="F12" s="4"/>
-      <c r="G12" s="32" t="s">
-        <v>33</v>
-      </c>
-      <c r="H12" s="35" t="str">
+      <c r="G12" s="35" t="s">
+        <v>30</v>
+      </c>
+      <c r="H12" s="37" t="str">
         <f>D12</f>
         <v>CSE 121b 
 JavaScript 
@@ -1280,8 +1273,8 @@
       </c>
       <c r="I12" s="4"/>
       <c r="J12" s="4"/>
-      <c r="K12" s="31" t="s">
-        <v>123</v>
+      <c r="K12" s="36" t="s">
+        <v>120</v>
       </c>
     </row>
     <row r="13" spans="1:21" ht="12.75" x14ac:dyDescent="0.2">
@@ -1289,45 +1282,45 @@
         <v>0.4375</v>
       </c>
       <c r="B13" s="4"/>
-      <c r="C13" s="34"/>
-      <c r="D13" s="35"/>
+      <c r="C13" s="33"/>
+      <c r="D13" s="37"/>
       <c r="E13" s="4"/>
       <c r="F13" s="4"/>
-      <c r="G13" s="34"/>
-      <c r="H13" s="35"/>
+      <c r="G13" s="33"/>
+      <c r="H13" s="37"/>
       <c r="I13" s="4"/>
       <c r="J13" s="4"/>
-      <c r="K13" s="31"/>
+      <c r="K13" s="36"/>
     </row>
     <row r="14" spans="1:21" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A14" s="8">
         <v>0.44791666666666669</v>
       </c>
       <c r="B14" s="4"/>
-      <c r="C14" s="34"/>
-      <c r="D14" s="35"/>
+      <c r="C14" s="33"/>
+      <c r="D14" s="37"/>
       <c r="E14" s="4"/>
       <c r="F14" s="4"/>
-      <c r="G14" s="34"/>
-      <c r="H14" s="35"/>
+      <c r="G14" s="33"/>
+      <c r="H14" s="37"/>
       <c r="I14" s="4"/>
       <c r="J14" s="4"/>
-      <c r="K14" s="31"/>
+      <c r="K14" s="36"/>
     </row>
     <row r="15" spans="1:21" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A15" s="8">
         <v>0.45833333333333331</v>
       </c>
       <c r="B15" s="4"/>
-      <c r="C15" s="34"/>
-      <c r="D15" s="35"/>
+      <c r="C15" s="33"/>
+      <c r="D15" s="37"/>
       <c r="E15" s="4"/>
       <c r="F15" s="4"/>
-      <c r="G15" s="34"/>
-      <c r="H15" s="35"/>
+      <c r="G15" s="33"/>
+      <c r="H15" s="37"/>
       <c r="I15" s="4"/>
       <c r="J15" s="4"/>
-      <c r="K15" s="31"/>
+      <c r="K15" s="36"/>
     </row>
     <row r="16" spans="1:21" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A16" s="8">
@@ -1348,13 +1341,13 @@
       <c r="A17" s="8">
         <v>0.47916666666666669</v>
       </c>
-      <c r="B17" s="36" t="s">
-        <v>34</v>
+      <c r="B17" s="32" t="s">
+        <v>31</v>
       </c>
       <c r="C17" s="25"/>
       <c r="D17" s="12"/>
       <c r="E17" s="12"/>
-      <c r="F17" s="36" t="str">
+      <c r="F17" s="34" t="str">
         <f>B17</f>
         <v>CSE 450
 Machine Learning
@@ -1364,7 +1357,7 @@
       <c r="G17" s="12"/>
       <c r="H17" s="12"/>
       <c r="I17" s="12"/>
-      <c r="J17" s="36" t="str">
+      <c r="J17" s="34" t="str">
         <f>F17</f>
         <v>CSE 450
 Machine Learning
@@ -1377,45 +1370,45 @@
       <c r="A18" s="8">
         <v>0.48958333333333331</v>
       </c>
-      <c r="B18" s="34"/>
+      <c r="B18" s="33"/>
       <c r="C18" s="25"/>
       <c r="D18" s="12"/>
       <c r="E18" s="12"/>
-      <c r="F18" s="34"/>
+      <c r="F18" s="33"/>
       <c r="G18" s="12"/>
       <c r="H18" s="12"/>
       <c r="I18" s="12"/>
-      <c r="J18" s="34"/>
+      <c r="J18" s="33"/>
       <c r="K18" s="25"/>
     </row>
     <row r="19" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A19" s="8">
         <v>0.5</v>
       </c>
-      <c r="B19" s="34"/>
+      <c r="B19" s="33"/>
       <c r="C19" s="25"/>
       <c r="D19" s="12"/>
       <c r="E19" s="12"/>
-      <c r="F19" s="34"/>
+      <c r="F19" s="33"/>
       <c r="G19" s="12"/>
       <c r="H19" s="12"/>
       <c r="I19" s="12"/>
-      <c r="J19" s="34"/>
+      <c r="J19" s="33"/>
       <c r="K19" s="25"/>
     </row>
     <row r="20" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A20" s="8">
         <v>0.51041666666666663</v>
       </c>
-      <c r="B20" s="34"/>
+      <c r="B20" s="33"/>
       <c r="C20" s="25"/>
       <c r="D20" s="4"/>
       <c r="E20" s="4"/>
-      <c r="F20" s="34"/>
+      <c r="F20" s="33"/>
       <c r="G20" s="4"/>
       <c r="H20" s="4"/>
       <c r="I20" s="4"/>
-      <c r="J20" s="34"/>
+      <c r="J20" s="33"/>
       <c r="K20" s="25"/>
     </row>
     <row r="21" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
@@ -1437,67 +1430,67 @@
       <c r="A22" s="8">
         <v>0.53125</v>
       </c>
-      <c r="C22" s="32" t="s">
+      <c r="C22" s="35" t="s">
+        <v>117</v>
+      </c>
+      <c r="D22" s="4"/>
+      <c r="E22" s="35" t="s">
+        <v>29</v>
+      </c>
+      <c r="F22" s="4"/>
+      <c r="G22" s="35" t="s">
+        <v>117</v>
+      </c>
+      <c r="H22" s="4"/>
+      <c r="I22" s="35" t="s">
+        <v>30</v>
+      </c>
+      <c r="J22" s="4"/>
+      <c r="K22" s="36" t="s">
         <v>120</v>
-      </c>
-      <c r="D22" s="4"/>
-      <c r="E22" s="32" t="s">
-        <v>32</v>
-      </c>
-      <c r="F22" s="4"/>
-      <c r="G22" s="32" t="s">
-        <v>120</v>
-      </c>
-      <c r="H22" s="4"/>
-      <c r="I22" s="32" t="s">
-        <v>33</v>
-      </c>
-      <c r="J22" s="4"/>
-      <c r="K22" s="31" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="23" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A23" s="8">
         <v>0.54166666666666663</v>
       </c>
-      <c r="C23" s="34"/>
+      <c r="C23" s="33"/>
       <c r="D23" s="4"/>
-      <c r="E23" s="34"/>
+      <c r="E23" s="33"/>
       <c r="F23" s="4"/>
-      <c r="G23" s="34"/>
+      <c r="G23" s="33"/>
       <c r="H23" s="4"/>
-      <c r="I23" s="34"/>
+      <c r="I23" s="33"/>
       <c r="J23" s="4"/>
-      <c r="K23" s="31"/>
+      <c r="K23" s="36"/>
     </row>
     <row r="24" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A24" s="8">
         <v>0.55208333333333337</v>
       </c>
-      <c r="C24" s="34"/>
+      <c r="C24" s="33"/>
       <c r="D24" s="4"/>
-      <c r="E24" s="34"/>
+      <c r="E24" s="33"/>
       <c r="F24" s="4"/>
-      <c r="G24" s="34"/>
+      <c r="G24" s="33"/>
       <c r="H24" s="4"/>
-      <c r="I24" s="34"/>
+      <c r="I24" s="33"/>
       <c r="J24" s="4"/>
-      <c r="K24" s="31"/>
+      <c r="K24" s="36"/>
     </row>
     <row r="25" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A25" s="8">
         <v>0.5625</v>
       </c>
-      <c r="C25" s="34"/>
+      <c r="C25" s="33"/>
       <c r="D25" s="4"/>
-      <c r="E25" s="34"/>
+      <c r="E25" s="33"/>
       <c r="F25" s="4"/>
-      <c r="G25" s="34"/>
+      <c r="G25" s="33"/>
       <c r="H25" s="4"/>
-      <c r="I25" s="34"/>
+      <c r="I25" s="33"/>
       <c r="J25" s="4"/>
-      <c r="K25" s="31"/>
+      <c r="K25" s="36"/>
     </row>
     <row r="26" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A26" s="8">
@@ -1518,15 +1511,15 @@
       <c r="A27" s="8">
         <v>0.58333333333333337</v>
       </c>
-      <c r="B27" s="33" t="s">
-        <v>35</v>
+      <c r="B27" s="30" t="s">
+        <v>32</v>
       </c>
       <c r="C27" s="25"/>
       <c r="D27" s="4"/>
-      <c r="E27" s="32" t="s">
-        <v>36</v>
-      </c>
-      <c r="F27" s="33" t="str">
+      <c r="E27" s="35" t="s">
+        <v>33</v>
+      </c>
+      <c r="F27" s="30" t="str">
         <f>B27</f>
         <v>MATH 325
 Intermediate Stats 
@@ -1535,10 +1528,10 @@
       </c>
       <c r="G27" s="25"/>
       <c r="H27" s="4"/>
-      <c r="I27" s="32" t="s">
-        <v>36</v>
-      </c>
-      <c r="J27" s="33" t="str">
+      <c r="I27" s="35" t="s">
+        <v>33</v>
+      </c>
+      <c r="J27" s="30" t="str">
         <f>F27</f>
         <v>MATH 325
 Intermediate Stats 
@@ -1551,45 +1544,45 @@
       <c r="A28" s="8">
         <v>0.59375</v>
       </c>
-      <c r="B28" s="34"/>
+      <c r="B28" s="33"/>
       <c r="C28" s="25"/>
       <c r="D28" s="4"/>
-      <c r="E28" s="34"/>
-      <c r="F28" s="34"/>
+      <c r="E28" s="33"/>
+      <c r="F28" s="33"/>
       <c r="G28" s="25"/>
       <c r="H28" s="4"/>
-      <c r="I28" s="34"/>
-      <c r="J28" s="34"/>
+      <c r="I28" s="33"/>
+      <c r="J28" s="33"/>
       <c r="K28" s="25"/>
     </row>
     <row r="29" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A29" s="8">
         <v>0.60416666666666663</v>
       </c>
-      <c r="B29" s="34"/>
+      <c r="B29" s="33"/>
       <c r="C29" s="25"/>
       <c r="D29" s="4"/>
-      <c r="E29" s="34"/>
-      <c r="F29" s="34"/>
+      <c r="E29" s="33"/>
+      <c r="F29" s="33"/>
       <c r="G29" s="25"/>
       <c r="H29" s="4"/>
-      <c r="I29" s="34"/>
-      <c r="J29" s="34"/>
+      <c r="I29" s="33"/>
+      <c r="J29" s="33"/>
       <c r="K29" s="25"/>
     </row>
     <row r="30" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A30" s="8">
         <v>0.61458333333333337</v>
       </c>
-      <c r="B30" s="34"/>
+      <c r="B30" s="33"/>
       <c r="C30" s="25"/>
       <c r="D30" s="4"/>
-      <c r="E30" s="34"/>
-      <c r="F30" s="34"/>
+      <c r="E30" s="33"/>
+      <c r="F30" s="33"/>
       <c r="G30" s="25"/>
       <c r="H30" s="4"/>
-      <c r="I30" s="34"/>
-      <c r="J30" s="34"/>
+      <c r="I30" s="33"/>
+      <c r="J30" s="33"/>
       <c r="K30" s="25"/>
     </row>
     <row r="31" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
@@ -1601,7 +1594,7 @@
       <c r="D31" s="4"/>
       <c r="E31" s="4"/>
       <c r="F31" s="4" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="G31" s="25"/>
       <c r="H31" s="4"/>
@@ -1614,14 +1607,14 @@
         <v>0.63541666666666663</v>
       </c>
       <c r="B32" s="6"/>
-      <c r="C32" s="31" t="s">
-        <v>122</v>
+      <c r="C32" s="36" t="s">
+        <v>119</v>
       </c>
       <c r="D32" s="6"/>
       <c r="E32" s="6"/>
       <c r="F32" s="6"/>
-      <c r="G32" s="31" t="s">
-        <v>122</v>
+      <c r="G32" s="36" t="s">
+        <v>119</v>
       </c>
       <c r="H32" s="6"/>
       <c r="I32" s="6"/>
@@ -1633,11 +1626,11 @@
         <v>0.64583333333333337</v>
       </c>
       <c r="B33" s="6"/>
-      <c r="C33" s="32"/>
+      <c r="C33" s="35"/>
       <c r="D33" s="6"/>
       <c r="E33" s="6"/>
       <c r="F33" s="6"/>
-      <c r="G33" s="32"/>
+      <c r="G33" s="35"/>
       <c r="H33" s="6"/>
       <c r="I33" s="6"/>
       <c r="J33" s="6"/>
@@ -1648,11 +1641,11 @@
         <v>0.65625</v>
       </c>
       <c r="B34" s="6"/>
-      <c r="C34" s="32"/>
+      <c r="C34" s="35"/>
       <c r="D34" s="6"/>
       <c r="E34" s="6"/>
       <c r="F34" s="6"/>
-      <c r="G34" s="32"/>
+      <c r="G34" s="35"/>
       <c r="H34" s="6"/>
       <c r="I34" s="6"/>
       <c r="J34" s="6"/>
@@ -1663,11 +1656,11 @@
         <v>0.66666666666666663</v>
       </c>
       <c r="B35" s="6"/>
-      <c r="C35" s="32"/>
+      <c r="C35" s="35"/>
       <c r="D35" s="6"/>
       <c r="E35" s="6"/>
       <c r="F35" s="6"/>
-      <c r="G35" s="32"/>
+      <c r="G35" s="35"/>
       <c r="H35" s="6"/>
       <c r="I35" s="6"/>
       <c r="J35" s="6"/>
@@ -1678,11 +1671,11 @@
         <v>0.67708333333333337</v>
       </c>
       <c r="B36" s="4"/>
-      <c r="C36" s="32"/>
+      <c r="C36" s="35"/>
       <c r="D36" s="4"/>
       <c r="E36" s="4"/>
       <c r="F36" s="4"/>
-      <c r="G36" s="32"/>
+      <c r="G36" s="35"/>
       <c r="H36" s="4"/>
       <c r="I36" s="4"/>
       <c r="J36" s="4"/>
@@ -1695,18 +1688,6 @@
     </row>
   </sheetData>
   <mergeCells count="27">
-    <mergeCell ref="B1:C1"/>
-    <mergeCell ref="D1:E1"/>
-    <mergeCell ref="F1:G1"/>
-    <mergeCell ref="H1:I1"/>
-    <mergeCell ref="J1:K1"/>
-    <mergeCell ref="D3:D8"/>
-    <mergeCell ref="H3:H8"/>
-    <mergeCell ref="E22:E25"/>
-    <mergeCell ref="E27:E30"/>
-    <mergeCell ref="I22:I25"/>
-    <mergeCell ref="I27:I30"/>
-    <mergeCell ref="G22:G25"/>
     <mergeCell ref="C32:C36"/>
     <mergeCell ref="G32:G36"/>
     <mergeCell ref="K12:K15"/>
@@ -1722,8 +1703,22 @@
     <mergeCell ref="F17:F20"/>
     <mergeCell ref="J17:J20"/>
     <mergeCell ref="C22:C25"/>
+    <mergeCell ref="D3:D8"/>
+    <mergeCell ref="H3:H8"/>
+    <mergeCell ref="E22:E25"/>
+    <mergeCell ref="E27:E30"/>
+    <mergeCell ref="I22:I25"/>
+    <mergeCell ref="I27:I30"/>
+    <mergeCell ref="G22:G25"/>
+    <mergeCell ref="B1:C1"/>
+    <mergeCell ref="D1:E1"/>
+    <mergeCell ref="F1:G1"/>
+    <mergeCell ref="H1:I1"/>
+    <mergeCell ref="J1:K1"/>
   </mergeCells>
+  <phoneticPr fontId="16" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1755,26 +1750,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="B1" s="33" t="s">
+      <c r="B1" s="30" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="38"/>
-      <c r="D1" s="33" t="s">
+      <c r="C1" s="31"/>
+      <c r="D1" s="30" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="38"/>
-      <c r="F1" s="33" t="s">
+      <c r="E1" s="31"/>
+      <c r="F1" s="30" t="s">
         <v>2</v>
       </c>
-      <c r="G1" s="38"/>
-      <c r="H1" s="33" t="s">
+      <c r="G1" s="31"/>
+      <c r="H1" s="30" t="s">
         <v>3</v>
       </c>
-      <c r="I1" s="38"/>
-      <c r="J1" s="33" t="s">
+      <c r="I1" s="31"/>
+      <c r="J1" s="30" t="s">
         <v>4</v>
       </c>
-      <c r="K1" s="38"/>
+      <c r="K1" s="31"/>
       <c r="L1" s="1"/>
       <c r="M1" s="2" t="s">
         <v>5</v>
@@ -1810,7 +1805,7 @@
       </c>
       <c r="B2" s="4"/>
       <c r="D2" s="39" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="E2" s="4"/>
       <c r="F2" s="4"/>
@@ -1859,11 +1854,11 @@
         <v>0.34375</v>
       </c>
       <c r="B3" s="4"/>
-      <c r="D3" s="38"/>
+      <c r="D3" s="31"/>
       <c r="E3" s="4"/>
       <c r="F3" s="4"/>
       <c r="G3" s="4"/>
-      <c r="H3" s="38"/>
+      <c r="H3" s="31"/>
       <c r="I3" s="4"/>
       <c r="J3" s="4"/>
       <c r="K3" s="4"/>
@@ -1901,23 +1896,23 @@
         <v>0.35416666666666669</v>
       </c>
       <c r="B4" s="4"/>
-      <c r="D4" s="38"/>
+      <c r="D4" s="31"/>
       <c r="E4" s="4"/>
       <c r="F4" s="4"/>
       <c r="G4" s="4"/>
-      <c r="H4" s="38"/>
+      <c r="H4" s="31"/>
       <c r="I4" s="4"/>
       <c r="J4" s="4"/>
       <c r="K4" s="4"/>
       <c r="L4" s="4"/>
       <c r="M4" s="2" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="N4" s="2">
         <v>330</v>
       </c>
       <c r="O4" s="2" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="P4" s="2" t="s">
         <v>16</v>
@@ -1926,13 +1921,13 @@
         <v>347</v>
       </c>
       <c r="R4" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="S4" s="2" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="T4" s="13" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="U4" s="2">
         <v>3</v>
@@ -1943,11 +1938,11 @@
         <v>0.36458333333333331</v>
       </c>
       <c r="B5" s="4"/>
-      <c r="D5" s="38"/>
+      <c r="D5" s="31"/>
       <c r="E5" s="4"/>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
-      <c r="H5" s="38"/>
+      <c r="H5" s="31"/>
       <c r="I5" s="4"/>
       <c r="J5" s="4"/>
       <c r="K5" s="4"/>
@@ -1959,7 +1954,7 @@
         <v>341</v>
       </c>
       <c r="O5" s="2" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="P5" s="2" t="s">
         <v>22</v>
@@ -1968,13 +1963,13 @@
         <v>23</v>
       </c>
       <c r="R5" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="S5" s="2" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="T5" s="13" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="U5" s="2">
         <v>3</v>
@@ -1985,11 +1980,11 @@
         <v>0.375</v>
       </c>
       <c r="B6" s="4"/>
-      <c r="D6" s="38"/>
+      <c r="D6" s="31"/>
       <c r="E6" s="4"/>
       <c r="F6" s="4"/>
       <c r="G6" s="4"/>
-      <c r="H6" s="38"/>
+      <c r="H6" s="31"/>
       <c r="I6" s="4"/>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
@@ -2000,17 +1995,17 @@
         <v>0.38541666666666669</v>
       </c>
       <c r="B7" s="4"/>
-      <c r="D7" s="38"/>
+      <c r="D7" s="31"/>
       <c r="E7" s="4"/>
       <c r="F7" s="4"/>
       <c r="G7" s="4"/>
-      <c r="H7" s="38"/>
+      <c r="H7" s="31"/>
       <c r="I7" s="4"/>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
       <c r="L7" s="4"/>
       <c r="M7" s="9" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
     </row>
     <row r="8" spans="1:21" x14ac:dyDescent="0.2">
@@ -2028,7 +2023,7 @@
       <c r="K8" s="4"/>
       <c r="L8" s="4"/>
       <c r="M8" s="10" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
     </row>
     <row r="9" spans="1:21" x14ac:dyDescent="0.2">
@@ -2037,13 +2032,13 @@
       </c>
       <c r="B9" s="4"/>
       <c r="D9" s="39" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="E9" s="4"/>
       <c r="F9" s="4"/>
       <c r="G9" s="4"/>
       <c r="H9" s="39" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="I9" s="4"/>
       <c r="J9" s="4"/>
@@ -2055,11 +2050,11 @@
         <v>0.41666666666666669</v>
       </c>
       <c r="B10" s="4"/>
-      <c r="D10" s="38"/>
+      <c r="D10" s="31"/>
       <c r="E10" s="4"/>
       <c r="F10" s="4"/>
       <c r="G10" s="4"/>
-      <c r="H10" s="38"/>
+      <c r="H10" s="31"/>
       <c r="I10" s="4"/>
       <c r="J10" s="4"/>
       <c r="K10" s="4"/>
@@ -2070,19 +2065,19 @@
         <v>0.42708333333333331</v>
       </c>
       <c r="B11" s="1"/>
-      <c r="C11" s="40" t="s">
-        <v>32</v>
-      </c>
-      <c r="D11" s="38"/>
+      <c r="C11" s="38" t="s">
+        <v>29</v>
+      </c>
+      <c r="D11" s="31"/>
       <c r="E11" s="4"/>
       <c r="F11" s="1">
         <f>B11</f>
         <v>0</v>
       </c>
-      <c r="G11" s="40" t="s">
-        <v>33</v>
-      </c>
-      <c r="H11" s="38"/>
+      <c r="G11" s="38" t="s">
+        <v>30</v>
+      </c>
+      <c r="H11" s="31"/>
       <c r="I11" s="4"/>
       <c r="J11" s="1"/>
     </row>
@@ -2091,12 +2086,12 @@
         <v>0.4375</v>
       </c>
       <c r="B12" s="1"/>
-      <c r="C12" s="38"/>
-      <c r="D12" s="38"/>
+      <c r="C12" s="31"/>
+      <c r="D12" s="31"/>
       <c r="E12" s="4"/>
       <c r="F12" s="1"/>
-      <c r="G12" s="38"/>
-      <c r="H12" s="38"/>
+      <c r="G12" s="31"/>
+      <c r="H12" s="31"/>
       <c r="I12" s="4"/>
       <c r="J12" s="1"/>
     </row>
@@ -2105,12 +2100,12 @@
         <v>0.44791666666666669</v>
       </c>
       <c r="B13" s="1"/>
-      <c r="C13" s="38"/>
-      <c r="D13" s="38"/>
+      <c r="C13" s="31"/>
+      <c r="D13" s="31"/>
       <c r="E13" s="4"/>
       <c r="F13" s="1"/>
-      <c r="G13" s="38"/>
-      <c r="H13" s="38"/>
+      <c r="G13" s="31"/>
+      <c r="H13" s="31"/>
       <c r="I13" s="4"/>
       <c r="J13" s="1"/>
     </row>
@@ -2119,12 +2114,12 @@
         <v>0.45833333333333331</v>
       </c>
       <c r="B14" s="1"/>
-      <c r="C14" s="38"/>
-      <c r="D14" s="38"/>
+      <c r="C14" s="31"/>
+      <c r="D14" s="31"/>
       <c r="E14" s="4"/>
       <c r="F14" s="1"/>
-      <c r="G14" s="38"/>
-      <c r="H14" s="38"/>
+      <c r="G14" s="31"/>
+      <c r="H14" s="31"/>
       <c r="I14" s="4"/>
       <c r="J14" s="1"/>
     </row>
@@ -2145,12 +2140,12 @@
       <c r="A16" s="8">
         <v>0.47916666666666669</v>
       </c>
-      <c r="B16" s="36" t="s">
-        <v>34</v>
+      <c r="B16" s="34" t="s">
+        <v>31</v>
       </c>
       <c r="D16" s="12"/>
       <c r="E16" s="12"/>
-      <c r="F16" s="36" t="str">
+      <c r="F16" s="34" t="str">
         <f>B16</f>
         <v>CSE 450
 Machine Learning
@@ -2160,7 +2155,7 @@
       <c r="G16" s="12"/>
       <c r="H16" s="12"/>
       <c r="I16" s="12"/>
-      <c r="J16" s="36" t="str">
+      <c r="J16" s="34" t="str">
         <f>F16</f>
         <v>CSE 450
 Machine Learning
@@ -2172,40 +2167,40 @@
       <c r="A17" s="8">
         <v>0.48958333333333331</v>
       </c>
-      <c r="B17" s="38"/>
+      <c r="B17" s="31"/>
       <c r="D17" s="12"/>
       <c r="E17" s="12"/>
-      <c r="F17" s="38"/>
+      <c r="F17" s="31"/>
       <c r="G17" s="12"/>
       <c r="H17" s="12"/>
       <c r="I17" s="12"/>
-      <c r="J17" s="38"/>
+      <c r="J17" s="31"/>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A18" s="8">
         <v>0.5</v>
       </c>
-      <c r="B18" s="38"/>
+      <c r="B18" s="31"/>
       <c r="D18" s="12"/>
       <c r="E18" s="12"/>
-      <c r="F18" s="38"/>
+      <c r="F18" s="31"/>
       <c r="G18" s="12"/>
       <c r="H18" s="12"/>
       <c r="I18" s="12"/>
-      <c r="J18" s="38"/>
+      <c r="J18" s="31"/>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A19" s="8">
         <v>0.51041666666666663</v>
       </c>
-      <c r="B19" s="38"/>
+      <c r="B19" s="31"/>
       <c r="D19" s="4"/>
       <c r="E19" s="4"/>
-      <c r="F19" s="38"/>
+      <c r="F19" s="31"/>
       <c r="G19" s="4"/>
       <c r="H19" s="4"/>
       <c r="I19" s="4"/>
-      <c r="J19" s="38"/>
+      <c r="J19" s="31"/>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A20" s="8">
@@ -2226,14 +2221,14 @@
       </c>
       <c r="B21" s="4"/>
       <c r="D21" s="4"/>
-      <c r="E21" s="40" t="s">
-        <v>32</v>
+      <c r="E21" s="38" t="s">
+        <v>29</v>
       </c>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
       <c r="H21" s="4"/>
-      <c r="I21" s="40" t="s">
-        <v>33</v>
+      <c r="I21" s="38" t="s">
+        <v>30</v>
       </c>
       <c r="J21" s="4"/>
     </row>
@@ -2243,11 +2238,11 @@
       </c>
       <c r="B22" s="4"/>
       <c r="D22" s="4"/>
-      <c r="E22" s="38"/>
+      <c r="E22" s="31"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
-      <c r="I22" s="38"/>
+      <c r="I22" s="31"/>
       <c r="J22" s="4"/>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.2">
@@ -2256,11 +2251,11 @@
       </c>
       <c r="B23" s="4"/>
       <c r="D23" s="4"/>
-      <c r="E23" s="38"/>
+      <c r="E23" s="31"/>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
-      <c r="I23" s="38"/>
+      <c r="I23" s="31"/>
       <c r="J23" s="4"/>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.2">
@@ -2269,11 +2264,11 @@
       </c>
       <c r="B24" s="4"/>
       <c r="D24" s="4"/>
-      <c r="E24" s="38"/>
+      <c r="E24" s="31"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
-      <c r="I24" s="38"/>
+      <c r="I24" s="31"/>
       <c r="J24" s="4"/>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.2">
@@ -2285,14 +2280,14 @@
       <c r="A26" s="8">
         <v>0.58333333333333337</v>
       </c>
-      <c r="B26" s="33" t="s">
-        <v>35</v>
+      <c r="B26" s="30" t="s">
+        <v>32</v>
       </c>
       <c r="D26" s="1"/>
-      <c r="E26" s="32" t="s">
-        <v>36</v>
-      </c>
-      <c r="F26" s="33" t="str">
+      <c r="E26" s="35" t="s">
+        <v>33</v>
+      </c>
+      <c r="F26" s="30" t="str">
         <f>B26</f>
         <v>MATH 325
 Intermediate Stats 
@@ -2300,10 +2295,10 @@
 Remote</v>
       </c>
       <c r="H26" s="1"/>
-      <c r="I26" s="32" t="s">
-        <v>36</v>
-      </c>
-      <c r="J26" s="33" t="str">
+      <c r="I26" s="35" t="s">
+        <v>33</v>
+      </c>
+      <c r="J26" s="30" t="str">
         <f>F26</f>
         <v>MATH 325
 Intermediate Stats 
@@ -2315,37 +2310,37 @@
       <c r="A27" s="8">
         <v>0.59375</v>
       </c>
-      <c r="B27" s="38"/>
+      <c r="B27" s="31"/>
       <c r="D27" s="1"/>
-      <c r="E27" s="38"/>
-      <c r="F27" s="38"/>
+      <c r="E27" s="31"/>
+      <c r="F27" s="31"/>
       <c r="H27" s="1"/>
-      <c r="I27" s="38"/>
-      <c r="J27" s="38"/>
+      <c r="I27" s="31"/>
+      <c r="J27" s="31"/>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A28" s="8">
         <v>0.60416666666666663</v>
       </c>
-      <c r="B28" s="38"/>
+      <c r="B28" s="31"/>
       <c r="D28" s="1"/>
-      <c r="E28" s="38"/>
-      <c r="F28" s="38"/>
+      <c r="E28" s="31"/>
+      <c r="F28" s="31"/>
       <c r="H28" s="1"/>
-      <c r="I28" s="38"/>
-      <c r="J28" s="38"/>
+      <c r="I28" s="31"/>
+      <c r="J28" s="31"/>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A29" s="8">
         <v>0.61458333333333337</v>
       </c>
-      <c r="B29" s="38"/>
+      <c r="B29" s="31"/>
       <c r="D29" s="1"/>
-      <c r="E29" s="38"/>
-      <c r="F29" s="38"/>
+      <c r="E29" s="31"/>
+      <c r="F29" s="31"/>
       <c r="H29" s="1"/>
-      <c r="I29" s="38"/>
-      <c r="J29" s="38"/>
+      <c r="I29" s="31"/>
+      <c r="J29" s="31"/>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A30" s="8">
@@ -2355,7 +2350,7 @@
       <c r="D30" s="4"/>
       <c r="E30" s="4"/>
       <c r="F30" s="1" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="H30" s="4"/>
       <c r="I30" s="4"/>
@@ -2433,11 +2428,12 @@
     </row>
   </sheetData>
   <mergeCells count="21">
-    <mergeCell ref="B1:C1"/>
-    <mergeCell ref="D1:E1"/>
-    <mergeCell ref="F1:G1"/>
-    <mergeCell ref="H1:I1"/>
-    <mergeCell ref="C11:C14"/>
+    <mergeCell ref="B16:B19"/>
+    <mergeCell ref="F16:F19"/>
+    <mergeCell ref="J16:J19"/>
+    <mergeCell ref="B26:B29"/>
+    <mergeCell ref="F26:F29"/>
+    <mergeCell ref="J26:J29"/>
     <mergeCell ref="J1:K1"/>
     <mergeCell ref="D2:D7"/>
     <mergeCell ref="D9:D14"/>
@@ -2448,12 +2444,11 @@
     <mergeCell ref="G11:G14"/>
     <mergeCell ref="H2:H7"/>
     <mergeCell ref="H9:H14"/>
-    <mergeCell ref="B16:B19"/>
-    <mergeCell ref="F16:F19"/>
-    <mergeCell ref="J16:J19"/>
-    <mergeCell ref="B26:B29"/>
-    <mergeCell ref="F26:F29"/>
-    <mergeCell ref="J26:J29"/>
+    <mergeCell ref="B1:C1"/>
+    <mergeCell ref="D1:E1"/>
+    <mergeCell ref="F1:G1"/>
+    <mergeCell ref="H1:I1"/>
+    <mergeCell ref="C11:C14"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2475,202 +2470,202 @@
   <sheetData>
     <row r="1" spans="1:6" ht="15" x14ac:dyDescent="0.2">
       <c r="A1" s="14" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="B1" s="15" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="C1" s="15">
         <v>1</v>
       </c>
       <c r="D1" s="15" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="E1" s="16" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="F1" s="15" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="15" x14ac:dyDescent="0.2">
       <c r="A2" s="14" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="B2" s="17" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="C2" s="17">
         <v>1</v>
       </c>
       <c r="D2" s="17" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="E2" s="18" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="F2" s="17" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="15" x14ac:dyDescent="0.2">
       <c r="A3" s="19" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="B3" s="18" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="C3" s="17">
         <v>1</v>
       </c>
       <c r="D3" s="17" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="E3" s="18" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="F3" s="18" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="15" x14ac:dyDescent="0.2">
       <c r="A4" s="19" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="B4" s="17" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="C4" s="17">
         <v>1</v>
       </c>
       <c r="D4" s="17" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="E4" s="18" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="F4" s="18" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="15" x14ac:dyDescent="0.2">
       <c r="A5" s="14" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="B5" s="15" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="C5" s="15">
         <v>1</v>
       </c>
       <c r="D5" s="15" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="E5" s="16" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="F5" s="15" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="15" x14ac:dyDescent="0.2">
       <c r="A6" s="14" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="B6" s="17" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="C6" s="17">
         <v>1</v>
       </c>
       <c r="D6" s="17" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="E6" s="18" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="F6" s="17" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="26" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="B7" s="28" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="C7" s="28">
         <v>1</v>
       </c>
       <c r="D7" s="28" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="E7" s="28" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="F7" s="28" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="26" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="B8" s="27" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="C8" s="27">
         <v>1</v>
       </c>
       <c r="D8" s="27" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="E8" s="27" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="F8" s="27" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="26" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="B9" s="28" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="C9" s="28">
         <v>3</v>
       </c>
       <c r="D9" s="28" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="E9" s="28" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="F9" s="27" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="15" x14ac:dyDescent="0.2">
       <c r="A10" s="26" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="B10" s="27" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="C10" s="27">
         <v>3</v>
       </c>
       <c r="D10" s="27" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="E10" s="27" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="F10" s="27" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="12.75" x14ac:dyDescent="0.2"/>
@@ -2685,222 +2680,222 @@
     <row r="20" spans="1:6" ht="12.75" x14ac:dyDescent="0.2"/>
     <row r="21" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A21" s="20" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="B21" s="21" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="C21" s="21">
         <v>2</v>
       </c>
       <c r="D21" s="21" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="E21" s="22" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="F21" s="21" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
     </row>
     <row r="22" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A22" s="20" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="B22" s="23" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="C22" s="23">
         <v>2</v>
       </c>
       <c r="D22" s="23" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="E22" s="24" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="F22" s="23" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
     </row>
     <row r="23" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="20" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="B23" s="21" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="C23" s="21">
         <v>2</v>
       </c>
       <c r="D23" s="21" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="E23" s="22" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="F23" s="22" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
     </row>
     <row r="24" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="20" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="B24" s="23" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="C24" s="23">
         <v>2</v>
       </c>
       <c r="D24" s="23" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="E24" s="24" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="F24" s="23" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
     </row>
     <row r="25" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="20" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="B25" s="21" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="C25" s="21">
         <v>2</v>
       </c>
       <c r="D25" s="21" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="E25" s="22" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="F25" s="21" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
     </row>
     <row r="26" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="20" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="B26" s="21" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="C26" s="21">
         <v>3</v>
       </c>
       <c r="D26" s="21" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="E26" s="22" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="F26" s="22" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
     </row>
     <row r="27" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="20" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="B27" s="23" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="C27" s="23">
         <v>3</v>
       </c>
       <c r="D27" s="23" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="E27" s="24" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="F27" s="22" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
     </row>
     <row r="28" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="20" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="B28" s="21" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="C28" s="21">
         <v>3</v>
       </c>
       <c r="D28" s="21" t="s">
+        <v>83</v>
+      </c>
+      <c r="E28" s="22" t="s">
         <v>86</v>
       </c>
-      <c r="E28" s="22" t="s">
-        <v>89</v>
-      </c>
       <c r="F28" s="22" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
     </row>
     <row r="29" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="20" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="B29" s="23" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="C29" s="23">
         <v>3</v>
       </c>
       <c r="D29" s="23" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="E29" s="24" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="F29" s="23" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
     </row>
     <row r="30" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="20" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="B30" s="21" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="C30" s="21">
         <v>3</v>
       </c>
       <c r="D30" s="21" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="E30" s="22" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="F30" s="21" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
     </row>
     <row r="31" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="20" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="B31" s="23" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="C31" s="23">
         <v>3</v>
       </c>
       <c r="D31" s="23" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="E31" s="24" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="F31" s="23" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
     </row>
   </sheetData>
@@ -2991,47 +2986,47 @@
       <c r="A7" s="8">
         <v>0.42708333333333331</v>
       </c>
-      <c r="B7" s="33" t="s">
-        <v>113</v>
+      <c r="B7" s="30" t="s">
+        <v>110</v>
       </c>
       <c r="C7" s="4"/>
-      <c r="D7" s="33" t="s">
-        <v>113</v>
+      <c r="D7" s="30" t="s">
+        <v>110</v>
       </c>
       <c r="E7" s="4"/>
-      <c r="F7" s="33" t="s">
-        <v>113</v>
+      <c r="F7" s="30" t="s">
+        <v>110</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" s="8">
         <v>0.4375</v>
       </c>
-      <c r="B8" s="38"/>
+      <c r="B8" s="31"/>
       <c r="C8" s="4"/>
-      <c r="D8" s="38"/>
+      <c r="D8" s="31"/>
       <c r="E8" s="4"/>
-      <c r="F8" s="38"/>
+      <c r="F8" s="31"/>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" s="8">
         <v>0.44791666666666669</v>
       </c>
-      <c r="B9" s="38"/>
+      <c r="B9" s="31"/>
       <c r="C9" s="4"/>
-      <c r="D9" s="38"/>
+      <c r="D9" s="31"/>
       <c r="E9" s="4"/>
-      <c r="F9" s="38"/>
+      <c r="F9" s="31"/>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" s="8">
         <v>0.45833333333333331</v>
       </c>
-      <c r="B10" s="38"/>
+      <c r="B10" s="31"/>
       <c r="C10" s="4"/>
-      <c r="D10" s="38"/>
+      <c r="D10" s="31"/>
       <c r="E10" s="4"/>
-      <c r="F10" s="38"/>
+      <c r="F10" s="31"/>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" s="8">
@@ -3147,47 +3142,47 @@
       <c r="A22" s="8">
         <v>0.58333333333333337</v>
       </c>
-      <c r="B22" s="33" t="s">
-        <v>114</v>
+      <c r="B22" s="30" t="s">
+        <v>111</v>
       </c>
       <c r="C22" s="4"/>
-      <c r="D22" s="33" t="s">
-        <v>114</v>
+      <c r="D22" s="30" t="s">
+        <v>111</v>
       </c>
       <c r="E22" s="4"/>
-      <c r="F22" s="33" t="s">
-        <v>114</v>
+      <c r="F22" s="30" t="s">
+        <v>111</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A23" s="8">
         <v>0.59375</v>
       </c>
-      <c r="B23" s="38"/>
+      <c r="B23" s="31"/>
       <c r="C23" s="4"/>
-      <c r="D23" s="38"/>
+      <c r="D23" s="31"/>
       <c r="E23" s="4"/>
-      <c r="F23" s="38"/>
+      <c r="F23" s="31"/>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A24" s="8">
         <v>0.60416666666666663</v>
       </c>
-      <c r="B24" s="38"/>
+      <c r="B24" s="31"/>
       <c r="C24" s="4"/>
-      <c r="D24" s="38"/>
+      <c r="D24" s="31"/>
       <c r="E24" s="4"/>
-      <c r="F24" s="38"/>
+      <c r="F24" s="31"/>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A25" s="8">
         <v>0.61458333333333337</v>
       </c>
-      <c r="B25" s="38"/>
+      <c r="B25" s="31"/>
       <c r="C25" s="4"/>
-      <c r="D25" s="38"/>
+      <c r="D25" s="31"/>
       <c r="E25" s="4"/>
-      <c r="F25" s="38"/>
+      <c r="F25" s="31"/>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A26" s="8">
@@ -3196,7 +3191,7 @@
       <c r="B26" s="4"/>
       <c r="C26" s="4"/>
       <c r="D26" s="1" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="E26" s="4"/>
       <c r="F26" s="4"/>
@@ -3205,47 +3200,47 @@
       <c r="A27" s="8">
         <v>0.63541666666666663</v>
       </c>
-      <c r="B27" s="36" t="s">
-        <v>115</v>
+      <c r="B27" s="34" t="s">
+        <v>112</v>
       </c>
       <c r="C27" s="6"/>
-      <c r="D27" s="36" t="s">
-        <v>115</v>
+      <c r="D27" s="34" t="s">
+        <v>112</v>
       </c>
       <c r="E27" s="6"/>
-      <c r="F27" s="36" t="s">
-        <v>115</v>
+      <c r="F27" s="34" t="s">
+        <v>112</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A28" s="8">
         <v>0.64583333333333337</v>
       </c>
-      <c r="B28" s="38"/>
+      <c r="B28" s="31"/>
       <c r="C28" s="6"/>
-      <c r="D28" s="38"/>
+      <c r="D28" s="31"/>
       <c r="E28" s="6"/>
-      <c r="F28" s="38"/>
+      <c r="F28" s="31"/>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A29" s="8">
         <v>0.65625</v>
       </c>
-      <c r="B29" s="38"/>
+      <c r="B29" s="31"/>
       <c r="C29" s="6"/>
-      <c r="D29" s="38"/>
+      <c r="D29" s="31"/>
       <c r="E29" s="6"/>
-      <c r="F29" s="38"/>
+      <c r="F29" s="31"/>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A30" s="8">
         <v>0.66666666666666663</v>
       </c>
-      <c r="B30" s="38"/>
+      <c r="B30" s="31"/>
       <c r="C30" s="6"/>
-      <c r="D30" s="38"/>
+      <c r="D30" s="31"/>
       <c r="E30" s="6"/>
-      <c r="F30" s="38"/>
+      <c r="F30" s="31"/>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A31" s="8">

</xml_diff>

<commit_message>
Update at 13:22 on 09/02/2020
</commit_message>
<xml_diff>
--- a/site_libs/records/fall 2020.xlsx
+++ b/site_libs/records/fall 2020.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Portfolio\site_libs\records\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C00CCAC3-EEF5-41ED-92FC-78DCE6F15CC8}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C8B1B8A-D56E-42F1-A823-104999045D89}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30" yWindow="0" windowWidth="20460" windowHeight="10920" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Schedule" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="235" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="230" uniqueCount="126">
   <si>
     <t>Monday</t>
   </si>
@@ -431,20 +431,26 @@
 Jack</t>
   </si>
   <si>
-    <t>8:00-9:00</t>
-  </si>
-  <si>
     <t>2:00-3:00</t>
   </si>
   <si>
-    <t>CSE 341 Web Backend 2 Birch Remote</t>
+    <t>DEVO</t>
+  </si>
+  <si>
+    <t>JA</t>
+  </si>
+  <si>
+    <t>15-20</t>
+  </si>
+  <si>
+    <t>Depart</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="17" x14ac:knownFonts="1">
+  <fonts count="20" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -536,6 +542,24 @@
       <sz val="8"/>
       <name val="Arial"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF0070C0"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FFC00000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -569,13 +593,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="19" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -641,40 +664,46 @@
     <xf numFmtId="0" fontId="13" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -893,828 +922,715 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:U37"/>
+  <dimension ref="A1:P59"/>
   <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="11.7109375" customWidth="1"/>
     <col min="2" max="2" width="11.140625" customWidth="1"/>
-    <col min="3" max="3" width="9.42578125" customWidth="1"/>
-    <col min="4" max="4" width="10.42578125" customWidth="1"/>
-    <col min="5" max="5" width="8.7109375" customWidth="1"/>
-    <col min="6" max="6" width="11.28515625" customWidth="1"/>
-    <col min="7" max="7" width="9.42578125" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" customWidth="1"/>
-    <col min="9" max="9" width="9.85546875" customWidth="1"/>
-    <col min="10" max="10" width="11.7109375" customWidth="1"/>
-    <col min="11" max="11" width="6.140625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="4" customWidth="1"/>
-    <col min="13" max="13" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="5.5703125" customWidth="1"/>
-    <col min="15" max="15" width="16.140625" customWidth="1"/>
-    <col min="16" max="17" width="7.7109375" customWidth="1"/>
-    <col min="18" max="18" width="5.5703125" customWidth="1"/>
-    <col min="19" max="19" width="11" customWidth="1"/>
-    <col min="20" max="20" width="9.85546875" customWidth="1"/>
-    <col min="21" max="21" width="5" customWidth="1"/>
+    <col min="3" max="3" width="10.42578125" customWidth="1"/>
+    <col min="4" max="4" width="11.28515625" customWidth="1"/>
+    <col min="5" max="5" width="10.140625" customWidth="1"/>
+    <col min="6" max="6" width="11.7109375" customWidth="1"/>
+    <col min="7" max="7" width="4" customWidth="1"/>
+    <col min="8" max="8" width="6.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="5.5703125" customWidth="1"/>
+    <col min="10" max="10" width="16.140625" customWidth="1"/>
+    <col min="11" max="12" width="7.7109375" customWidth="1"/>
+    <col min="13" max="13" width="5.5703125" customWidth="1"/>
+    <col min="14" max="14" width="11" customWidth="1"/>
+    <col min="15" max="15" width="9.85546875" customWidth="1"/>
+    <col min="16" max="16" width="4.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B1" s="30" t="s">
+    <row r="1" spans="1:16" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B1" s="28" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="31"/>
-      <c r="D1" s="30" t="s">
+      <c r="C1" s="28" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="31"/>
-      <c r="F1" s="30" t="s">
+      <c r="D1" s="28" t="s">
         <v>2</v>
       </c>
-      <c r="G1" s="31"/>
-      <c r="H1" s="30" t="s">
+      <c r="E1" s="28" t="s">
         <v>3</v>
       </c>
-      <c r="I1" s="31"/>
-      <c r="J1" s="30" t="s">
+      <c r="F1" s="28" t="s">
         <v>4</v>
       </c>
-      <c r="K1" s="31"/>
-      <c r="L1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="43" t="s">
+        <v>125</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>9</v>
+      </c>
       <c r="M1" s="2" t="s">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="N1" s="2" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="O1" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="P1" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:16" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A2" s="7">
+        <v>0.36458333333333298</v>
+      </c>
+      <c r="B2" s="28"/>
+      <c r="C2" s="28"/>
+      <c r="D2" s="28"/>
+      <c r="E2" s="28"/>
+      <c r="F2" s="28"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="I2" s="12" t="s">
+        <v>113</v>
+      </c>
+      <c r="J2" s="12" t="s">
+        <v>114</v>
+      </c>
+      <c r="K2" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="L2" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="M2" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="N2" s="12" t="s">
+        <v>115</v>
+      </c>
+      <c r="O2" s="12" t="s">
+        <v>116</v>
+      </c>
+      <c r="P2" s="12">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A3" s="7">
+        <v>0.375</v>
+      </c>
+      <c r="B3" s="28"/>
+      <c r="C3" s="28"/>
+      <c r="D3" s="28"/>
+      <c r="E3" s="28"/>
+      <c r="F3" s="28"/>
+      <c r="G3" s="3"/>
+      <c r="H3" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="I3" s="6">
+        <v>450</v>
+      </c>
+      <c r="J3" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="K3" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="L3" s="6">
+        <v>347</v>
+      </c>
+      <c r="M3" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="N3" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="O3" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="P3" s="12">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A4" s="7">
+        <v>0.38541666666666702</v>
+      </c>
+      <c r="B4" s="28"/>
+      <c r="C4" s="28"/>
+      <c r="D4" s="28"/>
+      <c r="E4" s="28"/>
+      <c r="F4" s="28"/>
+      <c r="G4" s="3"/>
+      <c r="H4" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="I4" s="6">
+        <v>325</v>
+      </c>
+      <c r="J4" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="K4" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="L4" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="M4" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="N4" s="6" t="s">
+        <v>121</v>
+      </c>
+      <c r="O4" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="P4" s="6">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A5" s="7">
+        <v>0.39583333333333331</v>
+      </c>
+      <c r="B5" s="3"/>
+      <c r="C5" s="3"/>
+      <c r="D5" s="3"/>
+      <c r="E5" s="3"/>
+      <c r="F5" s="3"/>
+      <c r="G5" s="3"/>
+      <c r="P5" s="6"/>
+    </row>
+    <row r="6" spans="1:16" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A6" s="7">
+        <v>0.40625</v>
+      </c>
+      <c r="B6" s="3"/>
+      <c r="C6" s="10"/>
+      <c r="D6" s="3"/>
+      <c r="E6" s="10"/>
+      <c r="F6" s="3"/>
+      <c r="G6" s="3"/>
+      <c r="P6">
+        <f>SUM(P2:P5)</f>
         <v>7</v>
       </c>
-      <c r="P1" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="Q1" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="R1" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="S1" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="T1" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="U1" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="2" spans="1:21" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A2" s="3">
-        <v>0.32291666666666669</v>
-      </c>
-      <c r="B2" s="4"/>
-      <c r="C2" s="25"/>
-      <c r="D2" s="6"/>
-      <c r="E2" s="6"/>
-      <c r="F2" s="6"/>
-      <c r="G2" s="6"/>
-      <c r="H2" s="6"/>
-      <c r="I2" s="4"/>
-      <c r="J2" s="4"/>
-      <c r="K2" s="4"/>
-      <c r="L2" s="4"/>
-      <c r="M2" s="13" t="s">
-        <v>14</v>
-      </c>
-      <c r="N2" s="13" t="s">
-        <v>113</v>
-      </c>
-      <c r="O2" s="13" t="s">
-        <v>114</v>
-      </c>
-      <c r="P2" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="Q2" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="R2" s="13" t="s">
-        <v>26</v>
-      </c>
-      <c r="S2" s="13" t="s">
-        <v>115</v>
-      </c>
-      <c r="T2" s="13" t="s">
-        <v>116</v>
-      </c>
-      <c r="U2" s="13">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:21" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A3" s="8">
-        <v>0.33333333333333331</v>
-      </c>
-      <c r="B3" s="4"/>
-      <c r="C3" s="25"/>
-      <c r="D3" s="32" t="s">
-        <v>123</v>
-      </c>
-      <c r="E3" s="40"/>
-      <c r="F3" s="40"/>
-      <c r="G3" s="40"/>
-      <c r="H3" s="32" t="s">
-        <v>123</v>
-      </c>
-      <c r="I3" s="4"/>
-      <c r="J3" s="4"/>
-      <c r="K3" s="4"/>
-      <c r="L3" s="4"/>
-      <c r="M3" t="s">
-        <v>14</v>
-      </c>
-      <c r="N3">
-        <v>341</v>
-      </c>
-      <c r="O3" t="s">
-        <v>40</v>
-      </c>
-      <c r="P3" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="Q3" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="R3" s="13" t="s">
-        <v>26</v>
-      </c>
-      <c r="S3" s="13" t="s">
-        <v>121</v>
-      </c>
-      <c r="T3" s="13" t="s">
-        <v>42</v>
-      </c>
-      <c r="U3" s="13">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="4" spans="1:21" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A4" s="8">
-        <v>0.34375</v>
-      </c>
-      <c r="B4" s="4"/>
-      <c r="C4" s="25"/>
-      <c r="D4" s="32"/>
-      <c r="E4" s="40"/>
-      <c r="F4" s="40"/>
-      <c r="G4" s="40"/>
-      <c r="H4" s="32"/>
-      <c r="I4" s="4"/>
-      <c r="J4" s="4"/>
-      <c r="K4" s="4"/>
-      <c r="L4" s="4"/>
-      <c r="M4" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="N4" s="7">
-        <v>450</v>
-      </c>
-      <c r="O4" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="P4" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="Q4" s="7">
-        <v>347</v>
-      </c>
-      <c r="R4" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="S4" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="T4" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="U4" s="7">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="5" spans="1:21" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A5" s="8">
-        <v>0.35416666666666669</v>
-      </c>
-      <c r="B5" s="4"/>
-      <c r="C5" s="25"/>
-      <c r="D5" s="32"/>
-      <c r="E5" s="40"/>
-      <c r="F5" s="40"/>
-      <c r="G5" s="40"/>
-      <c r="H5" s="32"/>
-      <c r="I5" s="4"/>
-      <c r="J5" s="4"/>
-      <c r="K5" s="4"/>
-      <c r="L5" s="4"/>
-      <c r="M5" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="N5" s="7">
-        <v>325</v>
-      </c>
-      <c r="O5" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="P5" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="Q5" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="R5" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="S5" s="7" t="s">
-        <v>122</v>
-      </c>
-      <c r="T5" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="U5" s="7">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="6" spans="1:21" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A6" s="8">
-        <v>0.36458333333333331</v>
-      </c>
-      <c r="B6" s="4"/>
-      <c r="C6" s="25"/>
-      <c r="D6" s="32"/>
-      <c r="E6" s="40"/>
-      <c r="F6" s="40"/>
-      <c r="G6" s="40"/>
-      <c r="H6" s="32"/>
-      <c r="I6" s="4"/>
-      <c r="J6" s="4"/>
-      <c r="K6" s="4"/>
-      <c r="L6" s="4"/>
-      <c r="U6">
-        <f>SUM(U2:U5)</f>
-        <v>10</v>
-      </c>
-    </row>
-    <row r="7" spans="1:21" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A7" s="8">
-        <v>0.375</v>
-      </c>
-      <c r="B7" s="4"/>
-      <c r="C7" s="25"/>
-      <c r="D7" s="32"/>
-      <c r="E7" s="40"/>
-      <c r="F7" s="40"/>
-      <c r="G7" s="40"/>
-      <c r="H7" s="32"/>
-      <c r="I7" s="4"/>
-      <c r="J7" s="4"/>
-      <c r="K7" s="4"/>
-      <c r="L7" s="4"/>
-    </row>
-    <row r="8" spans="1:21" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A8" s="8">
-        <v>0.38541666666666669</v>
-      </c>
-      <c r="B8" s="4"/>
-      <c r="C8" s="25"/>
-      <c r="D8" s="32"/>
-      <c r="E8" s="40"/>
-      <c r="F8" s="40"/>
-      <c r="G8" s="40"/>
-      <c r="H8" s="32"/>
-      <c r="I8" s="4"/>
-      <c r="J8" s="4"/>
-      <c r="K8" s="4"/>
-      <c r="L8" s="4"/>
-    </row>
-    <row r="9" spans="1:21" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A9" s="8">
-        <v>0.39583333333333331</v>
-      </c>
-      <c r="B9" s="4"/>
-      <c r="C9" s="25"/>
-      <c r="D9" s="4"/>
-      <c r="E9" s="4"/>
-      <c r="F9" s="4"/>
-      <c r="G9" s="4"/>
-      <c r="H9" s="4"/>
-      <c r="I9" s="4"/>
-      <c r="J9" s="4"/>
-      <c r="K9" s="4"/>
-      <c r="L9" s="4"/>
-      <c r="M9" s="9"/>
-    </row>
-    <row r="10" spans="1:21" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A10" s="8">
-        <v>0.40625</v>
-      </c>
-      <c r="B10" s="4"/>
-      <c r="C10" s="25"/>
-      <c r="D10" s="11"/>
-      <c r="E10" s="4"/>
-      <c r="F10" s="4"/>
-      <c r="G10" s="4"/>
-      <c r="H10" s="11"/>
-      <c r="I10" s="4"/>
-      <c r="J10" s="4"/>
-      <c r="K10" s="4"/>
-      <c r="L10" s="4"/>
-      <c r="M10" s="10" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="11" spans="1:21" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A11" s="8">
+    </row>
+    <row r="7" spans="1:16" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A7" s="7">
         <v>0.41666666666666669</v>
       </c>
-      <c r="B11" s="4"/>
-      <c r="C11" s="25"/>
-      <c r="D11" s="11"/>
-      <c r="E11" s="4"/>
-      <c r="F11" s="4"/>
-      <c r="G11" s="4"/>
-      <c r="H11" s="11"/>
-      <c r="I11" s="4"/>
-      <c r="J11" s="4"/>
-      <c r="K11" s="4"/>
-      <c r="L11" s="4"/>
-    </row>
-    <row r="12" spans="1:21" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A12" s="8">
+      <c r="B7" s="3"/>
+      <c r="C7" s="10"/>
+      <c r="D7" s="3"/>
+      <c r="E7" s="10"/>
+      <c r="F7" s="3"/>
+      <c r="G7" s="3"/>
+    </row>
+    <row r="8" spans="1:16" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A8" s="7">
         <v>0.42708333333333331</v>
       </c>
-      <c r="B12" s="4"/>
-      <c r="C12" s="35" t="s">
+      <c r="B8" s="32" t="s">
         <v>29</v>
       </c>
-      <c r="D12" s="37" t="s">
+      <c r="C8" s="36" t="s">
         <v>118</v>
       </c>
-      <c r="E12" s="4"/>
-      <c r="F12" s="4"/>
-      <c r="G12" s="35" t="s">
+      <c r="D8" s="32" t="s">
         <v>30</v>
       </c>
-      <c r="H12" s="37" t="str">
-        <f>D12</f>
+      <c r="E8" s="36" t="str">
+        <f>C8</f>
         <v>CSE 121b 
 JavaScript 
 Barney 
 Remote</v>
       </c>
-      <c r="I12" s="4"/>
-      <c r="J12" s="4"/>
-      <c r="K12" s="36" t="s">
+      <c r="F8" s="35" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="13" spans="1:21" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A13" s="8">
+      <c r="G8" s="3"/>
+      <c r="H8" s="8"/>
+    </row>
+    <row r="9" spans="1:16" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A9" s="7">
         <v>0.4375</v>
       </c>
-      <c r="B13" s="4"/>
-      <c r="C13" s="33"/>
-      <c r="D13" s="37"/>
-      <c r="E13" s="4"/>
-      <c r="F13" s="4"/>
-      <c r="G13" s="33"/>
-      <c r="H13" s="37"/>
-      <c r="I13" s="4"/>
-      <c r="J13" s="4"/>
-      <c r="K13" s="36"/>
-    </row>
-    <row r="14" spans="1:21" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A14" s="8">
+      <c r="B9" s="33"/>
+      <c r="C9" s="36"/>
+      <c r="D9" s="33"/>
+      <c r="E9" s="36"/>
+      <c r="F9" s="35"/>
+      <c r="G9" s="3"/>
+      <c r="H9" s="41" t="s">
+        <v>28</v>
+      </c>
+      <c r="I9" s="41">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="10" spans="1:16" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A10" s="7">
         <v>0.44791666666666669</v>
       </c>
-      <c r="B14" s="4"/>
-      <c r="C14" s="33"/>
-      <c r="D14" s="37"/>
-      <c r="E14" s="4"/>
-      <c r="F14" s="4"/>
-      <c r="G14" s="33"/>
-      <c r="H14" s="37"/>
-      <c r="I14" s="4"/>
-      <c r="J14" s="4"/>
-      <c r="K14" s="36"/>
-    </row>
-    <row r="15" spans="1:21" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A15" s="8">
+      <c r="B10" s="33"/>
+      <c r="C10" s="36"/>
+      <c r="D10" s="33"/>
+      <c r="E10" s="36"/>
+      <c r="F10" s="35"/>
+      <c r="G10" s="3"/>
+      <c r="H10" s="42" t="s">
+        <v>123</v>
+      </c>
+      <c r="I10" s="42" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="11" spans="1:16" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A11" s="7">
         <v>0.45833333333333331</v>
       </c>
-      <c r="B15" s="4"/>
-      <c r="C15" s="33"/>
-      <c r="D15" s="37"/>
-      <c r="E15" s="4"/>
-      <c r="F15" s="4"/>
-      <c r="G15" s="33"/>
-      <c r="H15" s="37"/>
-      <c r="I15" s="4"/>
-      <c r="J15" s="4"/>
-      <c r="K15" s="36"/>
-    </row>
-    <row r="16" spans="1:21" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A16" s="8">
+      <c r="B11" s="33"/>
+      <c r="C11" s="36"/>
+      <c r="D11" s="33"/>
+      <c r="E11" s="36"/>
+      <c r="F11" s="35"/>
+      <c r="G11" s="3"/>
+    </row>
+    <row r="12" spans="1:16" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A12" s="7">
         <v>0.46875</v>
       </c>
-      <c r="B16" s="4"/>
-      <c r="C16" s="25"/>
-      <c r="D16" s="4"/>
-      <c r="E16" s="4"/>
-      <c r="F16" s="4"/>
-      <c r="G16" s="4"/>
-      <c r="H16" s="4"/>
-      <c r="I16" s="4"/>
-      <c r="J16" s="4"/>
-      <c r="K16" s="29"/>
-    </row>
-    <row r="17" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A17" s="8">
+      <c r="B12" s="3"/>
+      <c r="C12" s="3"/>
+      <c r="D12" s="3"/>
+      <c r="E12" s="3"/>
+      <c r="F12" s="3"/>
+    </row>
+    <row r="13" spans="1:16" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A13" s="7">
         <v>0.47916666666666669</v>
       </c>
-      <c r="B17" s="32" t="s">
+      <c r="B13" s="37" t="s">
         <v>31</v>
       </c>
-      <c r="C17" s="25"/>
-      <c r="D17" s="12"/>
-      <c r="E17" s="12"/>
-      <c r="F17" s="34" t="str">
-        <f>B17</f>
+      <c r="C13" s="34" t="s">
+        <v>122</v>
+      </c>
+      <c r="D13" s="38" t="str">
+        <f>B13</f>
         <v>CSE 450
 Machine Learning
 Burton 
 STC  394</v>
       </c>
-      <c r="G17" s="12"/>
-      <c r="H17" s="12"/>
-      <c r="I17" s="12"/>
-      <c r="J17" s="34" t="str">
-        <f>F17</f>
+      <c r="E13" s="34" t="s">
+        <v>122</v>
+      </c>
+      <c r="F13" s="38" t="str">
+        <f>D13</f>
         <v>CSE 450
 Machine Learning
 Burton 
 STC  394</v>
       </c>
-      <c r="K17" s="25"/>
-    </row>
-    <row r="18" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A18" s="8">
+    </row>
+    <row r="14" spans="1:16" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A14" s="7">
         <v>0.48958333333333331</v>
       </c>
-      <c r="B18" s="33"/>
-      <c r="C18" s="25"/>
-      <c r="D18" s="12"/>
-      <c r="E18" s="12"/>
-      <c r="F18" s="33"/>
-      <c r="G18" s="12"/>
-      <c r="H18" s="12"/>
-      <c r="I18" s="12"/>
-      <c r="J18" s="33"/>
-      <c r="K18" s="25"/>
-    </row>
-    <row r="19" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A19" s="8">
+      <c r="B14" s="33"/>
+      <c r="C14" s="34"/>
+      <c r="D14" s="33"/>
+      <c r="E14" s="34"/>
+      <c r="F14" s="33"/>
+    </row>
+    <row r="15" spans="1:16" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A15" s="7">
         <v>0.5</v>
       </c>
+      <c r="B15" s="33"/>
+      <c r="C15" s="34"/>
+      <c r="D15" s="33"/>
+      <c r="E15" s="34"/>
+      <c r="F15" s="33"/>
+    </row>
+    <row r="16" spans="1:16" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A16" s="7">
+        <v>0.51041666666666663</v>
+      </c>
+      <c r="B16" s="33"/>
+      <c r="C16" s="34"/>
+      <c r="D16" s="33"/>
+      <c r="E16" s="34"/>
+      <c r="F16" s="33"/>
+    </row>
+    <row r="17" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A17" s="7">
+        <v>0.52083333333333337</v>
+      </c>
+      <c r="B17" s="3"/>
+      <c r="C17" s="3"/>
+      <c r="D17" s="3"/>
+      <c r="E17" s="3"/>
+      <c r="F17" s="3"/>
+    </row>
+    <row r="18" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A18" s="7">
+        <v>0.53125</v>
+      </c>
+      <c r="B18" s="32" t="s">
+        <v>117</v>
+      </c>
+      <c r="C18" s="32" t="s">
+        <v>29</v>
+      </c>
+      <c r="D18" s="32" t="s">
+        <v>117</v>
+      </c>
+      <c r="E18" s="32" t="s">
+        <v>30</v>
+      </c>
+      <c r="F18" s="35" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A19" s="7">
+        <v>0.54166666666666663</v>
+      </c>
       <c r="B19" s="33"/>
-      <c r="C19" s="25"/>
-      <c r="D19" s="12"/>
-      <c r="E19" s="12"/>
-      <c r="F19" s="33"/>
-      <c r="G19" s="12"/>
-      <c r="H19" s="12"/>
-      <c r="I19" s="12"/>
-      <c r="J19" s="33"/>
-      <c r="K19" s="25"/>
-    </row>
-    <row r="20" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A20" s="8">
-        <v>0.51041666666666663</v>
+      <c r="C19" s="33"/>
+      <c r="D19" s="33"/>
+      <c r="E19" s="33"/>
+      <c r="F19" s="35"/>
+    </row>
+    <row r="20" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A20" s="7">
+        <v>0.55208333333333337</v>
       </c>
       <c r="B20" s="33"/>
-      <c r="C20" s="25"/>
-      <c r="D20" s="4"/>
-      <c r="E20" s="4"/>
-      <c r="F20" s="33"/>
-      <c r="G20" s="4"/>
-      <c r="H20" s="4"/>
-      <c r="I20" s="4"/>
-      <c r="J20" s="33"/>
-      <c r="K20" s="25"/>
-    </row>
-    <row r="21" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A21" s="8">
-        <v>0.52083333333333337</v>
-      </c>
-      <c r="B21" s="4"/>
-      <c r="C21" s="25"/>
-      <c r="D21" s="4"/>
-      <c r="E21" s="4"/>
-      <c r="F21" s="4"/>
-      <c r="G21" s="4"/>
-      <c r="H21" s="4"/>
-      <c r="I21" s="4"/>
-      <c r="J21" s="4"/>
-      <c r="K21" s="25"/>
-    </row>
-    <row r="22" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A22" s="8">
-        <v>0.53125</v>
-      </c>
-      <c r="C22" s="35" t="s">
-        <v>117</v>
-      </c>
-      <c r="D22" s="4"/>
-      <c r="E22" s="35" t="s">
-        <v>29</v>
-      </c>
-      <c r="F22" s="4"/>
-      <c r="G22" s="35" t="s">
-        <v>117</v>
-      </c>
-      <c r="H22" s="4"/>
-      <c r="I22" s="35" t="s">
-        <v>30</v>
-      </c>
-      <c r="J22" s="4"/>
-      <c r="K22" s="36" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="23" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A23" s="8">
-        <v>0.54166666666666663</v>
-      </c>
-      <c r="C23" s="33"/>
-      <c r="D23" s="4"/>
-      <c r="E23" s="33"/>
-      <c r="F23" s="4"/>
-      <c r="G23" s="33"/>
-      <c r="H23" s="4"/>
-      <c r="I23" s="33"/>
-      <c r="J23" s="4"/>
-      <c r="K23" s="36"/>
-    </row>
-    <row r="24" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A24" s="8">
-        <v>0.55208333333333337</v>
-      </c>
-      <c r="C24" s="33"/>
-      <c r="D24" s="4"/>
-      <c r="E24" s="33"/>
-      <c r="F24" s="4"/>
-      <c r="G24" s="33"/>
-      <c r="H24" s="4"/>
-      <c r="I24" s="33"/>
-      <c r="J24" s="4"/>
-      <c r="K24" s="36"/>
-    </row>
-    <row r="25" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A25" s="8">
+      <c r="C20" s="33"/>
+      <c r="D20" s="33"/>
+      <c r="E20" s="33"/>
+      <c r="F20" s="35"/>
+    </row>
+    <row r="21" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A21" s="7">
         <v>0.5625</v>
       </c>
-      <c r="C25" s="33"/>
-      <c r="D25" s="4"/>
-      <c r="E25" s="33"/>
-      <c r="F25" s="4"/>
-      <c r="G25" s="33"/>
-      <c r="H25" s="4"/>
-      <c r="I25" s="33"/>
-      <c r="J25" s="4"/>
-      <c r="K25" s="36"/>
-    </row>
-    <row r="26" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A26" s="8">
+      <c r="B21" s="33"/>
+      <c r="C21" s="33"/>
+      <c r="D21" s="33"/>
+      <c r="E21" s="33"/>
+      <c r="F21" s="35"/>
+    </row>
+    <row r="22" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A22" s="7">
         <v>0.57291666666666663</v>
       </c>
-      <c r="B26" s="25"/>
-      <c r="C26" s="25"/>
-      <c r="D26" s="25"/>
-      <c r="E26" s="25"/>
-      <c r="F26" s="25"/>
-      <c r="G26" s="25"/>
-      <c r="H26" s="25"/>
-      <c r="I26" s="25"/>
-      <c r="J26" s="25"/>
-      <c r="K26" s="25"/>
-    </row>
-    <row r="27" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A27" s="8">
+      <c r="B22" s="24"/>
+      <c r="C22" s="29"/>
+      <c r="D22" s="24"/>
+      <c r="E22" s="29"/>
+      <c r="F22" s="24"/>
+    </row>
+    <row r="23" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A23" s="7">
         <v>0.58333333333333337</v>
       </c>
-      <c r="B27" s="30" t="s">
+      <c r="B23" s="30" t="s">
         <v>32</v>
       </c>
-      <c r="C27" s="25"/>
-      <c r="D27" s="4"/>
-      <c r="E27" s="35" t="s">
+      <c r="C23" s="32" t="s">
         <v>33</v>
       </c>
-      <c r="F27" s="30" t="str">
-        <f>B27</f>
+      <c r="D23" s="30" t="str">
+        <f>B23</f>
         <v>MATH 325
 Intermediate Stats 
 Saunders 
 Remote</v>
       </c>
-      <c r="G27" s="25"/>
-      <c r="H27" s="4"/>
-      <c r="I27" s="35" t="s">
+      <c r="E23" s="32" t="s">
         <v>33</v>
       </c>
-      <c r="J27" s="30" t="str">
-        <f>F27</f>
+      <c r="F23" s="30" t="str">
+        <f>D23</f>
         <v>MATH 325
 Intermediate Stats 
 Saunders 
 Remote</v>
       </c>
-      <c r="K27" s="25"/>
-    </row>
-    <row r="28" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A28" s="8">
+    </row>
+    <row r="24" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A24" s="7">
         <v>0.59375</v>
       </c>
-      <c r="B28" s="33"/>
-      <c r="C28" s="25"/>
-      <c r="D28" s="4"/>
-      <c r="E28" s="33"/>
-      <c r="F28" s="33"/>
-      <c r="G28" s="25"/>
-      <c r="H28" s="4"/>
-      <c r="I28" s="33"/>
-      <c r="J28" s="33"/>
-      <c r="K28" s="25"/>
-    </row>
-    <row r="29" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A29" s="8">
+      <c r="B24" s="33"/>
+      <c r="C24" s="33"/>
+      <c r="D24" s="33"/>
+      <c r="E24" s="33"/>
+      <c r="F24" s="33"/>
+    </row>
+    <row r="25" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A25" s="7">
         <v>0.60416666666666663</v>
       </c>
-      <c r="B29" s="33"/>
-      <c r="C29" s="25"/>
-      <c r="D29" s="4"/>
-      <c r="E29" s="33"/>
-      <c r="F29" s="33"/>
-      <c r="G29" s="25"/>
-      <c r="H29" s="4"/>
-      <c r="I29" s="33"/>
-      <c r="J29" s="33"/>
-      <c r="K29" s="25"/>
-    </row>
-    <row r="30" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A30" s="8">
+      <c r="B25" s="33"/>
+      <c r="C25" s="33"/>
+      <c r="D25" s="33"/>
+      <c r="E25" s="33"/>
+      <c r="F25" s="33"/>
+    </row>
+    <row r="26" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A26" s="7">
         <v>0.61458333333333337</v>
       </c>
-      <c r="B30" s="33"/>
-      <c r="C30" s="25"/>
-      <c r="D30" s="4"/>
-      <c r="E30" s="33"/>
-      <c r="F30" s="33"/>
-      <c r="G30" s="25"/>
-      <c r="H30" s="4"/>
-      <c r="I30" s="33"/>
-      <c r="J30" s="33"/>
-      <c r="K30" s="25"/>
-    </row>
-    <row r="31" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A31" s="8">
+      <c r="B26" s="33"/>
+      <c r="C26" s="33"/>
+      <c r="D26" s="33"/>
+      <c r="E26" s="33"/>
+      <c r="F26" s="33"/>
+    </row>
+    <row r="27" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A27" s="7">
         <v>0.625</v>
       </c>
-      <c r="B31" s="4"/>
-      <c r="C31" s="25"/>
-      <c r="D31" s="4"/>
-      <c r="E31" s="4"/>
-      <c r="F31" s="4" t="s">
+      <c r="B27" s="3"/>
+      <c r="C27" s="3"/>
+      <c r="D27" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="G31" s="25"/>
-      <c r="H31" s="4"/>
-      <c r="I31" s="4"/>
-      <c r="J31" s="4"/>
-      <c r="K31" s="25"/>
-    </row>
-    <row r="32" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A32" s="8">
+      <c r="E27" s="3"/>
+      <c r="F27" s="3"/>
+    </row>
+    <row r="28" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A28" s="7">
         <v>0.63541666666666663</v>
       </c>
-      <c r="B32" s="6"/>
-      <c r="C32" s="36" t="s">
+      <c r="B28" s="35" t="s">
         <v>119</v>
       </c>
-      <c r="D32" s="6"/>
-      <c r="E32" s="6"/>
-      <c r="F32" s="6"/>
-      <c r="G32" s="36" t="s">
+      <c r="C28" s="5"/>
+      <c r="D28" s="35" t="s">
         <v>119</v>
       </c>
-      <c r="H32" s="6"/>
-      <c r="I32" s="6"/>
-      <c r="J32" s="6"/>
-      <c r="K32" s="25"/>
-    </row>
-    <row r="33" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A33" s="8">
+      <c r="E28" s="5"/>
+      <c r="F28" s="5"/>
+    </row>
+    <row r="29" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A29" s="7">
         <v>0.64583333333333337</v>
       </c>
-      <c r="B33" s="6"/>
-      <c r="C33" s="35"/>
-      <c r="D33" s="6"/>
-      <c r="E33" s="6"/>
-      <c r="F33" s="6"/>
-      <c r="G33" s="35"/>
-      <c r="H33" s="6"/>
-      <c r="I33" s="6"/>
-      <c r="J33" s="6"/>
-      <c r="K33" s="25"/>
-    </row>
-    <row r="34" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A34" s="8">
+      <c r="B29" s="32"/>
+      <c r="C29" s="5"/>
+      <c r="D29" s="32"/>
+      <c r="E29" s="5"/>
+      <c r="F29" s="5"/>
+    </row>
+    <row r="30" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A30" s="7">
         <v>0.65625</v>
       </c>
-      <c r="B34" s="6"/>
-      <c r="C34" s="35"/>
-      <c r="D34" s="6"/>
-      <c r="E34" s="6"/>
-      <c r="F34" s="6"/>
-      <c r="G34" s="35"/>
-      <c r="H34" s="6"/>
-      <c r="I34" s="6"/>
-      <c r="J34" s="6"/>
-      <c r="K34" s="25"/>
-    </row>
-    <row r="35" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A35" s="8">
+      <c r="B30" s="32"/>
+      <c r="C30" s="5"/>
+      <c r="D30" s="32"/>
+      <c r="E30" s="5"/>
+      <c r="F30" s="5"/>
+    </row>
+    <row r="31" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A31" s="7">
         <v>0.66666666666666663</v>
       </c>
-      <c r="B35" s="6"/>
-      <c r="C35" s="35"/>
-      <c r="D35" s="6"/>
-      <c r="E35" s="6"/>
-      <c r="F35" s="6"/>
-      <c r="G35" s="35"/>
-      <c r="H35" s="6"/>
-      <c r="I35" s="6"/>
-      <c r="J35" s="6"/>
-      <c r="K35" s="25"/>
-    </row>
-    <row r="36" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A36" s="8">
+      <c r="B31" s="32"/>
+      <c r="C31" s="5"/>
+      <c r="D31" s="32"/>
+      <c r="E31" s="5"/>
+      <c r="F31" s="5"/>
+    </row>
+    <row r="32" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A32" s="7">
         <v>0.67708333333333337</v>
       </c>
-      <c r="B36" s="4"/>
-      <c r="C36" s="35"/>
-      <c r="D36" s="4"/>
-      <c r="E36" s="4"/>
-      <c r="F36" s="4"/>
-      <c r="G36" s="35"/>
-      <c r="H36" s="4"/>
-      <c r="I36" s="4"/>
-      <c r="J36" s="4"/>
-      <c r="K36" s="25"/>
-    </row>
-    <row r="37" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A37" s="8">
+      <c r="B32" s="32"/>
+      <c r="C32" s="3"/>
+      <c r="D32" s="32"/>
+      <c r="E32" s="3"/>
+      <c r="F32" s="3"/>
+    </row>
+    <row r="33" spans="1:1" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A33" s="7">
         <v>0.6875</v>
       </c>
     </row>
+    <row r="34" spans="1:1" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A34" s="7">
+        <v>0.69791666666666696</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A35" s="7">
+        <v>0.70833333333333404</v>
+      </c>
+    </row>
+    <row r="36" spans="1:1" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A36" s="7">
+        <v>0.718750000000001</v>
+      </c>
+    </row>
+    <row r="37" spans="1:1" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A37" s="7">
+        <v>0.72916666666666696</v>
+      </c>
+    </row>
+    <row r="38" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A38" s="7">
+        <v>0.73958333333333404</v>
+      </c>
+    </row>
+    <row r="39" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A39" s="7">
+        <v>0.750000000000001</v>
+      </c>
+    </row>
+    <row r="40" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A40" s="7">
+        <v>0.76041666666666796</v>
+      </c>
+    </row>
+    <row r="41" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A41" s="7">
+        <v>0.77083333333333504</v>
+      </c>
+    </row>
+    <row r="42" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A42" s="7">
+        <v>0.781250000000001</v>
+      </c>
+    </row>
+    <row r="43" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A43" s="7">
+        <v>0.79166666666666796</v>
+      </c>
+    </row>
+    <row r="44" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A44" s="7">
+        <v>0.80208333333333504</v>
+      </c>
+    </row>
+    <row r="45" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A45" s="7">
+        <v>0.812500000000002</v>
+      </c>
+    </row>
+    <row r="46" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A46" s="7">
+        <v>0.82291666666666796</v>
+      </c>
+    </row>
+    <row r="47" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A47" s="7">
+        <v>0.83333333333333504</v>
+      </c>
+    </row>
+    <row r="48" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A48" s="7">
+        <v>0.843750000000002</v>
+      </c>
+    </row>
+    <row r="49" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A49" s="7">
+        <v>0.85416666666666896</v>
+      </c>
+    </row>
+    <row r="50" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A50" s="7">
+        <v>0.86458333333333504</v>
+      </c>
+    </row>
+    <row r="51" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A51" s="7">
+        <v>0.874999999999999</v>
+      </c>
+    </row>
+    <row r="52" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A52" s="7">
+        <v>0.88541666666666596</v>
+      </c>
+    </row>
+    <row r="53" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A53" s="7">
+        <v>0.89583333333333204</v>
+      </c>
+    </row>
+    <row r="54" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A54" s="7">
+        <v>0.906249999999999</v>
+      </c>
+    </row>
+    <row r="55" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A55" s="7">
+        <v>0.91666666666666596</v>
+      </c>
+    </row>
+    <row r="56" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A56" s="7">
+        <v>0.92708333333333204</v>
+      </c>
+    </row>
+    <row r="57" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A57" s="7">
+        <v>0.937499999999999</v>
+      </c>
+    </row>
+    <row r="58" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A58" s="7">
+        <v>0.94791666666666596</v>
+      </c>
+    </row>
+    <row r="59" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A59" s="7">
+        <v>0.95833333333333204</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="27">
-    <mergeCell ref="C32:C36"/>
-    <mergeCell ref="G32:G36"/>
-    <mergeCell ref="K12:K15"/>
-    <mergeCell ref="K22:K25"/>
-    <mergeCell ref="B27:B30"/>
-    <mergeCell ref="F27:F30"/>
-    <mergeCell ref="J27:J30"/>
-    <mergeCell ref="D12:D15"/>
-    <mergeCell ref="H12:H15"/>
-    <mergeCell ref="C12:C15"/>
-    <mergeCell ref="G12:G15"/>
-    <mergeCell ref="B17:B20"/>
-    <mergeCell ref="F17:F20"/>
-    <mergeCell ref="J17:J20"/>
-    <mergeCell ref="C22:C25"/>
-    <mergeCell ref="D3:D8"/>
-    <mergeCell ref="H3:H8"/>
-    <mergeCell ref="E22:E25"/>
-    <mergeCell ref="E27:E30"/>
-    <mergeCell ref="I22:I25"/>
-    <mergeCell ref="I27:I30"/>
-    <mergeCell ref="G22:G25"/>
-    <mergeCell ref="B1:C1"/>
-    <mergeCell ref="D1:E1"/>
-    <mergeCell ref="F1:G1"/>
-    <mergeCell ref="H1:I1"/>
-    <mergeCell ref="J1:K1"/>
+  <mergeCells count="22">
+    <mergeCell ref="B28:B32"/>
+    <mergeCell ref="C23:C26"/>
+    <mergeCell ref="D8:D11"/>
+    <mergeCell ref="D28:D32"/>
+    <mergeCell ref="E23:E26"/>
+    <mergeCell ref="B23:B26"/>
+    <mergeCell ref="D23:D26"/>
+    <mergeCell ref="F23:F26"/>
+    <mergeCell ref="C8:C11"/>
+    <mergeCell ref="E8:E11"/>
+    <mergeCell ref="B13:B16"/>
+    <mergeCell ref="D13:D16"/>
+    <mergeCell ref="F13:F16"/>
+    <mergeCell ref="C18:C21"/>
+    <mergeCell ref="B8:B11"/>
+    <mergeCell ref="B18:B21"/>
+    <mergeCell ref="F8:F11"/>
+    <mergeCell ref="F18:F21"/>
+    <mergeCell ref="C13:C16"/>
+    <mergeCell ref="E13:E16"/>
+    <mergeCell ref="D18:D21"/>
+    <mergeCell ref="E18:E21"/>
   </mergeCells>
   <phoneticPr fontId="16" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1800,27 +1716,27 @@
       </c>
     </row>
     <row r="2" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A2" s="8">
+      <c r="A2" s="7">
         <v>0.33333333333333331</v>
       </c>
-      <c r="B2" s="4"/>
-      <c r="D2" s="39" t="s">
+      <c r="B2" s="3"/>
+      <c r="D2" s="40" t="s">
         <v>35</v>
       </c>
-      <c r="E2" s="4"/>
-      <c r="F2" s="4"/>
-      <c r="G2" s="4"/>
-      <c r="H2" s="39" t="str">
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="40" t="str">
         <f>D2</f>
         <v>CSE 341
 Web Backend 2
 Birch 
 Remote</v>
       </c>
-      <c r="I2" s="4"/>
-      <c r="J2" s="4"/>
-      <c r="K2" s="4"/>
-      <c r="L2" s="4"/>
+      <c r="I2" s="3"/>
+      <c r="J2" s="3"/>
+      <c r="K2" s="3"/>
+      <c r="L2" s="3"/>
       <c r="M2" s="2" t="s">
         <v>14</v>
       </c>
@@ -1850,19 +1766,19 @@
       </c>
     </row>
     <row r="3" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A3" s="8">
+      <c r="A3" s="7">
         <v>0.34375</v>
       </c>
-      <c r="B3" s="4"/>
+      <c r="B3" s="3"/>
       <c r="D3" s="31"/>
-      <c r="E3" s="4"/>
-      <c r="F3" s="4"/>
-      <c r="G3" s="4"/>
+      <c r="E3" s="3"/>
+      <c r="F3" s="3"/>
+      <c r="G3" s="3"/>
       <c r="H3" s="31"/>
-      <c r="I3" s="4"/>
-      <c r="J3" s="4"/>
-      <c r="K3" s="4"/>
-      <c r="L3" s="4"/>
+      <c r="I3" s="3"/>
+      <c r="J3" s="3"/>
+      <c r="K3" s="3"/>
+      <c r="L3" s="3"/>
       <c r="M3" s="2" t="s">
         <v>20</v>
       </c>
@@ -1892,19 +1808,19 @@
       </c>
     </row>
     <row r="4" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A4" s="8">
+      <c r="A4" s="7">
         <v>0.35416666666666669</v>
       </c>
-      <c r="B4" s="4"/>
+      <c r="B4" s="3"/>
       <c r="D4" s="31"/>
-      <c r="E4" s="4"/>
-      <c r="F4" s="4"/>
-      <c r="G4" s="4"/>
+      <c r="E4" s="3"/>
+      <c r="F4" s="3"/>
+      <c r="G4" s="3"/>
       <c r="H4" s="31"/>
-      <c r="I4" s="4"/>
-      <c r="J4" s="4"/>
-      <c r="K4" s="4"/>
-      <c r="L4" s="4"/>
+      <c r="I4" s="3"/>
+      <c r="J4" s="3"/>
+      <c r="K4" s="3"/>
+      <c r="L4" s="3"/>
       <c r="M4" s="2" t="s">
         <v>36</v>
       </c>
@@ -1926,7 +1842,7 @@
       <c r="S4" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="T4" s="13" t="s">
+      <c r="T4" s="12" t="s">
         <v>39</v>
       </c>
       <c r="U4" s="2">
@@ -1934,19 +1850,19 @@
       </c>
     </row>
     <row r="5" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A5" s="8">
+      <c r="A5" s="7">
         <v>0.36458333333333331</v>
       </c>
-      <c r="B5" s="4"/>
+      <c r="B5" s="3"/>
       <c r="D5" s="31"/>
-      <c r="E5" s="4"/>
-      <c r="F5" s="4"/>
-      <c r="G5" s="4"/>
+      <c r="E5" s="3"/>
+      <c r="F5" s="3"/>
+      <c r="G5" s="3"/>
       <c r="H5" s="31"/>
-      <c r="I5" s="4"/>
-      <c r="J5" s="4"/>
-      <c r="K5" s="4"/>
-      <c r="L5" s="4"/>
+      <c r="I5" s="3"/>
+      <c r="J5" s="3"/>
+      <c r="K5" s="3"/>
+      <c r="L5" s="3"/>
       <c r="M5" s="2" t="s">
         <v>14</v>
       </c>
@@ -1968,7 +1884,7 @@
       <c r="S5" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="T5" s="13" t="s">
+      <c r="T5" s="12" t="s">
         <v>42</v>
       </c>
       <c r="U5" s="2">
@@ -1976,186 +1892,186 @@
       </c>
     </row>
     <row r="6" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A6" s="8">
+      <c r="A6" s="7">
         <v>0.375</v>
       </c>
-      <c r="B6" s="4"/>
+      <c r="B6" s="3"/>
       <c r="D6" s="31"/>
-      <c r="E6" s="4"/>
-      <c r="F6" s="4"/>
-      <c r="G6" s="4"/>
+      <c r="E6" s="3"/>
+      <c r="F6" s="3"/>
+      <c r="G6" s="3"/>
       <c r="H6" s="31"/>
-      <c r="I6" s="4"/>
-      <c r="J6" s="4"/>
-      <c r="K6" s="4"/>
-      <c r="L6" s="4"/>
+      <c r="I6" s="3"/>
+      <c r="J6" s="3"/>
+      <c r="K6" s="3"/>
+      <c r="L6" s="3"/>
     </row>
     <row r="7" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A7" s="8">
+      <c r="A7" s="7">
         <v>0.38541666666666669</v>
       </c>
-      <c r="B7" s="4"/>
+      <c r="B7" s="3"/>
       <c r="D7" s="31"/>
-      <c r="E7" s="4"/>
-      <c r="F7" s="4"/>
-      <c r="G7" s="4"/>
+      <c r="E7" s="3"/>
+      <c r="F7" s="3"/>
+      <c r="G7" s="3"/>
       <c r="H7" s="31"/>
-      <c r="I7" s="4"/>
-      <c r="J7" s="4"/>
-      <c r="K7" s="4"/>
-      <c r="L7" s="4"/>
-      <c r="M7" s="9" t="s">
+      <c r="I7" s="3"/>
+      <c r="J7" s="3"/>
+      <c r="K7" s="3"/>
+      <c r="L7" s="3"/>
+      <c r="M7" s="8" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="8" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A8" s="8">
+      <c r="A8" s="7">
         <v>0.39583333333333331</v>
       </c>
-      <c r="B8" s="4"/>
-      <c r="D8" s="4"/>
-      <c r="E8" s="4"/>
-      <c r="F8" s="4"/>
-      <c r="G8" s="4"/>
-      <c r="H8" s="4"/>
-      <c r="I8" s="4"/>
-      <c r="J8" s="4"/>
-      <c r="K8" s="4"/>
-      <c r="L8" s="4"/>
-      <c r="M8" s="10" t="s">
+      <c r="B8" s="3"/>
+      <c r="D8" s="3"/>
+      <c r="E8" s="3"/>
+      <c r="F8" s="3"/>
+      <c r="G8" s="3"/>
+      <c r="H8" s="3"/>
+      <c r="I8" s="3"/>
+      <c r="J8" s="3"/>
+      <c r="K8" s="3"/>
+      <c r="L8" s="3"/>
+      <c r="M8" s="9" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="9" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A9" s="8">
+      <c r="A9" s="7">
         <v>0.40625</v>
       </c>
-      <c r="B9" s="4"/>
-      <c r="D9" s="39" t="s">
+      <c r="B9" s="3"/>
+      <c r="D9" s="40" t="s">
         <v>43</v>
       </c>
-      <c r="E9" s="4"/>
-      <c r="F9" s="4"/>
-      <c r="G9" s="4"/>
-      <c r="H9" s="39" t="s">
+      <c r="E9" s="3"/>
+      <c r="F9" s="3"/>
+      <c r="G9" s="3"/>
+      <c r="H9" s="40" t="s">
         <v>43</v>
       </c>
-      <c r="I9" s="4"/>
-      <c r="J9" s="4"/>
-      <c r="K9" s="4"/>
-      <c r="L9" s="4"/>
+      <c r="I9" s="3"/>
+      <c r="J9" s="3"/>
+      <c r="K9" s="3"/>
+      <c r="L9" s="3"/>
     </row>
     <row r="10" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A10" s="8">
+      <c r="A10" s="7">
         <v>0.41666666666666669</v>
       </c>
-      <c r="B10" s="4"/>
+      <c r="B10" s="3"/>
       <c r="D10" s="31"/>
-      <c r="E10" s="4"/>
-      <c r="F10" s="4"/>
-      <c r="G10" s="4"/>
+      <c r="E10" s="3"/>
+      <c r="F10" s="3"/>
+      <c r="G10" s="3"/>
       <c r="H10" s="31"/>
-      <c r="I10" s="4"/>
-      <c r="J10" s="4"/>
-      <c r="K10" s="4"/>
-      <c r="L10" s="4"/>
+      <c r="I10" s="3"/>
+      <c r="J10" s="3"/>
+      <c r="K10" s="3"/>
+      <c r="L10" s="3"/>
     </row>
     <row r="11" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A11" s="8">
+      <c r="A11" s="7">
         <v>0.42708333333333331</v>
       </c>
       <c r="B11" s="1"/>
-      <c r="C11" s="38" t="s">
+      <c r="C11" s="39" t="s">
         <v>29</v>
       </c>
       <c r="D11" s="31"/>
-      <c r="E11" s="4"/>
+      <c r="E11" s="3"/>
       <c r="F11" s="1">
         <f>B11</f>
         <v>0</v>
       </c>
-      <c r="G11" s="38" t="s">
+      <c r="G11" s="39" t="s">
         <v>30</v>
       </c>
       <c r="H11" s="31"/>
-      <c r="I11" s="4"/>
+      <c r="I11" s="3"/>
       <c r="J11" s="1"/>
     </row>
     <row r="12" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A12" s="8">
+      <c r="A12" s="7">
         <v>0.4375</v>
       </c>
       <c r="B12" s="1"/>
       <c r="C12" s="31"/>
       <c r="D12" s="31"/>
-      <c r="E12" s="4"/>
+      <c r="E12" s="3"/>
       <c r="F12" s="1"/>
       <c r="G12" s="31"/>
       <c r="H12" s="31"/>
-      <c r="I12" s="4"/>
+      <c r="I12" s="3"/>
       <c r="J12" s="1"/>
     </row>
     <row r="13" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A13" s="8">
+      <c r="A13" s="7">
         <v>0.44791666666666669</v>
       </c>
       <c r="B13" s="1"/>
       <c r="C13" s="31"/>
       <c r="D13" s="31"/>
-      <c r="E13" s="4"/>
+      <c r="E13" s="3"/>
       <c r="F13" s="1"/>
       <c r="G13" s="31"/>
       <c r="H13" s="31"/>
-      <c r="I13" s="4"/>
+      <c r="I13" s="3"/>
       <c r="J13" s="1"/>
     </row>
     <row r="14" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A14" s="8">
+      <c r="A14" s="7">
         <v>0.45833333333333331</v>
       </c>
       <c r="B14" s="1"/>
       <c r="C14" s="31"/>
       <c r="D14" s="31"/>
-      <c r="E14" s="4"/>
+      <c r="E14" s="3"/>
       <c r="F14" s="1"/>
       <c r="G14" s="31"/>
       <c r="H14" s="31"/>
-      <c r="I14" s="4"/>
+      <c r="I14" s="3"/>
       <c r="J14" s="1"/>
     </row>
     <row r="15" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A15" s="8">
+      <c r="A15" s="7">
         <v>0.46875</v>
       </c>
-      <c r="B15" s="4"/>
-      <c r="D15" s="4"/>
-      <c r="E15" s="4"/>
-      <c r="F15" s="4"/>
-      <c r="G15" s="4"/>
-      <c r="H15" s="4"/>
-      <c r="I15" s="4"/>
-      <c r="J15" s="4"/>
+      <c r="B15" s="3"/>
+      <c r="D15" s="3"/>
+      <c r="E15" s="3"/>
+      <c r="F15" s="3"/>
+      <c r="G15" s="3"/>
+      <c r="H15" s="3"/>
+      <c r="I15" s="3"/>
+      <c r="J15" s="3"/>
     </row>
     <row r="16" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A16" s="8">
+      <c r="A16" s="7">
         <v>0.47916666666666669</v>
       </c>
-      <c r="B16" s="34" t="s">
+      <c r="B16" s="38" t="s">
         <v>31</v>
       </c>
-      <c r="D16" s="12"/>
-      <c r="E16" s="12"/>
-      <c r="F16" s="34" t="str">
+      <c r="D16" s="11"/>
+      <c r="E16" s="11"/>
+      <c r="F16" s="38" t="str">
         <f>B16</f>
         <v>CSE 450
 Machine Learning
 Burton 
 STC  394</v>
       </c>
-      <c r="G16" s="12"/>
-      <c r="H16" s="12"/>
-      <c r="I16" s="12"/>
-      <c r="J16" s="34" t="str">
+      <c r="G16" s="11"/>
+      <c r="H16" s="11"/>
+      <c r="I16" s="11"/>
+      <c r="J16" s="38" t="str">
         <f>F16</f>
         <v>CSE 450
 Machine Learning
@@ -2164,127 +2080,127 @@
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A17" s="8">
+      <c r="A17" s="7">
         <v>0.48958333333333331</v>
       </c>
       <c r="B17" s="31"/>
-      <c r="D17" s="12"/>
-      <c r="E17" s="12"/>
+      <c r="D17" s="11"/>
+      <c r="E17" s="11"/>
       <c r="F17" s="31"/>
-      <c r="G17" s="12"/>
-      <c r="H17" s="12"/>
-      <c r="I17" s="12"/>
+      <c r="G17" s="11"/>
+      <c r="H17" s="11"/>
+      <c r="I17" s="11"/>
       <c r="J17" s="31"/>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A18" s="8">
+      <c r="A18" s="7">
         <v>0.5</v>
       </c>
       <c r="B18" s="31"/>
-      <c r="D18" s="12"/>
-      <c r="E18" s="12"/>
+      <c r="D18" s="11"/>
+      <c r="E18" s="11"/>
       <c r="F18" s="31"/>
-      <c r="G18" s="12"/>
-      <c r="H18" s="12"/>
-      <c r="I18" s="12"/>
+      <c r="G18" s="11"/>
+      <c r="H18" s="11"/>
+      <c r="I18" s="11"/>
       <c r="J18" s="31"/>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A19" s="8">
+      <c r="A19" s="7">
         <v>0.51041666666666663</v>
       </c>
       <c r="B19" s="31"/>
-      <c r="D19" s="4"/>
-      <c r="E19" s="4"/>
+      <c r="D19" s="3"/>
+      <c r="E19" s="3"/>
       <c r="F19" s="31"/>
-      <c r="G19" s="4"/>
-      <c r="H19" s="4"/>
-      <c r="I19" s="4"/>
+      <c r="G19" s="3"/>
+      <c r="H19" s="3"/>
+      <c r="I19" s="3"/>
       <c r="J19" s="31"/>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A20" s="8">
+      <c r="A20" s="7">
         <v>0.52083333333333337</v>
       </c>
-      <c r="B20" s="4"/>
-      <c r="D20" s="4"/>
-      <c r="E20" s="4"/>
-      <c r="F20" s="4"/>
-      <c r="G20" s="4"/>
-      <c r="H20" s="4"/>
-      <c r="I20" s="4"/>
-      <c r="J20" s="4"/>
+      <c r="B20" s="3"/>
+      <c r="D20" s="3"/>
+      <c r="E20" s="3"/>
+      <c r="F20" s="3"/>
+      <c r="G20" s="3"/>
+      <c r="H20" s="3"/>
+      <c r="I20" s="3"/>
+      <c r="J20" s="3"/>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A21" s="8">
+      <c r="A21" s="7">
         <v>0.53125</v>
       </c>
-      <c r="B21" s="4"/>
-      <c r="D21" s="4"/>
-      <c r="E21" s="38" t="s">
+      <c r="B21" s="3"/>
+      <c r="D21" s="3"/>
+      <c r="E21" s="39" t="s">
         <v>29</v>
       </c>
-      <c r="F21" s="4"/>
-      <c r="G21" s="4"/>
-      <c r="H21" s="4"/>
-      <c r="I21" s="38" t="s">
+      <c r="F21" s="3"/>
+      <c r="G21" s="3"/>
+      <c r="H21" s="3"/>
+      <c r="I21" s="39" t="s">
         <v>30</v>
       </c>
-      <c r="J21" s="4"/>
+      <c r="J21" s="3"/>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A22" s="8">
+      <c r="A22" s="7">
         <v>0.54166666666666663</v>
       </c>
-      <c r="B22" s="4"/>
-      <c r="D22" s="4"/>
+      <c r="B22" s="3"/>
+      <c r="D22" s="3"/>
       <c r="E22" s="31"/>
-      <c r="F22" s="4"/>
-      <c r="G22" s="4"/>
-      <c r="H22" s="4"/>
+      <c r="F22" s="3"/>
+      <c r="G22" s="3"/>
+      <c r="H22" s="3"/>
       <c r="I22" s="31"/>
-      <c r="J22" s="4"/>
+      <c r="J22" s="3"/>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A23" s="8">
+      <c r="A23" s="7">
         <v>0.55208333333333337</v>
       </c>
-      <c r="B23" s="4"/>
-      <c r="D23" s="4"/>
+      <c r="B23" s="3"/>
+      <c r="D23" s="3"/>
       <c r="E23" s="31"/>
-      <c r="F23" s="4"/>
-      <c r="G23" s="4"/>
-      <c r="H23" s="4"/>
+      <c r="F23" s="3"/>
+      <c r="G23" s="3"/>
+      <c r="H23" s="3"/>
       <c r="I23" s="31"/>
-      <c r="J23" s="4"/>
+      <c r="J23" s="3"/>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A24" s="8">
+      <c r="A24" s="7">
         <v>0.5625</v>
       </c>
-      <c r="B24" s="4"/>
-      <c r="D24" s="4"/>
+      <c r="B24" s="3"/>
+      <c r="D24" s="3"/>
       <c r="E24" s="31"/>
-      <c r="F24" s="4"/>
-      <c r="G24" s="4"/>
-      <c r="H24" s="4"/>
+      <c r="F24" s="3"/>
+      <c r="G24" s="3"/>
+      <c r="H24" s="3"/>
       <c r="I24" s="31"/>
-      <c r="J24" s="4"/>
+      <c r="J24" s="3"/>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A25" s="8">
+      <c r="A25" s="7">
         <v>0.57291666666666663</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A26" s="8">
+      <c r="A26" s="7">
         <v>0.58333333333333337</v>
       </c>
       <c r="B26" s="30" t="s">
         <v>32</v>
       </c>
       <c r="D26" s="1"/>
-      <c r="E26" s="35" t="s">
+      <c r="E26" s="32" t="s">
         <v>33</v>
       </c>
       <c r="F26" s="30" t="str">
@@ -2295,7 +2211,7 @@
 Remote</v>
       </c>
       <c r="H26" s="1"/>
-      <c r="I26" s="35" t="s">
+      <c r="I26" s="32" t="s">
         <v>33</v>
       </c>
       <c r="J26" s="30" t="str">
@@ -2307,7 +2223,7 @@
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A27" s="8">
+      <c r="A27" s="7">
         <v>0.59375</v>
       </c>
       <c r="B27" s="31"/>
@@ -2319,7 +2235,7 @@
       <c r="J27" s="31"/>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A28" s="8">
+      <c r="A28" s="7">
         <v>0.60416666666666663</v>
       </c>
       <c r="B28" s="31"/>
@@ -2331,7 +2247,7 @@
       <c r="J28" s="31"/>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A29" s="8">
+      <c r="A29" s="7">
         <v>0.61458333333333337</v>
       </c>
       <c r="B29" s="31"/>
@@ -2343,88 +2259,88 @@
       <c r="J29" s="31"/>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A30" s="8">
+      <c r="A30" s="7">
         <v>0.625</v>
       </c>
-      <c r="B30" s="4"/>
-      <c r="D30" s="4"/>
-      <c r="E30" s="4"/>
+      <c r="B30" s="3"/>
+      <c r="D30" s="3"/>
+      <c r="E30" s="3"/>
       <c r="F30" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="H30" s="4"/>
-      <c r="I30" s="4"/>
-      <c r="J30" s="4"/>
+      <c r="H30" s="3"/>
+      <c r="I30" s="3"/>
+      <c r="J30" s="3"/>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A31" s="8">
+      <c r="A31" s="7">
         <v>0.63541666666666663</v>
       </c>
-      <c r="B31" s="5"/>
-      <c r="C31" s="5"/>
-      <c r="D31" s="5"/>
-      <c r="E31" s="5"/>
-      <c r="F31" s="5"/>
-      <c r="G31" s="5"/>
-      <c r="H31" s="5"/>
-      <c r="I31" s="5"/>
-      <c r="J31" s="5"/>
+      <c r="B31" s="4"/>
+      <c r="C31" s="4"/>
+      <c r="D31" s="4"/>
+      <c r="E31" s="4"/>
+      <c r="F31" s="4"/>
+      <c r="G31" s="4"/>
+      <c r="H31" s="4"/>
+      <c r="I31" s="4"/>
+      <c r="J31" s="4"/>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A32" s="8">
+      <c r="A32" s="7">
         <v>0.64583333333333337</v>
       </c>
-      <c r="B32" s="5"/>
-      <c r="C32" s="5"/>
-      <c r="D32" s="5"/>
-      <c r="E32" s="5"/>
-      <c r="F32" s="5"/>
-      <c r="G32" s="5"/>
-      <c r="H32" s="5"/>
-      <c r="I32" s="5"/>
-      <c r="J32" s="5"/>
+      <c r="B32" s="4"/>
+      <c r="C32" s="4"/>
+      <c r="D32" s="4"/>
+      <c r="E32" s="4"/>
+      <c r="F32" s="4"/>
+      <c r="G32" s="4"/>
+      <c r="H32" s="4"/>
+      <c r="I32" s="4"/>
+      <c r="J32" s="4"/>
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A33" s="8">
+      <c r="A33" s="7">
         <v>0.65625</v>
       </c>
-      <c r="B33" s="5"/>
-      <c r="C33" s="5"/>
-      <c r="D33" s="5"/>
-      <c r="E33" s="5"/>
-      <c r="F33" s="5"/>
-      <c r="G33" s="5"/>
-      <c r="H33" s="5"/>
-      <c r="I33" s="5"/>
-      <c r="J33" s="5"/>
+      <c r="B33" s="4"/>
+      <c r="C33" s="4"/>
+      <c r="D33" s="4"/>
+      <c r="E33" s="4"/>
+      <c r="F33" s="4"/>
+      <c r="G33" s="4"/>
+      <c r="H33" s="4"/>
+      <c r="I33" s="4"/>
+      <c r="J33" s="4"/>
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A34" s="8">
+      <c r="A34" s="7">
         <v>0.66666666666666663</v>
       </c>
-      <c r="B34" s="5"/>
-      <c r="C34" s="5"/>
-      <c r="D34" s="5"/>
-      <c r="E34" s="5"/>
-      <c r="F34" s="5"/>
-      <c r="G34" s="5"/>
-      <c r="H34" s="5"/>
-      <c r="I34" s="5"/>
-      <c r="J34" s="5"/>
+      <c r="B34" s="4"/>
+      <c r="C34" s="4"/>
+      <c r="D34" s="4"/>
+      <c r="E34" s="4"/>
+      <c r="F34" s="4"/>
+      <c r="G34" s="4"/>
+      <c r="H34" s="4"/>
+      <c r="I34" s="4"/>
+      <c r="J34" s="4"/>
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A35" s="8">
+      <c r="A35" s="7">
         <v>0.67708333333333337</v>
       </c>
-      <c r="B35" s="4"/>
-      <c r="C35" s="4"/>
-      <c r="D35" s="4"/>
-      <c r="E35" s="4"/>
-      <c r="F35" s="4"/>
-      <c r="G35" s="4"/>
-      <c r="H35" s="4"/>
-      <c r="I35" s="4"/>
-      <c r="J35" s="4"/>
+      <c r="B35" s="3"/>
+      <c r="C35" s="3"/>
+      <c r="D35" s="3"/>
+      <c r="E35" s="3"/>
+      <c r="F35" s="3"/>
+      <c r="G35" s="3"/>
+      <c r="H35" s="3"/>
+      <c r="I35" s="3"/>
+      <c r="J35" s="3"/>
     </row>
   </sheetData>
   <mergeCells count="21">
@@ -2462,209 +2378,210 @@
   <dimension ref="A1:F31"/>
   <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="32.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="34" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="2.28515625" customWidth="1"/>
-    <col min="4" max="4" width="25.140625" customWidth="1"/>
-    <col min="5" max="5" width="51.7109375" customWidth="1"/>
+    <col min="4" max="4" width="26.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="48.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="15" x14ac:dyDescent="0.2">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="13" t="s">
         <v>44</v>
       </c>
-      <c r="B1" s="15" t="s">
+      <c r="B1" s="14" t="s">
         <v>45</v>
       </c>
-      <c r="C1" s="15">
+      <c r="C1" s="14">
         <v>1</v>
       </c>
-      <c r="D1" s="15" t="s">
+      <c r="D1" s="14" t="s">
         <v>46</v>
       </c>
-      <c r="E1" s="16" t="s">
+      <c r="E1" s="15" t="s">
         <v>47</v>
       </c>
-      <c r="F1" s="15" t="s">
+      <c r="F1" s="14" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="15" x14ac:dyDescent="0.2">
-      <c r="A2" s="14" t="s">
+      <c r="A2" s="13" t="s">
         <v>49</v>
       </c>
-      <c r="B2" s="17" t="s">
+      <c r="B2" s="16" t="s">
         <v>45</v>
       </c>
-      <c r="C2" s="17">
+      <c r="C2" s="16">
         <v>1</v>
       </c>
-      <c r="D2" s="17" t="s">
+      <c r="D2" s="16" t="s">
         <v>46</v>
       </c>
-      <c r="E2" s="18" t="s">
+      <c r="E2" s="17" t="s">
         <v>50</v>
       </c>
-      <c r="F2" s="17" t="s">
+      <c r="F2" s="16" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="15" x14ac:dyDescent="0.2">
-      <c r="A3" s="19" t="s">
+      <c r="A3" s="18" t="s">
         <v>56</v>
       </c>
-      <c r="B3" s="18" t="s">
+      <c r="B3" s="17" t="s">
         <v>57</v>
       </c>
-      <c r="C3" s="17">
+      <c r="C3" s="16">
         <v>1</v>
       </c>
-      <c r="D3" s="17" t="s">
+      <c r="D3" s="16" t="s">
         <v>58</v>
       </c>
-      <c r="E3" s="18" t="s">
+      <c r="E3" s="17" t="s">
         <v>59</v>
       </c>
-      <c r="F3" s="18" t="s">
+      <c r="F3" s="17" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="15" x14ac:dyDescent="0.2">
-      <c r="A4" s="19" t="s">
+      <c r="A4" s="18" t="s">
         <v>61</v>
       </c>
-      <c r="B4" s="17" t="s">
+      <c r="B4" s="16" t="s">
         <v>62</v>
       </c>
-      <c r="C4" s="17">
+      <c r="C4" s="16">
         <v>1</v>
       </c>
-      <c r="D4" s="17" t="s">
+      <c r="D4" s="16" t="s">
         <v>58</v>
       </c>
-      <c r="E4" s="18" t="s">
+      <c r="E4" s="17" t="s">
         <v>63</v>
       </c>
-      <c r="F4" s="18" t="s">
+      <c r="F4" s="17" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="15" x14ac:dyDescent="0.2">
-      <c r="A5" s="14" t="s">
+      <c r="A5" s="13" t="s">
         <v>51</v>
       </c>
-      <c r="B5" s="15" t="s">
+      <c r="B5" s="14" t="s">
         <v>52</v>
       </c>
-      <c r="C5" s="15">
+      <c r="C5" s="14">
         <v>1</v>
       </c>
-      <c r="D5" s="15" t="s">
+      <c r="D5" s="14" t="s">
         <v>46</v>
       </c>
-      <c r="E5" s="16" t="s">
+      <c r="E5" s="15" t="s">
         <v>53</v>
       </c>
-      <c r="F5" s="15" t="s">
+      <c r="F5" s="14" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="15" x14ac:dyDescent="0.2">
-      <c r="A6" s="14" t="s">
+      <c r="A6" s="13" t="s">
         <v>54</v>
       </c>
-      <c r="B6" s="17" t="s">
+      <c r="B6" s="16" t="s">
         <v>52</v>
       </c>
-      <c r="C6" s="17">
+      <c r="C6" s="16">
         <v>1</v>
       </c>
-      <c r="D6" s="17" t="s">
+      <c r="D6" s="16" t="s">
         <v>46</v>
       </c>
-      <c r="E6" s="18" t="s">
+      <c r="E6" s="17" t="s">
         <v>55</v>
       </c>
-      <c r="F6" s="17" t="s">
+      <c r="F6" s="16" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="26" t="s">
+      <c r="A7" s="25" t="s">
         <v>87</v>
       </c>
-      <c r="B7" s="28" t="s">
+      <c r="B7" s="27" t="s">
         <v>88</v>
       </c>
-      <c r="C7" s="28">
+      <c r="C7" s="27">
         <v>1</v>
       </c>
-      <c r="D7" s="28" t="s">
+      <c r="D7" s="27" t="s">
         <v>83</v>
       </c>
-      <c r="E7" s="28" t="s">
+      <c r="E7" s="27" t="s">
         <v>89</v>
       </c>
-      <c r="F7" s="28" t="s">
+      <c r="F7" s="27" t="s">
         <v>90</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="26" t="s">
+      <c r="A8" s="25" t="s">
         <v>91</v>
       </c>
-      <c r="B8" s="27" t="s">
+      <c r="B8" s="26" t="s">
         <v>88</v>
       </c>
-      <c r="C8" s="27">
+      <c r="C8" s="26">
         <v>1</v>
       </c>
-      <c r="D8" s="27" t="s">
+      <c r="D8" s="26" t="s">
         <v>83</v>
       </c>
-      <c r="E8" s="27" t="s">
+      <c r="E8" s="26" t="s">
         <v>92</v>
       </c>
-      <c r="F8" s="27" t="s">
+      <c r="F8" s="26" t="s">
         <v>90</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="26" t="s">
+      <c r="A9" s="25" t="s">
         <v>93</v>
       </c>
-      <c r="B9" s="28" t="s">
+      <c r="B9" s="27" t="s">
         <v>94</v>
       </c>
-      <c r="C9" s="28">
+      <c r="C9" s="27">
         <v>3</v>
       </c>
-      <c r="D9" s="28" t="s">
+      <c r="D9" s="27" t="s">
         <v>83</v>
       </c>
-      <c r="E9" s="28" t="s">
+      <c r="E9" s="27" t="s">
         <v>95</v>
       </c>
-      <c r="F9" s="27" t="s">
+      <c r="F9" s="26" t="s">
         <v>96</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="15" x14ac:dyDescent="0.2">
-      <c r="A10" s="26" t="s">
+      <c r="A10" s="25" t="s">
         <v>98</v>
       </c>
-      <c r="B10" s="27" t="s">
+      <c r="B10" s="26" t="s">
         <v>99</v>
       </c>
-      <c r="C10" s="27">
+      <c r="C10" s="26">
         <v>3</v>
       </c>
-      <c r="D10" s="27" t="s">
+      <c r="D10" s="26" t="s">
         <v>46</v>
       </c>
-      <c r="E10" s="27" t="s">
+      <c r="E10" s="26" t="s">
         <v>100</v>
       </c>
-      <c r="F10" s="27" t="s">
+      <c r="F10" s="26" t="s">
         <v>74</v>
       </c>
     </row>
@@ -2679,222 +2596,222 @@
     <row r="19" spans="1:6" ht="12.75" x14ac:dyDescent="0.2"/>
     <row r="20" spans="1:6" ht="12.75" x14ac:dyDescent="0.2"/>
     <row r="21" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A21" s="20" t="s">
+      <c r="A21" s="19" t="s">
         <v>65</v>
       </c>
-      <c r="B21" s="21" t="s">
+      <c r="B21" s="20" t="s">
         <v>66</v>
       </c>
-      <c r="C21" s="21">
+      <c r="C21" s="20">
         <v>2</v>
       </c>
-      <c r="D21" s="21" t="s">
+      <c r="D21" s="20" t="s">
         <v>67</v>
       </c>
-      <c r="E21" s="22" t="s">
+      <c r="E21" s="21" t="s">
         <v>68</v>
       </c>
-      <c r="F21" s="21" t="s">
+      <c r="F21" s="20" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="22" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A22" s="20" t="s">
+      <c r="A22" s="19" t="s">
         <v>69</v>
       </c>
-      <c r="B22" s="23" t="s">
+      <c r="B22" s="22" t="s">
         <v>66</v>
       </c>
-      <c r="C22" s="23">
+      <c r="C22" s="22">
         <v>2</v>
       </c>
-      <c r="D22" s="23" t="s">
+      <c r="D22" s="22" t="s">
         <v>70</v>
       </c>
-      <c r="E22" s="24" t="s">
+      <c r="E22" s="23" t="s">
         <v>71</v>
       </c>
-      <c r="F22" s="23" t="s">
+      <c r="F22" s="22" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="23" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="20" t="s">
+      <c r="A23" s="19" t="s">
         <v>72</v>
       </c>
-      <c r="B23" s="21" t="s">
+      <c r="B23" s="20" t="s">
         <v>66</v>
       </c>
-      <c r="C23" s="21">
+      <c r="C23" s="20">
         <v>2</v>
       </c>
-      <c r="D23" s="21" t="s">
+      <c r="D23" s="20" t="s">
         <v>46</v>
       </c>
-      <c r="E23" s="22" t="s">
+      <c r="E23" s="21" t="s">
         <v>73</v>
       </c>
-      <c r="F23" s="22" t="s">
+      <c r="F23" s="21" t="s">
         <v>74</v>
       </c>
     </row>
     <row r="24" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="20" t="s">
+      <c r="A24" s="19" t="s">
         <v>75</v>
       </c>
-      <c r="B24" s="23" t="s">
+      <c r="B24" s="22" t="s">
         <v>66</v>
       </c>
-      <c r="C24" s="23">
+      <c r="C24" s="22">
         <v>2</v>
       </c>
-      <c r="D24" s="23" t="s">
+      <c r="D24" s="22" t="s">
         <v>76</v>
       </c>
-      <c r="E24" s="24" t="s">
+      <c r="E24" s="23" t="s">
         <v>77</v>
       </c>
-      <c r="F24" s="23" t="s">
+      <c r="F24" s="22" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="25" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="20" t="s">
+      <c r="A25" s="19" t="s">
         <v>78</v>
       </c>
-      <c r="B25" s="21" t="s">
+      <c r="B25" s="20" t="s">
         <v>66</v>
       </c>
-      <c r="C25" s="21">
+      <c r="C25" s="20">
         <v>2</v>
       </c>
-      <c r="D25" s="21" t="s">
+      <c r="D25" s="20" t="s">
         <v>79</v>
       </c>
-      <c r="E25" s="22" t="s">
+      <c r="E25" s="21" t="s">
         <v>80</v>
       </c>
-      <c r="F25" s="21" t="s">
+      <c r="F25" s="20" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="26" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="20" t="s">
+      <c r="A26" s="19" t="s">
         <v>81</v>
       </c>
-      <c r="B26" s="21" t="s">
+      <c r="B26" s="20" t="s">
         <v>82</v>
       </c>
-      <c r="C26" s="21">
+      <c r="C26" s="20">
         <v>3</v>
       </c>
-      <c r="D26" s="21" t="s">
+      <c r="D26" s="20" t="s">
         <v>83</v>
       </c>
-      <c r="E26" s="22" t="s">
+      <c r="E26" s="21" t="s">
         <v>84</v>
       </c>
-      <c r="F26" s="22" t="s">
+      <c r="F26" s="21" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="27" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="20" t="s">
+      <c r="A27" s="19" t="s">
         <v>85</v>
       </c>
-      <c r="B27" s="23" t="s">
+      <c r="B27" s="22" t="s">
         <v>82</v>
       </c>
-      <c r="C27" s="23">
+      <c r="C27" s="22">
         <v>3</v>
       </c>
-      <c r="D27" s="23" t="s">
+      <c r="D27" s="22" t="s">
         <v>76</v>
       </c>
-      <c r="E27" s="24" t="s">
+      <c r="E27" s="23" t="s">
         <v>86</v>
       </c>
-      <c r="F27" s="22" t="s">
+      <c r="F27" s="21" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="28" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="20" t="s">
+      <c r="A28" s="19" t="s">
         <v>97</v>
       </c>
-      <c r="B28" s="21" t="s">
+      <c r="B28" s="20" t="s">
         <v>94</v>
       </c>
-      <c r="C28" s="21">
+      <c r="C28" s="20">
         <v>3</v>
       </c>
-      <c r="D28" s="21" t="s">
+      <c r="D28" s="20" t="s">
         <v>83</v>
       </c>
-      <c r="E28" s="22" t="s">
+      <c r="E28" s="21" t="s">
         <v>86</v>
       </c>
-      <c r="F28" s="22" t="s">
+      <c r="F28" s="21" t="s">
         <v>96</v>
       </c>
     </row>
     <row r="29" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A29" s="20" t="s">
+      <c r="A29" s="19" t="s">
         <v>101</v>
       </c>
-      <c r="B29" s="23" t="s">
+      <c r="B29" s="22" t="s">
         <v>102</v>
       </c>
-      <c r="C29" s="23">
+      <c r="C29" s="22">
         <v>3</v>
       </c>
-      <c r="D29" s="23" t="s">
+      <c r="D29" s="22" t="s">
         <v>103</v>
       </c>
-      <c r="E29" s="24" t="s">
+      <c r="E29" s="23" t="s">
         <v>104</v>
       </c>
-      <c r="F29" s="23" t="s">
+      <c r="F29" s="22" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="30" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="20" t="s">
+      <c r="A30" s="19" t="s">
         <v>105</v>
       </c>
-      <c r="B30" s="21" t="s">
+      <c r="B30" s="20" t="s">
         <v>102</v>
       </c>
-      <c r="C30" s="21">
+      <c r="C30" s="20">
         <v>3</v>
       </c>
-      <c r="D30" s="21" t="s">
+      <c r="D30" s="20" t="s">
         <v>106</v>
       </c>
-      <c r="E30" s="22" t="s">
+      <c r="E30" s="21" t="s">
         <v>107</v>
       </c>
-      <c r="F30" s="21" t="s">
+      <c r="F30" s="20" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="31" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="20" t="s">
+      <c r="A31" s="19" t="s">
         <v>108</v>
       </c>
-      <c r="B31" s="23" t="s">
+      <c r="B31" s="22" t="s">
         <v>102</v>
       </c>
-      <c r="C31" s="23">
+      <c r="C31" s="22">
         <v>3</v>
       </c>
-      <c r="D31" s="23" t="s">
+      <c r="D31" s="22" t="s">
         <v>103</v>
       </c>
-      <c r="E31" s="24" t="s">
+      <c r="E31" s="23" t="s">
         <v>109</v>
       </c>
-      <c r="F31" s="23" t="s">
+      <c r="F31" s="22" t="s">
         <v>48</v>
       </c>
     </row>
@@ -2933,324 +2850,324 @@
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A2" s="8">
+      <c r="A2" s="7">
         <v>0.375</v>
       </c>
-      <c r="B2" s="4"/>
-      <c r="C2" s="4"/>
-      <c r="D2" s="4"/>
-      <c r="E2" s="4"/>
-      <c r="F2" s="4"/>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A3" s="8">
+      <c r="A3" s="7">
         <v>0.38541666666666669</v>
       </c>
-      <c r="B3" s="4"/>
-      <c r="C3" s="4"/>
-      <c r="D3" s="4"/>
-      <c r="E3" s="4"/>
-      <c r="F3" s="4"/>
+      <c r="B3" s="3"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3"/>
+      <c r="F3" s="3"/>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A4" s="8">
+      <c r="A4" s="7">
         <v>0.39583333333333331</v>
       </c>
-      <c r="B4" s="4"/>
-      <c r="C4" s="4"/>
-      <c r="D4" s="4"/>
-      <c r="E4" s="4"/>
-      <c r="F4" s="4"/>
+      <c r="B4" s="3"/>
+      <c r="C4" s="3"/>
+      <c r="D4" s="3"/>
+      <c r="E4" s="3"/>
+      <c r="F4" s="3"/>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A5" s="8">
+      <c r="A5" s="7">
         <v>0.40625</v>
       </c>
-      <c r="B5" s="4"/>
-      <c r="C5" s="4"/>
-      <c r="D5" s="4"/>
-      <c r="E5" s="4"/>
-      <c r="F5" s="4"/>
+      <c r="B5" s="3"/>
+      <c r="C5" s="3"/>
+      <c r="D5" s="3"/>
+      <c r="E5" s="3"/>
+      <c r="F5" s="3"/>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A6" s="8">
+      <c r="A6" s="7">
         <v>0.41666666666666669</v>
       </c>
-      <c r="B6" s="4"/>
-      <c r="C6" s="4"/>
-      <c r="D6" s="4"/>
-      <c r="E6" s="4"/>
-      <c r="F6" s="4"/>
+      <c r="B6" s="3"/>
+      <c r="C6" s="3"/>
+      <c r="D6" s="3"/>
+      <c r="E6" s="3"/>
+      <c r="F6" s="3"/>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A7" s="8">
+      <c r="A7" s="7">
         <v>0.42708333333333331</v>
       </c>
       <c r="B7" s="30" t="s">
         <v>110</v>
       </c>
-      <c r="C7" s="4"/>
+      <c r="C7" s="3"/>
       <c r="D7" s="30" t="s">
         <v>110</v>
       </c>
-      <c r="E7" s="4"/>
+      <c r="E7" s="3"/>
       <c r="F7" s="30" t="s">
         <v>110</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A8" s="8">
+      <c r="A8" s="7">
         <v>0.4375</v>
       </c>
       <c r="B8" s="31"/>
-      <c r="C8" s="4"/>
+      <c r="C8" s="3"/>
       <c r="D8" s="31"/>
-      <c r="E8" s="4"/>
+      <c r="E8" s="3"/>
       <c r="F8" s="31"/>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A9" s="8">
+      <c r="A9" s="7">
         <v>0.44791666666666669</v>
       </c>
       <c r="B9" s="31"/>
-      <c r="C9" s="4"/>
+      <c r="C9" s="3"/>
       <c r="D9" s="31"/>
-      <c r="E9" s="4"/>
+      <c r="E9" s="3"/>
       <c r="F9" s="31"/>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A10" s="8">
+      <c r="A10" s="7">
         <v>0.45833333333333331</v>
       </c>
       <c r="B10" s="31"/>
-      <c r="C10" s="4"/>
+      <c r="C10" s="3"/>
       <c r="D10" s="31"/>
-      <c r="E10" s="4"/>
+      <c r="E10" s="3"/>
       <c r="F10" s="31"/>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A11" s="8">
+      <c r="A11" s="7">
         <v>0.46875</v>
       </c>
-      <c r="B11" s="4"/>
-      <c r="C11" s="4"/>
-      <c r="D11" s="4"/>
-      <c r="E11" s="4"/>
-      <c r="F11" s="4"/>
+      <c r="B11" s="3"/>
+      <c r="C11" s="3"/>
+      <c r="D11" s="3"/>
+      <c r="E11" s="3"/>
+      <c r="F11" s="3"/>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A12" s="8">
+      <c r="A12" s="7">
         <v>0.47916666666666669</v>
       </c>
-      <c r="B12" s="12"/>
-      <c r="C12" s="12"/>
-      <c r="D12" s="12"/>
-      <c r="E12" s="12"/>
-      <c r="F12" s="12"/>
+      <c r="B12" s="11"/>
+      <c r="C12" s="11"/>
+      <c r="D12" s="11"/>
+      <c r="E12" s="11"/>
+      <c r="F12" s="11"/>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A13" s="8">
+      <c r="A13" s="7">
         <v>0.48958333333333331</v>
       </c>
-      <c r="B13" s="12"/>
-      <c r="C13" s="12"/>
-      <c r="D13" s="12"/>
-      <c r="E13" s="12"/>
-      <c r="F13" s="12"/>
+      <c r="B13" s="11"/>
+      <c r="C13" s="11"/>
+      <c r="D13" s="11"/>
+      <c r="E13" s="11"/>
+      <c r="F13" s="11"/>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A14" s="8">
+      <c r="A14" s="7">
         <v>0.5</v>
       </c>
-      <c r="B14" s="12"/>
-      <c r="C14" s="12"/>
-      <c r="D14" s="12"/>
-      <c r="E14" s="12"/>
-      <c r="F14" s="12"/>
+      <c r="B14" s="11"/>
+      <c r="C14" s="11"/>
+      <c r="D14" s="11"/>
+      <c r="E14" s="11"/>
+      <c r="F14" s="11"/>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A15" s="8">
+      <c r="A15" s="7">
         <v>0.51041666666666663</v>
       </c>
-      <c r="B15" s="12"/>
-      <c r="C15" s="12"/>
-      <c r="D15" s="12"/>
-      <c r="E15" s="12"/>
-      <c r="F15" s="12"/>
+      <c r="B15" s="11"/>
+      <c r="C15" s="11"/>
+      <c r="D15" s="11"/>
+      <c r="E15" s="11"/>
+      <c r="F15" s="11"/>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A16" s="8">
+      <c r="A16" s="7">
         <v>0.52083333333333337</v>
       </c>
-      <c r="B16" s="4"/>
-      <c r="C16" s="4"/>
-      <c r="D16" s="4"/>
-      <c r="E16" s="4"/>
-      <c r="F16" s="4"/>
+      <c r="B16" s="3"/>
+      <c r="C16" s="3"/>
+      <c r="D16" s="3"/>
+      <c r="E16" s="3"/>
+      <c r="F16" s="3"/>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A17" s="8">
+      <c r="A17" s="7">
         <v>0.53125</v>
       </c>
-      <c r="B17" s="4"/>
-      <c r="C17" s="4"/>
-      <c r="D17" s="4"/>
-      <c r="E17" s="4"/>
-      <c r="F17" s="4"/>
+      <c r="B17" s="3"/>
+      <c r="C17" s="3"/>
+      <c r="D17" s="3"/>
+      <c r="E17" s="3"/>
+      <c r="F17" s="3"/>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A18" s="8">
+      <c r="A18" s="7">
         <v>0.54166666666666663</v>
       </c>
-      <c r="B18" s="4"/>
-      <c r="C18" s="4"/>
-      <c r="D18" s="4"/>
-      <c r="E18" s="4"/>
-      <c r="F18" s="4"/>
+      <c r="B18" s="3"/>
+      <c r="C18" s="3"/>
+      <c r="D18" s="3"/>
+      <c r="E18" s="3"/>
+      <c r="F18" s="3"/>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A19" s="8">
+      <c r="A19" s="7">
         <v>0.55208333333333337</v>
       </c>
-      <c r="B19" s="4"/>
-      <c r="C19" s="4"/>
-      <c r="D19" s="4"/>
-      <c r="E19" s="4"/>
-      <c r="F19" s="4"/>
+      <c r="B19" s="3"/>
+      <c r="C19" s="3"/>
+      <c r="D19" s="3"/>
+      <c r="E19" s="3"/>
+      <c r="F19" s="3"/>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A20" s="8">
+      <c r="A20" s="7">
         <v>0.5625</v>
       </c>
-      <c r="B20" s="4"/>
-      <c r="C20" s="4"/>
-      <c r="D20" s="4"/>
-      <c r="E20" s="4"/>
-      <c r="F20" s="4"/>
+      <c r="B20" s="3"/>
+      <c r="C20" s="3"/>
+      <c r="D20" s="3"/>
+      <c r="E20" s="3"/>
+      <c r="F20" s="3"/>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A21" s="8">
+      <c r="A21" s="7">
         <v>0.57291666666666663</v>
       </c>
-      <c r="B21" s="4"/>
-      <c r="C21" s="4"/>
-      <c r="D21" s="4"/>
-      <c r="E21" s="4"/>
-      <c r="F21" s="4"/>
+      <c r="B21" s="3"/>
+      <c r="C21" s="3"/>
+      <c r="D21" s="3"/>
+      <c r="E21" s="3"/>
+      <c r="F21" s="3"/>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A22" s="8">
+      <c r="A22" s="7">
         <v>0.58333333333333337</v>
       </c>
       <c r="B22" s="30" t="s">
         <v>111</v>
       </c>
-      <c r="C22" s="4"/>
+      <c r="C22" s="3"/>
       <c r="D22" s="30" t="s">
         <v>111</v>
       </c>
-      <c r="E22" s="4"/>
+      <c r="E22" s="3"/>
       <c r="F22" s="30" t="s">
         <v>111</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A23" s="8">
+      <c r="A23" s="7">
         <v>0.59375</v>
       </c>
       <c r="B23" s="31"/>
-      <c r="C23" s="4"/>
+      <c r="C23" s="3"/>
       <c r="D23" s="31"/>
-      <c r="E23" s="4"/>
+      <c r="E23" s="3"/>
       <c r="F23" s="31"/>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A24" s="8">
+      <c r="A24" s="7">
         <v>0.60416666666666663</v>
       </c>
       <c r="B24" s="31"/>
-      <c r="C24" s="4"/>
+      <c r="C24" s="3"/>
       <c r="D24" s="31"/>
-      <c r="E24" s="4"/>
+      <c r="E24" s="3"/>
       <c r="F24" s="31"/>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A25" s="8">
+      <c r="A25" s="7">
         <v>0.61458333333333337</v>
       </c>
       <c r="B25" s="31"/>
-      <c r="C25" s="4"/>
+      <c r="C25" s="3"/>
       <c r="D25" s="31"/>
-      <c r="E25" s="4"/>
+      <c r="E25" s="3"/>
       <c r="F25" s="31"/>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A26" s="8">
+      <c r="A26" s="7">
         <v>0.625</v>
       </c>
-      <c r="B26" s="4"/>
-      <c r="C26" s="4"/>
+      <c r="B26" s="3"/>
+      <c r="C26" s="3"/>
       <c r="D26" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="E26" s="4"/>
-      <c r="F26" s="4"/>
+      <c r="E26" s="3"/>
+      <c r="F26" s="3"/>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A27" s="8">
+      <c r="A27" s="7">
         <v>0.63541666666666663</v>
       </c>
-      <c r="B27" s="34" t="s">
+      <c r="B27" s="38" t="s">
         <v>112</v>
       </c>
-      <c r="C27" s="6"/>
-      <c r="D27" s="34" t="s">
+      <c r="C27" s="5"/>
+      <c r="D27" s="38" t="s">
         <v>112</v>
       </c>
-      <c r="E27" s="6"/>
-      <c r="F27" s="34" t="s">
+      <c r="E27" s="5"/>
+      <c r="F27" s="38" t="s">
         <v>112</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A28" s="8">
+      <c r="A28" s="7">
         <v>0.64583333333333337</v>
       </c>
       <c r="B28" s="31"/>
-      <c r="C28" s="6"/>
+      <c r="C28" s="5"/>
       <c r="D28" s="31"/>
-      <c r="E28" s="6"/>
+      <c r="E28" s="5"/>
       <c r="F28" s="31"/>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A29" s="8">
+      <c r="A29" s="7">
         <v>0.65625</v>
       </c>
       <c r="B29" s="31"/>
-      <c r="C29" s="6"/>
+      <c r="C29" s="5"/>
       <c r="D29" s="31"/>
-      <c r="E29" s="6"/>
+      <c r="E29" s="5"/>
       <c r="F29" s="31"/>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A30" s="8">
+      <c r="A30" s="7">
         <v>0.66666666666666663</v>
       </c>
       <c r="B30" s="31"/>
-      <c r="C30" s="6"/>
+      <c r="C30" s="5"/>
       <c r="D30" s="31"/>
-      <c r="E30" s="6"/>
+      <c r="E30" s="5"/>
       <c r="F30" s="31"/>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A31" s="8">
+      <c r="A31" s="7">
         <v>0.67708333333333337</v>
       </c>
-      <c r="B31" s="4"/>
-      <c r="C31" s="4"/>
-      <c r="D31" s="4"/>
-      <c r="E31" s="4"/>
-      <c r="F31" s="4"/>
+      <c r="B31" s="3"/>
+      <c r="C31" s="3"/>
+      <c r="D31" s="3"/>
+      <c r="E31" s="3"/>
+      <c r="F31" s="3"/>
     </row>
   </sheetData>
   <mergeCells count="9">

</xml_diff>

<commit_message>
Update at 21:21 on 09/02/2020
</commit_message>
<xml_diff>
--- a/site_libs/records/fall 2020.xlsx
+++ b/site_libs/records/fall 2020.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Portfolio\site_libs\records\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C8B1B8A-D56E-42F1-A823-104999045D89}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0308017B-7DD9-400C-81E1-FB433F621D65}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="230" uniqueCount="126">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="123">
   <si>
     <t>Monday</t>
   </si>
@@ -398,29 +398,11 @@
 Falin</t>
   </si>
   <si>
-    <t>121b</t>
-  </si>
-  <si>
-    <t>JavaScript</t>
-  </si>
-  <si>
-    <t>10:15-11:15</t>
-  </si>
-  <si>
-    <t>Barney</t>
-  </si>
-  <si>
     <t>TA 
 ECEN 361
 Grimmett</t>
   </si>
   <si>
-    <t>CSE 121b 
-JavaScript 
-Barney 
-Remote</t>
-  </si>
-  <si>
     <t>TA 
 ECEN 340 
 Jack</t>
@@ -444,6 +426,15 @@
   </si>
   <si>
     <t>Depart</t>
+  </si>
+  <si>
+    <t>JavaScript
+Barney
+JA</t>
+  </si>
+  <si>
+    <t>DSS
+JA</t>
   </si>
 </sst>
 </file>
@@ -508,11 +499,6 @@
       <name val="Arial"/>
     </font>
     <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
       <b/>
       <sz val="11"/>
       <color rgb="FF0076B6"/>
@@ -556,7 +542,13 @@
     </font>
     <font>
       <sz val="10"/>
-      <color rgb="FFC00000"/>
+      <color rgb="FFFF0000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="4" tint="-0.249977111117893"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -593,7 +585,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -655,13 +647,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -670,40 +662,46 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -922,7 +920,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:P59"/>
+  <dimension ref="A1:P54"/>
   <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="11.7109375" customWidth="1"/>
@@ -959,8 +957,8 @@
         <v>4</v>
       </c>
       <c r="G1" s="1"/>
-      <c r="H1" s="43" t="s">
-        <v>125</v>
+      <c r="H1" s="31" t="s">
+        <v>120</v>
       </c>
       <c r="I1" s="2" t="s">
         <v>6</v>
@@ -989,230 +987,217 @@
     </row>
     <row r="2" spans="1:16" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A2" s="7">
-        <v>0.36458333333333298</v>
-      </c>
-      <c r="B2" s="28"/>
-      <c r="C2" s="28"/>
-      <c r="D2" s="28"/>
-      <c r="E2" s="28"/>
-      <c r="F2" s="28"/>
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="B2" s="3"/>
+      <c r="C2" s="10"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="10"/>
+      <c r="F2" s="3"/>
       <c r="G2" s="3"/>
-      <c r="H2" s="12" t="s">
+      <c r="H2" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="I2" s="12" t="s">
-        <v>113</v>
-      </c>
-      <c r="J2" s="12" t="s">
-        <v>114</v>
+      <c r="I2" s="6">
+        <v>450</v>
+      </c>
+      <c r="J2" s="6" t="s">
+        <v>15</v>
       </c>
       <c r="K2" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="L2" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="M2" s="12" t="s">
-        <v>26</v>
-      </c>
-      <c r="N2" s="12" t="s">
-        <v>115</v>
-      </c>
-      <c r="O2" s="12" t="s">
-        <v>116</v>
+        <v>16</v>
+      </c>
+      <c r="L2" s="6">
+        <v>347</v>
+      </c>
+      <c r="M2" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="N2" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="O2" s="6" t="s">
+        <v>19</v>
       </c>
       <c r="P2" s="12">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:16" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A3" s="7">
-        <v>0.375</v>
-      </c>
-      <c r="B3" s="28"/>
-      <c r="C3" s="28"/>
-      <c r="D3" s="28"/>
-      <c r="E3" s="28"/>
-      <c r="F3" s="28"/>
+        <v>0.42708333333333331</v>
+      </c>
+      <c r="B3" s="33" t="s">
+        <v>29</v>
+      </c>
+      <c r="C3" s="42" t="s">
+        <v>121</v>
+      </c>
+      <c r="D3" s="33" t="s">
+        <v>30</v>
+      </c>
+      <c r="E3" s="42" t="s">
+        <v>121</v>
+      </c>
+      <c r="F3" s="45" t="s">
+        <v>115</v>
+      </c>
       <c r="G3" s="3"/>
       <c r="H3" s="6" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="I3" s="6">
-        <v>450</v>
+        <v>325</v>
       </c>
       <c r="J3" s="6" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="K3" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="L3" s="6">
-        <v>347</v>
+        <v>22</v>
+      </c>
+      <c r="L3" s="6" t="s">
+        <v>23</v>
       </c>
       <c r="M3" s="6" t="s">
         <v>17</v>
       </c>
       <c r="N3" s="6" t="s">
-        <v>18</v>
+        <v>116</v>
       </c>
       <c r="O3" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="P3" s="12">
+        <v>25</v>
+      </c>
+      <c r="P3" s="6">
         <v>3</v>
       </c>
     </row>
     <row r="4" spans="1:16" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A4" s="7">
-        <v>0.38541666666666702</v>
-      </c>
-      <c r="B4" s="28"/>
-      <c r="C4" s="28"/>
-      <c r="D4" s="28"/>
-      <c r="E4" s="28"/>
-      <c r="F4" s="28"/>
+        <v>0.4375</v>
+      </c>
+      <c r="B4" s="34"/>
+      <c r="C4" s="42"/>
+      <c r="D4" s="34"/>
+      <c r="E4" s="42"/>
+      <c r="F4" s="45"/>
       <c r="G4" s="3"/>
-      <c r="H4" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="I4" s="6">
-        <v>325</v>
-      </c>
-      <c r="J4" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="K4" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="L4" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="M4" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="N4" s="6" t="s">
-        <v>121</v>
-      </c>
-      <c r="O4" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="P4" s="6">
-        <v>3</v>
-      </c>
+      <c r="P4" s="6"/>
     </row>
     <row r="5" spans="1:16" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A5" s="7">
-        <v>0.39583333333333331</v>
-      </c>
-      <c r="B5" s="3"/>
-      <c r="C5" s="3"/>
-      <c r="D5" s="3"/>
-      <c r="E5" s="3"/>
-      <c r="F5" s="3"/>
+        <v>0.44791666666666669</v>
+      </c>
+      <c r="B5" s="34"/>
+      <c r="C5" s="42"/>
+      <c r="D5" s="34"/>
+      <c r="E5" s="42"/>
+      <c r="F5" s="45"/>
       <c r="G5" s="3"/>
-      <c r="P5" s="6"/>
+      <c r="P5">
+        <f>SUM(P2:P4)</f>
+        <v>6</v>
+      </c>
     </row>
     <row r="6" spans="1:16" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A6" s="7">
-        <v>0.40625</v>
-      </c>
-      <c r="B6" s="3"/>
-      <c r="C6" s="10"/>
-      <c r="D6" s="3"/>
-      <c r="E6" s="10"/>
-      <c r="F6" s="3"/>
+        <v>0.45833333333333331</v>
+      </c>
+      <c r="B6" s="34"/>
+      <c r="C6" s="42"/>
+      <c r="D6" s="34"/>
+      <c r="E6" s="42"/>
+      <c r="F6" s="45"/>
       <c r="G6" s="3"/>
-      <c r="P6">
-        <f>SUM(P2:P5)</f>
-        <v>7</v>
-      </c>
     </row>
     <row r="7" spans="1:16" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A7" s="7">
-        <v>0.41666666666666669</v>
+        <v>0.46875</v>
       </c>
       <c r="B7" s="3"/>
-      <c r="C7" s="10"/>
+      <c r="C7" s="3"/>
       <c r="D7" s="3"/>
-      <c r="E7" s="10"/>
+      <c r="E7" s="3"/>
       <c r="F7" s="3"/>
       <c r="G7" s="3"/>
+      <c r="H7" s="8"/>
     </row>
     <row r="8" spans="1:16" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A8" s="7">
-        <v>0.42708333333333331</v>
-      </c>
-      <c r="B8" s="32" t="s">
-        <v>29</v>
-      </c>
-      <c r="C8" s="36" t="s">
-        <v>118</v>
-      </c>
-      <c r="D8" s="32" t="s">
-        <v>30</v>
-      </c>
-      <c r="E8" s="36" t="str">
-        <f>C8</f>
-        <v>CSE 121b 
-JavaScript 
-Barney 
-Remote</v>
-      </c>
-      <c r="F8" s="35" t="s">
-        <v>120</v>
+        <v>0.47916666666666669</v>
+      </c>
+      <c r="B8" s="36" t="s">
+        <v>31</v>
+      </c>
+      <c r="C8" s="38" t="s">
+        <v>117</v>
+      </c>
+      <c r="D8" s="37" t="str">
+        <f>B8</f>
+        <v>CSE 450
+Machine Learning
+Burton 
+STC  394</v>
+      </c>
+      <c r="E8" s="38" t="s">
+        <v>117</v>
+      </c>
+      <c r="F8" s="37" t="str">
+        <f>D8</f>
+        <v>CSE 450
+Machine Learning
+Burton 
+STC  394</v>
       </c>
       <c r="G8" s="3"/>
-      <c r="H8" s="8"/>
+      <c r="H8" s="30" t="s">
+        <v>28</v>
+      </c>
+      <c r="I8" s="30">
+        <v>12</v>
+      </c>
     </row>
     <row r="9" spans="1:16" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A9" s="7">
-        <v>0.4375</v>
-      </c>
-      <c r="B9" s="33"/>
-      <c r="C9" s="36"/>
-      <c r="D9" s="33"/>
-      <c r="E9" s="36"/>
-      <c r="F9" s="35"/>
+        <v>0.48958333333333331</v>
+      </c>
+      <c r="B9" s="34"/>
+      <c r="C9" s="38"/>
+      <c r="D9" s="34"/>
+      <c r="E9" s="38"/>
+      <c r="F9" s="34"/>
       <c r="G9" s="3"/>
-      <c r="H9" s="41" t="s">
-        <v>28</v>
-      </c>
-      <c r="I9" s="41">
-        <v>12</v>
+      <c r="H9" s="43" t="s">
+        <v>118</v>
+      </c>
+      <c r="I9" s="43" t="s">
+        <v>119</v>
       </c>
     </row>
     <row r="10" spans="1:16" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A10" s="7">
-        <v>0.44791666666666669</v>
-      </c>
-      <c r="B10" s="33"/>
-      <c r="C10" s="36"/>
-      <c r="D10" s="33"/>
-      <c r="E10" s="36"/>
-      <c r="F10" s="35"/>
+        <v>0.5</v>
+      </c>
+      <c r="B10" s="34"/>
+      <c r="C10" s="38"/>
+      <c r="D10" s="34"/>
+      <c r="E10" s="38"/>
+      <c r="F10" s="34"/>
       <c r="G10" s="3"/>
-      <c r="H10" s="42" t="s">
-        <v>123</v>
-      </c>
-      <c r="I10" s="42" t="s">
-        <v>124</v>
-      </c>
     </row>
     <row r="11" spans="1:16" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A11" s="7">
-        <v>0.45833333333333331</v>
-      </c>
-      <c r="B11" s="33"/>
-      <c r="C11" s="36"/>
-      <c r="D11" s="33"/>
-      <c r="E11" s="36"/>
-      <c r="F11" s="35"/>
+        <v>0.51041666666666663</v>
+      </c>
+      <c r="B11" s="34"/>
+      <c r="C11" s="38"/>
+      <c r="D11" s="34"/>
+      <c r="E11" s="38"/>
+      <c r="F11" s="34"/>
       <c r="G11" s="3"/>
     </row>
     <row r="12" spans="1:16" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A12" s="7">
-        <v>0.46875</v>
+        <v>0.52083333333333337</v>
       </c>
       <c r="B12" s="3"/>
       <c r="C12" s="3"/>
@@ -1222,417 +1207,357 @@
     </row>
     <row r="13" spans="1:16" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A13" s="7">
-        <v>0.47916666666666669</v>
-      </c>
-      <c r="B13" s="37" t="s">
-        <v>31</v>
-      </c>
-      <c r="C13" s="34" t="s">
-        <v>122</v>
-      </c>
-      <c r="D13" s="38" t="str">
-        <f>B13</f>
-        <v>CSE 450
-Machine Learning
-Burton 
-STC  394</v>
-      </c>
-      <c r="E13" s="34" t="s">
-        <v>122</v>
-      </c>
-      <c r="F13" s="38" t="str">
-        <f>D13</f>
-        <v>CSE 450
-Machine Learning
-Burton 
-STC  394</v>
+        <v>0.53125</v>
+      </c>
+      <c r="B13" s="33" t="s">
+        <v>113</v>
+      </c>
+      <c r="C13" s="33" t="s">
+        <v>29</v>
+      </c>
+      <c r="D13" s="33" t="s">
+        <v>113</v>
+      </c>
+      <c r="E13" s="33" t="s">
+        <v>30</v>
+      </c>
+      <c r="F13" s="32" t="s">
+        <v>115</v>
       </c>
     </row>
     <row r="14" spans="1:16" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A14" s="7">
-        <v>0.48958333333333331</v>
-      </c>
-      <c r="B14" s="33"/>
+        <v>0.54166666666666663</v>
+      </c>
+      <c r="B14" s="34"/>
       <c r="C14" s="34"/>
-      <c r="D14" s="33"/>
+      <c r="D14" s="34"/>
       <c r="E14" s="34"/>
-      <c r="F14" s="33"/>
+      <c r="F14" s="32"/>
     </row>
     <row r="15" spans="1:16" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A15" s="7">
-        <v>0.5</v>
-      </c>
-      <c r="B15" s="33"/>
+        <v>0.55208333333333337</v>
+      </c>
+      <c r="B15" s="34"/>
       <c r="C15" s="34"/>
-      <c r="D15" s="33"/>
+      <c r="D15" s="34"/>
       <c r="E15" s="34"/>
-      <c r="F15" s="33"/>
+      <c r="F15" s="32"/>
     </row>
     <row r="16" spans="1:16" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A16" s="7">
-        <v>0.51041666666666663</v>
-      </c>
-      <c r="B16" s="33"/>
+        <v>0.5625</v>
+      </c>
+      <c r="B16" s="34"/>
       <c r="C16" s="34"/>
-      <c r="D16" s="33"/>
+      <c r="D16" s="34"/>
       <c r="E16" s="34"/>
-      <c r="F16" s="33"/>
+      <c r="F16" s="32"/>
     </row>
     <row r="17" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A17" s="7">
-        <v>0.52083333333333337</v>
-      </c>
-      <c r="B17" s="3"/>
-      <c r="C17" s="3"/>
-      <c r="D17" s="3"/>
-      <c r="E17" s="3"/>
-      <c r="F17" s="3"/>
+        <v>0.57291666666666663</v>
+      </c>
+      <c r="B17" s="24"/>
+      <c r="C17" s="29"/>
+      <c r="D17" s="24"/>
+      <c r="E17" s="29"/>
+      <c r="F17" s="24"/>
     </row>
     <row r="18" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A18" s="7">
-        <v>0.53125</v>
-      </c>
-      <c r="B18" s="32" t="s">
-        <v>117</v>
-      </c>
-      <c r="C18" s="32" t="s">
-        <v>29</v>
-      </c>
-      <c r="D18" s="32" t="s">
-        <v>117</v>
-      </c>
-      <c r="E18" s="32" t="s">
-        <v>30</v>
-      </c>
-      <c r="F18" s="35" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A19" s="7">
-        <v>0.54166666666666663</v>
-      </c>
-      <c r="B19" s="33"/>
-      <c r="C19" s="33"/>
-      <c r="D19" s="33"/>
-      <c r="E19" s="33"/>
-      <c r="F19" s="35"/>
-    </row>
-    <row r="20" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A20" s="7">
-        <v>0.55208333333333337</v>
-      </c>
-      <c r="B20" s="33"/>
-      <c r="C20" s="33"/>
-      <c r="D20" s="33"/>
-      <c r="E20" s="33"/>
-      <c r="F20" s="35"/>
-    </row>
-    <row r="21" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A21" s="7">
-        <v>0.5625</v>
-      </c>
-      <c r="B21" s="33"/>
-      <c r="C21" s="33"/>
-      <c r="D21" s="33"/>
-      <c r="E21" s="33"/>
-      <c r="F21" s="35"/>
-    </row>
-    <row r="22" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A22" s="7">
-        <v>0.57291666666666663</v>
-      </c>
-      <c r="B22" s="24"/>
-      <c r="C22" s="29"/>
-      <c r="D22" s="24"/>
-      <c r="E22" s="29"/>
-      <c r="F22" s="24"/>
-    </row>
-    <row r="23" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A23" s="7">
         <v>0.58333333333333337</v>
       </c>
-      <c r="B23" s="30" t="s">
+      <c r="B18" s="35" t="s">
         <v>32</v>
       </c>
-      <c r="C23" s="32" t="s">
+      <c r="C18" s="33" t="s">
         <v>33</v>
       </c>
-      <c r="D23" s="30" t="str">
-        <f>B23</f>
+      <c r="D18" s="35" t="str">
+        <f>B18</f>
         <v>MATH 325
 Intermediate Stats 
 Saunders 
 Remote</v>
       </c>
-      <c r="E23" s="32" t="s">
+      <c r="E18" s="33" t="s">
         <v>33</v>
       </c>
-      <c r="F23" s="30" t="str">
-        <f>D23</f>
+      <c r="F18" s="35" t="str">
+        <f>D18</f>
         <v>MATH 325
 Intermediate Stats 
 Saunders 
 Remote</v>
       </c>
     </row>
+    <row r="19" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A19" s="7">
+        <v>0.59375</v>
+      </c>
+      <c r="B19" s="34"/>
+      <c r="C19" s="34"/>
+      <c r="D19" s="34"/>
+      <c r="E19" s="34"/>
+      <c r="F19" s="34"/>
+    </row>
+    <row r="20" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A20" s="7">
+        <v>0.60416666666666663</v>
+      </c>
+      <c r="B20" s="34"/>
+      <c r="C20" s="34"/>
+      <c r="D20" s="34"/>
+      <c r="E20" s="34"/>
+      <c r="F20" s="34"/>
+    </row>
+    <row r="21" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A21" s="7">
+        <v>0.61458333333333337</v>
+      </c>
+      <c r="B21" s="34"/>
+      <c r="C21" s="34"/>
+      <c r="D21" s="34"/>
+      <c r="E21" s="34"/>
+      <c r="F21" s="34"/>
+    </row>
+    <row r="22" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A22" s="7">
+        <v>0.625</v>
+      </c>
+      <c r="B22" s="3"/>
+      <c r="C22" s="3"/>
+      <c r="D22" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="E22" s="3"/>
+      <c r="F22" s="3"/>
+    </row>
+    <row r="23" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A23" s="7">
+        <v>0.63541666666666663</v>
+      </c>
+      <c r="B23" s="32" t="s">
+        <v>114</v>
+      </c>
+      <c r="C23" s="5"/>
+      <c r="D23" s="32" t="s">
+        <v>114</v>
+      </c>
+      <c r="E23" s="5"/>
+      <c r="F23" s="5"/>
+    </row>
     <row r="24" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A24" s="7">
-        <v>0.59375</v>
+        <v>0.64583333333333337</v>
       </c>
       <c r="B24" s="33"/>
-      <c r="C24" s="33"/>
+      <c r="C24" s="5"/>
       <c r="D24" s="33"/>
-      <c r="E24" s="33"/>
-      <c r="F24" s="33"/>
+      <c r="E24" s="5"/>
+      <c r="F24" s="5"/>
     </row>
     <row r="25" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A25" s="7">
-        <v>0.60416666666666663</v>
+        <v>0.65625</v>
       </c>
       <c r="B25" s="33"/>
-      <c r="C25" s="33"/>
+      <c r="C25" s="5"/>
       <c r="D25" s="33"/>
-      <c r="E25" s="33"/>
-      <c r="F25" s="33"/>
+      <c r="E25" s="5"/>
+      <c r="F25" s="5"/>
     </row>
     <row r="26" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A26" s="7">
-        <v>0.61458333333333337</v>
+        <v>0.66666666666666663</v>
       </c>
       <c r="B26" s="33"/>
-      <c r="C26" s="33"/>
+      <c r="C26" s="5"/>
       <c r="D26" s="33"/>
-      <c r="E26" s="33"/>
-      <c r="F26" s="33"/>
+      <c r="E26" s="5"/>
+      <c r="F26" s="5"/>
     </row>
     <row r="27" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A27" s="7">
-        <v>0.625</v>
-      </c>
-      <c r="B27" s="3"/>
+        <v>0.67708333333333337</v>
+      </c>
+      <c r="B27" s="33"/>
       <c r="C27" s="3"/>
-      <c r="D27" s="3" t="s">
-        <v>34</v>
-      </c>
+      <c r="D27" s="33"/>
       <c r="E27" s="3"/>
       <c r="F27" s="3"/>
     </row>
     <row r="28" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A28" s="7">
-        <v>0.63541666666666663</v>
-      </c>
-      <c r="B28" s="35" t="s">
-        <v>119</v>
-      </c>
-      <c r="C28" s="5"/>
-      <c r="D28" s="35" t="s">
-        <v>119</v>
-      </c>
-      <c r="E28" s="5"/>
-      <c r="F28" s="5"/>
+        <v>0.6875</v>
+      </c>
     </row>
     <row r="29" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A29" s="7">
-        <v>0.64583333333333337</v>
-      </c>
-      <c r="B29" s="32"/>
-      <c r="C29" s="5"/>
-      <c r="D29" s="32"/>
-      <c r="E29" s="5"/>
-      <c r="F29" s="5"/>
+        <v>0.69791666666666696</v>
+      </c>
     </row>
     <row r="30" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A30" s="7">
-        <v>0.65625</v>
-      </c>
-      <c r="B30" s="32"/>
-      <c r="C30" s="5"/>
-      <c r="D30" s="32"/>
-      <c r="E30" s="5"/>
-      <c r="F30" s="5"/>
+        <v>0.70833333333333404</v>
+      </c>
     </row>
     <row r="31" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A31" s="7">
-        <v>0.66666666666666663</v>
-      </c>
-      <c r="B31" s="32"/>
-      <c r="C31" s="5"/>
-      <c r="D31" s="32"/>
-      <c r="E31" s="5"/>
-      <c r="F31" s="5"/>
+        <v>0.718750000000001</v>
+      </c>
     </row>
     <row r="32" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A32" s="7">
-        <v>0.67708333333333337</v>
-      </c>
-      <c r="B32" s="32"/>
-      <c r="C32" s="3"/>
-      <c r="D32" s="32"/>
-      <c r="E32" s="3"/>
-      <c r="F32" s="3"/>
-    </row>
-    <row r="33" spans="1:1" ht="12.75" x14ac:dyDescent="0.2">
+        <v>0.72916666666666696</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A33" s="7">
-        <v>0.6875</v>
-      </c>
-    </row>
-    <row r="34" spans="1:1" ht="12.75" x14ac:dyDescent="0.2">
+        <v>0.73958333333333404</v>
+      </c>
+      <c r="D33" s="42" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A34" s="7">
-        <v>0.69791666666666696</v>
-      </c>
-    </row>
-    <row r="35" spans="1:1" ht="12.75" x14ac:dyDescent="0.2">
+        <v>0.750000000000001</v>
+      </c>
+      <c r="D34" s="44"/>
+    </row>
+    <row r="35" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A35" s="7">
-        <v>0.70833333333333404</v>
-      </c>
-    </row>
-    <row r="36" spans="1:1" ht="12.75" x14ac:dyDescent="0.2">
+        <v>0.76041666666666796</v>
+      </c>
+      <c r="D35" s="44"/>
+    </row>
+    <row r="36" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A36" s="7">
-        <v>0.718750000000001</v>
-      </c>
-    </row>
-    <row r="37" spans="1:1" ht="12.75" x14ac:dyDescent="0.2">
+        <v>0.77083333333333504</v>
+      </c>
+      <c r="D36" s="44"/>
+    </row>
+    <row r="37" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A37" s="7">
-        <v>0.72916666666666696</v>
-      </c>
-    </row>
-    <row r="38" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>0.781250000000001</v>
+      </c>
+      <c r="D37" s="44"/>
+    </row>
+    <row r="38" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="7">
-        <v>0.73958333333333404</v>
-      </c>
-    </row>
-    <row r="39" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>0.79166666666666796</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="7">
-        <v>0.750000000000001</v>
-      </c>
-    </row>
-    <row r="40" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>0.80208333333333504</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="7">
-        <v>0.76041666666666796</v>
-      </c>
-    </row>
-    <row r="41" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>0.812500000000002</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="7">
-        <v>0.77083333333333504</v>
-      </c>
-    </row>
-    <row r="42" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>0.82291666666666796</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="7">
-        <v>0.781250000000001</v>
-      </c>
-    </row>
-    <row r="43" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>0.83333333333333504</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="7">
-        <v>0.79166666666666796</v>
-      </c>
-    </row>
-    <row r="44" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>0.843750000000002</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="7">
-        <v>0.80208333333333504</v>
-      </c>
-    </row>
-    <row r="45" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>0.85416666666666896</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="7">
-        <v>0.812500000000002</v>
-      </c>
-    </row>
-    <row r="46" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>0.86458333333333504</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="7">
-        <v>0.82291666666666796</v>
-      </c>
-    </row>
-    <row r="47" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>0.874999999999999</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="7">
-        <v>0.83333333333333504</v>
-      </c>
-    </row>
-    <row r="48" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>0.88541666666666596</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" s="7">
-        <v>0.843750000000002</v>
+        <v>0.89583333333333204</v>
       </c>
     </row>
     <row r="49" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" s="7">
-        <v>0.85416666666666896</v>
+        <v>0.906249999999999</v>
       </c>
     </row>
     <row r="50" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" s="7">
-        <v>0.86458333333333504</v>
+        <v>0.91666666666666596</v>
       </c>
     </row>
     <row r="51" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A51" s="7">
-        <v>0.874999999999999</v>
+        <v>0.92708333333333204</v>
       </c>
     </row>
     <row r="52" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A52" s="7">
-        <v>0.88541666666666596</v>
+        <v>0.937499999999999</v>
       </c>
     </row>
     <row r="53" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A53" s="7">
-        <v>0.89583333333333204</v>
+        <v>0.94791666666666596</v>
       </c>
     </row>
     <row r="54" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A54" s="7">
-        <v>0.906249999999999</v>
-      </c>
-    </row>
-    <row r="55" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A55" s="7">
-        <v>0.91666666666666596</v>
-      </c>
-    </row>
-    <row r="56" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A56" s="7">
-        <v>0.92708333333333204</v>
-      </c>
-    </row>
-    <row r="57" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A57" s="7">
-        <v>0.937499999999999</v>
-      </c>
-    </row>
-    <row r="58" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A58" s="7">
-        <v>0.94791666666666596</v>
-      </c>
-    </row>
-    <row r="59" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A59" s="7">
         <v>0.95833333333333204</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="22">
-    <mergeCell ref="B28:B32"/>
-    <mergeCell ref="C23:C26"/>
+  <mergeCells count="23">
+    <mergeCell ref="D33:D37"/>
+    <mergeCell ref="F18:F21"/>
+    <mergeCell ref="B8:B11"/>
     <mergeCell ref="D8:D11"/>
-    <mergeCell ref="D28:D32"/>
-    <mergeCell ref="E23:E26"/>
-    <mergeCell ref="B23:B26"/>
-    <mergeCell ref="D23:D26"/>
-    <mergeCell ref="F23:F26"/>
+    <mergeCell ref="F8:F11"/>
+    <mergeCell ref="C13:C16"/>
+    <mergeCell ref="B3:B6"/>
+    <mergeCell ref="B13:B16"/>
+    <mergeCell ref="F3:F6"/>
+    <mergeCell ref="F13:F16"/>
     <mergeCell ref="C8:C11"/>
     <mergeCell ref="E8:E11"/>
-    <mergeCell ref="B13:B16"/>
     <mergeCell ref="D13:D16"/>
-    <mergeCell ref="F13:F16"/>
+    <mergeCell ref="E13:E16"/>
+    <mergeCell ref="C3:C6"/>
+    <mergeCell ref="B23:B27"/>
     <mergeCell ref="C18:C21"/>
-    <mergeCell ref="B8:B11"/>
+    <mergeCell ref="D3:D6"/>
+    <mergeCell ref="D23:D27"/>
+    <mergeCell ref="E18:E21"/>
     <mergeCell ref="B18:B21"/>
-    <mergeCell ref="F8:F11"/>
-    <mergeCell ref="F18:F21"/>
-    <mergeCell ref="C13:C16"/>
-    <mergeCell ref="E13:E16"/>
     <mergeCell ref="D18:D21"/>
-    <mergeCell ref="E18:E21"/>
+    <mergeCell ref="E3:E6"/>
   </mergeCells>
-  <phoneticPr fontId="16" type="noConversion"/>
+  <phoneticPr fontId="15" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
@@ -1666,26 +1591,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="B1" s="30" t="s">
+      <c r="B1" s="35" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="31"/>
-      <c r="D1" s="30" t="s">
+      <c r="C1" s="39"/>
+      <c r="D1" s="35" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="31"/>
-      <c r="F1" s="30" t="s">
+      <c r="E1" s="39"/>
+      <c r="F1" s="35" t="s">
         <v>2</v>
       </c>
-      <c r="G1" s="31"/>
-      <c r="H1" s="30" t="s">
+      <c r="G1" s="39"/>
+      <c r="H1" s="35" t="s">
         <v>3</v>
       </c>
-      <c r="I1" s="31"/>
-      <c r="J1" s="30" t="s">
+      <c r="I1" s="39"/>
+      <c r="J1" s="35" t="s">
         <v>4</v>
       </c>
-      <c r="K1" s="31"/>
+      <c r="K1" s="39"/>
       <c r="L1" s="1"/>
       <c r="M1" s="2" t="s">
         <v>5</v>
@@ -1770,11 +1695,11 @@
         <v>0.34375</v>
       </c>
       <c r="B3" s="3"/>
-      <c r="D3" s="31"/>
+      <c r="D3" s="39"/>
       <c r="E3" s="3"/>
       <c r="F3" s="3"/>
       <c r="G3" s="3"/>
-      <c r="H3" s="31"/>
+      <c r="H3" s="39"/>
       <c r="I3" s="3"/>
       <c r="J3" s="3"/>
       <c r="K3" s="3"/>
@@ -1812,11 +1737,11 @@
         <v>0.35416666666666669</v>
       </c>
       <c r="B4" s="3"/>
-      <c r="D4" s="31"/>
+      <c r="D4" s="39"/>
       <c r="E4" s="3"/>
       <c r="F4" s="3"/>
       <c r="G4" s="3"/>
-      <c r="H4" s="31"/>
+      <c r="H4" s="39"/>
       <c r="I4" s="3"/>
       <c r="J4" s="3"/>
       <c r="K4" s="3"/>
@@ -1854,11 +1779,11 @@
         <v>0.36458333333333331</v>
       </c>
       <c r="B5" s="3"/>
-      <c r="D5" s="31"/>
+      <c r="D5" s="39"/>
       <c r="E5" s="3"/>
       <c r="F5" s="3"/>
       <c r="G5" s="3"/>
-      <c r="H5" s="31"/>
+      <c r="H5" s="39"/>
       <c r="I5" s="3"/>
       <c r="J5" s="3"/>
       <c r="K5" s="3"/>
@@ -1896,11 +1821,11 @@
         <v>0.375</v>
       </c>
       <c r="B6" s="3"/>
-      <c r="D6" s="31"/>
+      <c r="D6" s="39"/>
       <c r="E6" s="3"/>
       <c r="F6" s="3"/>
       <c r="G6" s="3"/>
-      <c r="H6" s="31"/>
+      <c r="H6" s="39"/>
       <c r="I6" s="3"/>
       <c r="J6" s="3"/>
       <c r="K6" s="3"/>
@@ -1911,11 +1836,11 @@
         <v>0.38541666666666669</v>
       </c>
       <c r="B7" s="3"/>
-      <c r="D7" s="31"/>
+      <c r="D7" s="39"/>
       <c r="E7" s="3"/>
       <c r="F7" s="3"/>
       <c r="G7" s="3"/>
-      <c r="H7" s="31"/>
+      <c r="H7" s="39"/>
       <c r="I7" s="3"/>
       <c r="J7" s="3"/>
       <c r="K7" s="3"/>
@@ -1966,11 +1891,11 @@
         <v>0.41666666666666669</v>
       </c>
       <c r="B10" s="3"/>
-      <c r="D10" s="31"/>
+      <c r="D10" s="39"/>
       <c r="E10" s="3"/>
       <c r="F10" s="3"/>
       <c r="G10" s="3"/>
-      <c r="H10" s="31"/>
+      <c r="H10" s="39"/>
       <c r="I10" s="3"/>
       <c r="J10" s="3"/>
       <c r="K10" s="3"/>
@@ -1981,19 +1906,19 @@
         <v>0.42708333333333331</v>
       </c>
       <c r="B11" s="1"/>
-      <c r="C11" s="39" t="s">
+      <c r="C11" s="41" t="s">
         <v>29</v>
       </c>
-      <c r="D11" s="31"/>
+      <c r="D11" s="39"/>
       <c r="E11" s="3"/>
       <c r="F11" s="1">
         <f>B11</f>
         <v>0</v>
       </c>
-      <c r="G11" s="39" t="s">
+      <c r="G11" s="41" t="s">
         <v>30</v>
       </c>
-      <c r="H11" s="31"/>
+      <c r="H11" s="39"/>
       <c r="I11" s="3"/>
       <c r="J11" s="1"/>
     </row>
@@ -2002,12 +1927,12 @@
         <v>0.4375</v>
       </c>
       <c r="B12" s="1"/>
-      <c r="C12" s="31"/>
-      <c r="D12" s="31"/>
+      <c r="C12" s="39"/>
+      <c r="D12" s="39"/>
       <c r="E12" s="3"/>
       <c r="F12" s="1"/>
-      <c r="G12" s="31"/>
-      <c r="H12" s="31"/>
+      <c r="G12" s="39"/>
+      <c r="H12" s="39"/>
       <c r="I12" s="3"/>
       <c r="J12" s="1"/>
     </row>
@@ -2016,12 +1941,12 @@
         <v>0.44791666666666669</v>
       </c>
       <c r="B13" s="1"/>
-      <c r="C13" s="31"/>
-      <c r="D13" s="31"/>
+      <c r="C13" s="39"/>
+      <c r="D13" s="39"/>
       <c r="E13" s="3"/>
       <c r="F13" s="1"/>
-      <c r="G13" s="31"/>
-      <c r="H13" s="31"/>
+      <c r="G13" s="39"/>
+      <c r="H13" s="39"/>
       <c r="I13" s="3"/>
       <c r="J13" s="1"/>
     </row>
@@ -2030,12 +1955,12 @@
         <v>0.45833333333333331</v>
       </c>
       <c r="B14" s="1"/>
-      <c r="C14" s="31"/>
-      <c r="D14" s="31"/>
+      <c r="C14" s="39"/>
+      <c r="D14" s="39"/>
       <c r="E14" s="3"/>
       <c r="F14" s="1"/>
-      <c r="G14" s="31"/>
-      <c r="H14" s="31"/>
+      <c r="G14" s="39"/>
+      <c r="H14" s="39"/>
       <c r="I14" s="3"/>
       <c r="J14" s="1"/>
     </row>
@@ -2056,12 +1981,12 @@
       <c r="A16" s="7">
         <v>0.47916666666666669</v>
       </c>
-      <c r="B16" s="38" t="s">
+      <c r="B16" s="37" t="s">
         <v>31</v>
       </c>
       <c r="D16" s="11"/>
       <c r="E16" s="11"/>
-      <c r="F16" s="38" t="str">
+      <c r="F16" s="37" t="str">
         <f>B16</f>
         <v>CSE 450
 Machine Learning
@@ -2071,7 +1996,7 @@
       <c r="G16" s="11"/>
       <c r="H16" s="11"/>
       <c r="I16" s="11"/>
-      <c r="J16" s="38" t="str">
+      <c r="J16" s="37" t="str">
         <f>F16</f>
         <v>CSE 450
 Machine Learning
@@ -2083,40 +2008,40 @@
       <c r="A17" s="7">
         <v>0.48958333333333331</v>
       </c>
-      <c r="B17" s="31"/>
+      <c r="B17" s="39"/>
       <c r="D17" s="11"/>
       <c r="E17" s="11"/>
-      <c r="F17" s="31"/>
+      <c r="F17" s="39"/>
       <c r="G17" s="11"/>
       <c r="H17" s="11"/>
       <c r="I17" s="11"/>
-      <c r="J17" s="31"/>
+      <c r="J17" s="39"/>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A18" s="7">
         <v>0.5</v>
       </c>
-      <c r="B18" s="31"/>
+      <c r="B18" s="39"/>
       <c r="D18" s="11"/>
       <c r="E18" s="11"/>
-      <c r="F18" s="31"/>
+      <c r="F18" s="39"/>
       <c r="G18" s="11"/>
       <c r="H18" s="11"/>
       <c r="I18" s="11"/>
-      <c r="J18" s="31"/>
+      <c r="J18" s="39"/>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A19" s="7">
         <v>0.51041666666666663</v>
       </c>
-      <c r="B19" s="31"/>
+      <c r="B19" s="39"/>
       <c r="D19" s="3"/>
       <c r="E19" s="3"/>
-      <c r="F19" s="31"/>
+      <c r="F19" s="39"/>
       <c r="G19" s="3"/>
       <c r="H19" s="3"/>
       <c r="I19" s="3"/>
-      <c r="J19" s="31"/>
+      <c r="J19" s="39"/>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A20" s="7">
@@ -2137,13 +2062,13 @@
       </c>
       <c r="B21" s="3"/>
       <c r="D21" s="3"/>
-      <c r="E21" s="39" t="s">
+      <c r="E21" s="41" t="s">
         <v>29</v>
       </c>
       <c r="F21" s="3"/>
       <c r="G21" s="3"/>
       <c r="H21" s="3"/>
-      <c r="I21" s="39" t="s">
+      <c r="I21" s="41" t="s">
         <v>30</v>
       </c>
       <c r="J21" s="3"/>
@@ -2154,11 +2079,11 @@
       </c>
       <c r="B22" s="3"/>
       <c r="D22" s="3"/>
-      <c r="E22" s="31"/>
+      <c r="E22" s="39"/>
       <c r="F22" s="3"/>
       <c r="G22" s="3"/>
       <c r="H22" s="3"/>
-      <c r="I22" s="31"/>
+      <c r="I22" s="39"/>
       <c r="J22" s="3"/>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.2">
@@ -2167,11 +2092,11 @@
       </c>
       <c r="B23" s="3"/>
       <c r="D23" s="3"/>
-      <c r="E23" s="31"/>
+      <c r="E23" s="39"/>
       <c r="F23" s="3"/>
       <c r="G23" s="3"/>
       <c r="H23" s="3"/>
-      <c r="I23" s="31"/>
+      <c r="I23" s="39"/>
       <c r="J23" s="3"/>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.2">
@@ -2180,11 +2105,11 @@
       </c>
       <c r="B24" s="3"/>
       <c r="D24" s="3"/>
-      <c r="E24" s="31"/>
+      <c r="E24" s="39"/>
       <c r="F24" s="3"/>
       <c r="G24" s="3"/>
       <c r="H24" s="3"/>
-      <c r="I24" s="31"/>
+      <c r="I24" s="39"/>
       <c r="J24" s="3"/>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.2">
@@ -2196,14 +2121,14 @@
       <c r="A26" s="7">
         <v>0.58333333333333337</v>
       </c>
-      <c r="B26" s="30" t="s">
+      <c r="B26" s="35" t="s">
         <v>32</v>
       </c>
       <c r="D26" s="1"/>
-      <c r="E26" s="32" t="s">
+      <c r="E26" s="33" t="s">
         <v>33</v>
       </c>
-      <c r="F26" s="30" t="str">
+      <c r="F26" s="35" t="str">
         <f>B26</f>
         <v>MATH 325
 Intermediate Stats 
@@ -2211,10 +2136,10 @@
 Remote</v>
       </c>
       <c r="H26" s="1"/>
-      <c r="I26" s="32" t="s">
+      <c r="I26" s="33" t="s">
         <v>33</v>
       </c>
-      <c r="J26" s="30" t="str">
+      <c r="J26" s="35" t="str">
         <f>F26</f>
         <v>MATH 325
 Intermediate Stats 
@@ -2226,37 +2151,37 @@
       <c r="A27" s="7">
         <v>0.59375</v>
       </c>
-      <c r="B27" s="31"/>
+      <c r="B27" s="39"/>
       <c r="D27" s="1"/>
-      <c r="E27" s="31"/>
-      <c r="F27" s="31"/>
+      <c r="E27" s="39"/>
+      <c r="F27" s="39"/>
       <c r="H27" s="1"/>
-      <c r="I27" s="31"/>
-      <c r="J27" s="31"/>
+      <c r="I27" s="39"/>
+      <c r="J27" s="39"/>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A28" s="7">
         <v>0.60416666666666663</v>
       </c>
-      <c r="B28" s="31"/>
+      <c r="B28" s="39"/>
       <c r="D28" s="1"/>
-      <c r="E28" s="31"/>
-      <c r="F28" s="31"/>
+      <c r="E28" s="39"/>
+      <c r="F28" s="39"/>
       <c r="H28" s="1"/>
-      <c r="I28" s="31"/>
-      <c r="J28" s="31"/>
+      <c r="I28" s="39"/>
+      <c r="J28" s="39"/>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A29" s="7">
         <v>0.61458333333333337</v>
       </c>
-      <c r="B29" s="31"/>
+      <c r="B29" s="39"/>
       <c r="D29" s="1"/>
-      <c r="E29" s="31"/>
-      <c r="F29" s="31"/>
+      <c r="E29" s="39"/>
+      <c r="F29" s="39"/>
       <c r="H29" s="1"/>
-      <c r="I29" s="31"/>
-      <c r="J29" s="31"/>
+      <c r="I29" s="39"/>
+      <c r="J29" s="39"/>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A30" s="7">
@@ -2344,12 +2269,11 @@
     </row>
   </sheetData>
   <mergeCells count="21">
-    <mergeCell ref="B16:B19"/>
-    <mergeCell ref="F16:F19"/>
-    <mergeCell ref="J16:J19"/>
-    <mergeCell ref="B26:B29"/>
-    <mergeCell ref="F26:F29"/>
-    <mergeCell ref="J26:J29"/>
+    <mergeCell ref="B1:C1"/>
+    <mergeCell ref="D1:E1"/>
+    <mergeCell ref="F1:G1"/>
+    <mergeCell ref="H1:I1"/>
+    <mergeCell ref="C11:C14"/>
     <mergeCell ref="J1:K1"/>
     <mergeCell ref="D2:D7"/>
     <mergeCell ref="D9:D14"/>
@@ -2360,11 +2284,12 @@
     <mergeCell ref="G11:G14"/>
     <mergeCell ref="H2:H7"/>
     <mergeCell ref="H9:H14"/>
-    <mergeCell ref="B1:C1"/>
-    <mergeCell ref="D1:E1"/>
-    <mergeCell ref="F1:G1"/>
-    <mergeCell ref="H1:I1"/>
-    <mergeCell ref="C11:C14"/>
+    <mergeCell ref="B16:B19"/>
+    <mergeCell ref="F16:F19"/>
+    <mergeCell ref="J16:J19"/>
+    <mergeCell ref="B26:B29"/>
+    <mergeCell ref="F26:F29"/>
+    <mergeCell ref="J26:J29"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2903,15 +2828,15 @@
       <c r="A7" s="7">
         <v>0.42708333333333331</v>
       </c>
-      <c r="B7" s="30" t="s">
+      <c r="B7" s="35" t="s">
         <v>110</v>
       </c>
       <c r="C7" s="3"/>
-      <c r="D7" s="30" t="s">
+      <c r="D7" s="35" t="s">
         <v>110</v>
       </c>
       <c r="E7" s="3"/>
-      <c r="F7" s="30" t="s">
+      <c r="F7" s="35" t="s">
         <v>110</v>
       </c>
     </row>
@@ -2919,31 +2844,31 @@
       <c r="A8" s="7">
         <v>0.4375</v>
       </c>
-      <c r="B8" s="31"/>
+      <c r="B8" s="39"/>
       <c r="C8" s="3"/>
-      <c r="D8" s="31"/>
+      <c r="D8" s="39"/>
       <c r="E8" s="3"/>
-      <c r="F8" s="31"/>
+      <c r="F8" s="39"/>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" s="7">
         <v>0.44791666666666669</v>
       </c>
-      <c r="B9" s="31"/>
+      <c r="B9" s="39"/>
       <c r="C9" s="3"/>
-      <c r="D9" s="31"/>
+      <c r="D9" s="39"/>
       <c r="E9" s="3"/>
-      <c r="F9" s="31"/>
+      <c r="F9" s="39"/>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" s="7">
         <v>0.45833333333333331</v>
       </c>
-      <c r="B10" s="31"/>
+      <c r="B10" s="39"/>
       <c r="C10" s="3"/>
-      <c r="D10" s="31"/>
+      <c r="D10" s="39"/>
       <c r="E10" s="3"/>
-      <c r="F10" s="31"/>
+      <c r="F10" s="39"/>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" s="7">
@@ -3059,15 +2984,15 @@
       <c r="A22" s="7">
         <v>0.58333333333333337</v>
       </c>
-      <c r="B22" s="30" t="s">
+      <c r="B22" s="35" t="s">
         <v>111</v>
       </c>
       <c r="C22" s="3"/>
-      <c r="D22" s="30" t="s">
+      <c r="D22" s="35" t="s">
         <v>111</v>
       </c>
       <c r="E22" s="3"/>
-      <c r="F22" s="30" t="s">
+      <c r="F22" s="35" t="s">
         <v>111</v>
       </c>
     </row>
@@ -3075,31 +3000,31 @@
       <c r="A23" s="7">
         <v>0.59375</v>
       </c>
-      <c r="B23" s="31"/>
+      <c r="B23" s="39"/>
       <c r="C23" s="3"/>
-      <c r="D23" s="31"/>
+      <c r="D23" s="39"/>
       <c r="E23" s="3"/>
-      <c r="F23" s="31"/>
+      <c r="F23" s="39"/>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A24" s="7">
         <v>0.60416666666666663</v>
       </c>
-      <c r="B24" s="31"/>
+      <c r="B24" s="39"/>
       <c r="C24" s="3"/>
-      <c r="D24" s="31"/>
+      <c r="D24" s="39"/>
       <c r="E24" s="3"/>
-      <c r="F24" s="31"/>
+      <c r="F24" s="39"/>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A25" s="7">
         <v>0.61458333333333337</v>
       </c>
-      <c r="B25" s="31"/>
+      <c r="B25" s="39"/>
       <c r="C25" s="3"/>
-      <c r="D25" s="31"/>
+      <c r="D25" s="39"/>
       <c r="E25" s="3"/>
-      <c r="F25" s="31"/>
+      <c r="F25" s="39"/>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A26" s="7">
@@ -3117,15 +3042,15 @@
       <c r="A27" s="7">
         <v>0.63541666666666663</v>
       </c>
-      <c r="B27" s="38" t="s">
+      <c r="B27" s="37" t="s">
         <v>112</v>
       </c>
       <c r="C27" s="5"/>
-      <c r="D27" s="38" t="s">
+      <c r="D27" s="37" t="s">
         <v>112</v>
       </c>
       <c r="E27" s="5"/>
-      <c r="F27" s="38" t="s">
+      <c r="F27" s="37" t="s">
         <v>112</v>
       </c>
     </row>
@@ -3133,31 +3058,31 @@
       <c r="A28" s="7">
         <v>0.64583333333333337</v>
       </c>
-      <c r="B28" s="31"/>
+      <c r="B28" s="39"/>
       <c r="C28" s="5"/>
-      <c r="D28" s="31"/>
+      <c r="D28" s="39"/>
       <c r="E28" s="5"/>
-      <c r="F28" s="31"/>
+      <c r="F28" s="39"/>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A29" s="7">
         <v>0.65625</v>
       </c>
-      <c r="B29" s="31"/>
+      <c r="B29" s="39"/>
       <c r="C29" s="5"/>
-      <c r="D29" s="31"/>
+      <c r="D29" s="39"/>
       <c r="E29" s="5"/>
-      <c r="F29" s="31"/>
+      <c r="F29" s="39"/>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A30" s="7">
         <v>0.66666666666666663</v>
       </c>
-      <c r="B30" s="31"/>
+      <c r="B30" s="39"/>
       <c r="C30" s="5"/>
-      <c r="D30" s="31"/>
+      <c r="D30" s="39"/>
       <c r="E30" s="5"/>
-      <c r="F30" s="31"/>
+      <c r="F30" s="39"/>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A31" s="7">

</xml_diff>